<commit_message>
se agrega img de mantto y actualizacion de plantilla de gasolinera
</commit_message>
<xml_diff>
--- a/Inputs/BD.xlsx
+++ b/Inputs/BD.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/078e1a455e5c02ce/Documentos/GitHub/Proyecto_PIPC/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="332" documentId="13_ncr:1_{CF2C40B5-0007-4E87-85E3-0CDB05564647}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{74A2A6C4-9803-41B1-9CCE-216C45707E1B}"/>
+  <xr:revisionPtr revIDLastSave="337" documentId="13_ncr:1_{CF2C40B5-0007-4E87-85E3-0CDB05564647}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3C9CD797-6E54-4F62-8BA9-34B551057627}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3F095A75-F066-4695-8672-8D4315F1EF23}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{3F095A75-F066-4695-8672-8D4315F1EF23}"/>
   </bookViews>
   <sheets>
     <sheet name="BD" sheetId="1" r:id="rId1"/>
@@ -260,7 +260,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A78" authorId="0" shapeId="0" xr:uid="{733E70D1-98D2-4246-AFA3-A8F0F23DC8ED}">
+    <comment ref="A79" authorId="0" shapeId="0" xr:uid="{12F3D2AC-77D3-465B-9182-DE15CC16FEE6}">
       <text>
         <r>
           <rPr>
@@ -289,7 +289,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1804" uniqueCount="843">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1805" uniqueCount="845">
   <si>
     <t>dia</t>
   </si>
@@ -2818,6 +2818,12 @@
   </si>
   <si>
     <t>13 DE ABRIL DE 1999</t>
+  </si>
+  <si>
+    <t>mantto1</t>
+  </si>
+  <si>
+    <t>mantto2</t>
   </si>
 </sst>
 </file>
@@ -3071,6 +3077,10 @@
     <mc:Fallback/>
   </mc:AlternateContent>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -19338,15 +19348,15 @@
     </row>
     <row r="77" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>723</v>
+        <v>843</v>
       </c>
       <c r="B77" t="str">
         <f t="shared" si="21"/>
-        <v>mantto.png</v>
+        <v>mantto1.png</v>
       </c>
       <c r="C77" t="str">
         <f t="shared" si="22"/>
-        <v>{{ mantto }}</v>
+        <v>{{ mantto1 }}</v>
       </c>
       <c r="D77">
         <v>190</v>
@@ -19363,60 +19373,60 @@
       </c>
       <c r="H77" t="str">
         <f t="shared" si="13"/>
-        <v>'mantto': mantto,</v>
+        <v>'mantto1': mantto1,</v>
       </c>
       <c r="I77" t="s">
         <v>565</v>
       </c>
       <c r="J77" t="str">
         <f t="shared" si="14"/>
-        <v>img_path_mantto = os.path.join(IMAGES_PATH, r_val["mantto"])</v>
+        <v>img_path_mantto1 = os.path.join(IMAGES_PATH, r_val["mantto1"])</v>
       </c>
       <c r="K77" t="str">
         <f t="shared" si="15"/>
-        <v>if os.path.exists(img_path_mantto):</v>
+        <v>if os.path.exists(img_path_mantto1):</v>
       </c>
       <c r="L77" t="str">
         <f t="shared" si="16"/>
-        <v>mantto = InlineImage(docx_tpl, img_path_mantto, height=Mm(190))</v>
+        <v>mantto1 = InlineImage(docx_tpl, img_path_mantto1, height=Mm(190))</v>
       </c>
       <c r="M77" t="s">
         <v>567</v>
       </c>
       <c r="N77" t="str">
         <f t="shared" si="17"/>
-        <v>print(f'Advertencia: No se encontró la imagen {r_val["mantto"]}')</v>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["mantto1"]}')</v>
       </c>
       <c r="O77" t="str">
         <f t="shared" si="18"/>
-        <v>mantto = ''</v>
+        <v>mantto1 = ''</v>
       </c>
       <c r="P77" t="s">
         <v>566</v>
       </c>
       <c r="Q77" t="str">
         <f t="shared" si="19"/>
-        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["mantto"]}: {e}')</v>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["mantto1"]}: {e}')</v>
       </c>
       <c r="R77" t="str">
         <f t="shared" si="20"/>
-        <v>mantto = ''</v>
+        <v>mantto1 = ''</v>
       </c>
     </row>
     <row r="78" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>724</v>
+        <v>844</v>
       </c>
       <c r="B78" t="str">
         <f t="shared" si="21"/>
-        <v>simulacro.png</v>
+        <v>mantto2.png</v>
       </c>
       <c r="C78" t="str">
         <f t="shared" si="22"/>
-        <v>{{ simulacro }}</v>
+        <v>{{ mantto2 }}</v>
       </c>
       <c r="D78">
-        <v>95</v>
+        <v>190</v>
       </c>
       <c r="E78" t="s">
         <v>582</v>
@@ -19430,57 +19440,57 @@
       </c>
       <c r="H78" t="str">
         <f t="shared" si="13"/>
-        <v>'simulacro': simulacro,</v>
+        <v>'mantto2': mantto2,</v>
       </c>
       <c r="I78" t="s">
         <v>565</v>
       </c>
       <c r="J78" t="str">
         <f t="shared" si="14"/>
-        <v>img_path_simulacro = os.path.join(IMAGES_PATH, r_val["simulacro"])</v>
+        <v>img_path_mantto2 = os.path.join(IMAGES_PATH, r_val["mantto2"])</v>
       </c>
       <c r="K78" t="str">
         <f t="shared" si="15"/>
-        <v>if os.path.exists(img_path_simulacro):</v>
+        <v>if os.path.exists(img_path_mantto2):</v>
       </c>
       <c r="L78" t="str">
         <f t="shared" si="16"/>
-        <v>simulacro = InlineImage(docx_tpl, img_path_simulacro, height=Mm(95))</v>
+        <v>mantto2 = InlineImage(docx_tpl, img_path_mantto2, height=Mm(190))</v>
       </c>
       <c r="M78" t="s">
         <v>567</v>
       </c>
       <c r="N78" t="str">
         <f t="shared" si="17"/>
-        <v>print(f'Advertencia: No se encontró la imagen {r_val["simulacro"]}')</v>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["mantto2"]}')</v>
       </c>
       <c r="O78" t="str">
         <f t="shared" si="18"/>
-        <v>simulacro = ''</v>
+        <v>mantto2 = ''</v>
       </c>
       <c r="P78" t="s">
         <v>566</v>
       </c>
       <c r="Q78" t="str">
         <f t="shared" si="19"/>
-        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["simulacro"]}: {e}')</v>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["mantto2"]}: {e}')</v>
       </c>
       <c r="R78" t="str">
         <f t="shared" si="20"/>
-        <v>simulacro = ''</v>
+        <v>mantto2 = ''</v>
       </c>
     </row>
     <row r="79" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="B79" t="str">
-        <f t="shared" si="21"/>
-        <v>capacitacion.png</v>
+        <f t="shared" ref="B79:B91" si="23">+_xlfn.CONCAT(A79,".png")</f>
+        <v>simulacro.png</v>
       </c>
       <c r="C79" t="str">
-        <f t="shared" si="22"/>
-        <v>{{ capacitacion }}</v>
+        <f t="shared" ref="C79:C91" si="24">+_xlfn.CONCAT("{{ ",A79," }}")</f>
+        <v>{{ simulacro }}</v>
       </c>
       <c r="D79">
         <v>95</v>
@@ -19492,65 +19502,65 @@
         <v>580</v>
       </c>
       <c r="G79" t="str">
-        <f t="shared" ref="G79:G110" si="23">+_xlfn.CONCAT("'",E79,"' : r_val['",E79,"'],")</f>
+        <f t="shared" ref="G79:G110" si="25">+_xlfn.CONCAT("'",E79,"' : r_val['",E79,"'],")</f>
         <v>'ubicacion_site' : r_val['ubicacion_site'],</v>
       </c>
       <c r="H79" t="str">
         <f t="shared" si="13"/>
-        <v>'capacitacion': capacitacion,</v>
+        <v>'simulacro': simulacro,</v>
       </c>
       <c r="I79" t="s">
         <v>565</v>
       </c>
       <c r="J79" t="str">
         <f t="shared" si="14"/>
-        <v>img_path_capacitacion = os.path.join(IMAGES_PATH, r_val["capacitacion"])</v>
+        <v>img_path_simulacro = os.path.join(IMAGES_PATH, r_val["simulacro"])</v>
       </c>
       <c r="K79" t="str">
         <f t="shared" si="15"/>
-        <v>if os.path.exists(img_path_capacitacion):</v>
+        <v>if os.path.exists(img_path_simulacro):</v>
       </c>
       <c r="L79" t="str">
         <f t="shared" si="16"/>
-        <v>capacitacion = InlineImage(docx_tpl, img_path_capacitacion, height=Mm(95))</v>
+        <v>simulacro = InlineImage(docx_tpl, img_path_simulacro, height=Mm(95))</v>
       </c>
       <c r="M79" t="s">
         <v>567</v>
       </c>
       <c r="N79" t="str">
         <f t="shared" si="17"/>
-        <v>print(f'Advertencia: No se encontró la imagen {r_val["capacitacion"]}')</v>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["simulacro"]}')</v>
       </c>
       <c r="O79" t="str">
         <f t="shared" si="18"/>
-        <v>capacitacion = ''</v>
+        <v>simulacro = ''</v>
       </c>
       <c r="P79" t="s">
         <v>566</v>
       </c>
       <c r="Q79" t="str">
         <f t="shared" si="19"/>
-        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["capacitacion"]}: {e}')</v>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["simulacro"]}: {e}')</v>
       </c>
       <c r="R79" t="str">
         <f t="shared" si="20"/>
-        <v>capacitacion = ''</v>
+        <v>simulacro = ''</v>
       </c>
     </row>
     <row r="80" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="B80" t="str">
-        <f t="shared" si="21"/>
-        <v>inv_quim.png</v>
+        <f t="shared" si="23"/>
+        <v>capacitacion.png</v>
       </c>
       <c r="C80" t="str">
-        <f t="shared" si="22"/>
-        <v>{{ inv_quim }}</v>
+        <f t="shared" si="24"/>
+        <v>{{ capacitacion }}</v>
       </c>
       <c r="D80">
-        <v>190</v>
+        <v>95</v>
       </c>
       <c r="E80" t="s">
         <v>15</v>
@@ -19559,62 +19569,62 @@
         <v>302</v>
       </c>
       <c r="G80" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>'hidrantes' : r_val['hidrantes'],</v>
       </c>
       <c r="H80" t="str">
         <f t="shared" si="13"/>
-        <v>'inv_quim': inv_quim,</v>
+        <v>'capacitacion': capacitacion,</v>
       </c>
       <c r="I80" t="s">
         <v>565</v>
       </c>
       <c r="J80" t="str">
         <f t="shared" si="14"/>
-        <v>img_path_inv_quim = os.path.join(IMAGES_PATH, r_val["inv_quim"])</v>
+        <v>img_path_capacitacion = os.path.join(IMAGES_PATH, r_val["capacitacion"])</v>
       </c>
       <c r="K80" t="str">
         <f t="shared" si="15"/>
-        <v>if os.path.exists(img_path_inv_quim):</v>
+        <v>if os.path.exists(img_path_capacitacion):</v>
       </c>
       <c r="L80" t="str">
         <f t="shared" si="16"/>
-        <v>inv_quim = InlineImage(docx_tpl, img_path_inv_quim, height=Mm(190))</v>
+        <v>capacitacion = InlineImage(docx_tpl, img_path_capacitacion, height=Mm(95))</v>
       </c>
       <c r="M80" t="s">
         <v>567</v>
       </c>
       <c r="N80" t="str">
         <f t="shared" si="17"/>
-        <v>print(f'Advertencia: No se encontró la imagen {r_val["inv_quim"]}')</v>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["capacitacion"]}')</v>
       </c>
       <c r="O80" t="str">
         <f t="shared" si="18"/>
-        <v>inv_quim = ''</v>
+        <v>capacitacion = ''</v>
       </c>
       <c r="P80" t="s">
         <v>566</v>
       </c>
       <c r="Q80" t="str">
         <f t="shared" si="19"/>
-        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["inv_quim"]}: {e}')</v>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["capacitacion"]}: {e}')</v>
       </c>
       <c r="R80" t="str">
         <f t="shared" si="20"/>
-        <v>inv_quim = ''</v>
+        <v>capacitacion = ''</v>
       </c>
     </row>
     <row r="81" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="B81" t="str">
-        <f t="shared" si="21"/>
-        <v>inv_emer.png</v>
+        <f t="shared" si="23"/>
+        <v>inv_quim.png</v>
       </c>
       <c r="C81" t="str">
-        <f t="shared" si="22"/>
-        <v>{{ inv_emer }}</v>
+        <f t="shared" si="24"/>
+        <v>{{ inv_quim }}</v>
       </c>
       <c r="D81">
         <v>190</v>
@@ -19626,62 +19636,62 @@
         <v>303</v>
       </c>
       <c r="G81" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>'aspersores' : r_val['aspersores'],</v>
       </c>
       <c r="H81" t="str">
         <f t="shared" si="13"/>
-        <v>'inv_emer': inv_emer,</v>
+        <v>'inv_quim': inv_quim,</v>
       </c>
       <c r="I81" t="s">
         <v>565</v>
       </c>
       <c r="J81" t="str">
         <f t="shared" si="14"/>
-        <v>img_path_inv_emer = os.path.join(IMAGES_PATH, r_val["inv_emer"])</v>
+        <v>img_path_inv_quim = os.path.join(IMAGES_PATH, r_val["inv_quim"])</v>
       </c>
       <c r="K81" t="str">
         <f t="shared" si="15"/>
-        <v>if os.path.exists(img_path_inv_emer):</v>
+        <v>if os.path.exists(img_path_inv_quim):</v>
       </c>
       <c r="L81" t="str">
         <f t="shared" si="16"/>
-        <v>inv_emer = InlineImage(docx_tpl, img_path_inv_emer, height=Mm(190))</v>
+        <v>inv_quim = InlineImage(docx_tpl, img_path_inv_quim, height=Mm(190))</v>
       </c>
       <c r="M81" t="s">
         <v>567</v>
       </c>
       <c r="N81" t="str">
         <f t="shared" si="17"/>
-        <v>print(f'Advertencia: No se encontró la imagen {r_val["inv_emer"]}')</v>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["inv_quim"]}')</v>
       </c>
       <c r="O81" t="str">
         <f t="shared" si="18"/>
-        <v>inv_emer = ''</v>
+        <v>inv_quim = ''</v>
       </c>
       <c r="P81" t="s">
         <v>566</v>
       </c>
       <c r="Q81" t="str">
         <f t="shared" si="19"/>
-        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["inv_emer"]}: {e}')</v>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["inv_quim"]}: {e}')</v>
       </c>
       <c r="R81" t="str">
         <f t="shared" si="20"/>
-        <v>inv_emer = ''</v>
+        <v>inv_quim = ''</v>
       </c>
     </row>
     <row r="82" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="B82" t="str">
-        <f t="shared" si="21"/>
-        <v>bit_emer.png</v>
+        <f t="shared" si="23"/>
+        <v>inv_emer.png</v>
       </c>
       <c r="C82" t="str">
-        <f t="shared" si="22"/>
-        <v>{{ bit_emer }}</v>
+        <f t="shared" si="24"/>
+        <v>{{ inv_emer }}</v>
       </c>
       <c r="D82">
         <v>190</v>
@@ -19693,62 +19703,62 @@
         <v>304</v>
       </c>
       <c r="G82" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>'bomberos' : r_val['bomberos'],</v>
       </c>
       <c r="H82" t="str">
         <f t="shared" si="13"/>
-        <v>'bit_emer': bit_emer,</v>
+        <v>'inv_emer': inv_emer,</v>
       </c>
       <c r="I82" t="s">
         <v>565</v>
       </c>
       <c r="J82" t="str">
         <f t="shared" si="14"/>
-        <v>img_path_bit_emer = os.path.join(IMAGES_PATH, r_val["bit_emer"])</v>
+        <v>img_path_inv_emer = os.path.join(IMAGES_PATH, r_val["inv_emer"])</v>
       </c>
       <c r="K82" t="str">
         <f t="shared" si="15"/>
-        <v>if os.path.exists(img_path_bit_emer):</v>
+        <v>if os.path.exists(img_path_inv_emer):</v>
       </c>
       <c r="L82" t="str">
         <f t="shared" si="16"/>
-        <v>bit_emer = InlineImage(docx_tpl, img_path_bit_emer, height=Mm(190))</v>
+        <v>inv_emer = InlineImage(docx_tpl, img_path_inv_emer, height=Mm(190))</v>
       </c>
       <c r="M82" t="s">
         <v>567</v>
       </c>
       <c r="N82" t="str">
         <f t="shared" si="17"/>
-        <v>print(f'Advertencia: No se encontró la imagen {r_val["bit_emer"]}')</v>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["inv_emer"]}')</v>
       </c>
       <c r="O82" t="str">
         <f t="shared" si="18"/>
-        <v>bit_emer = ''</v>
+        <v>inv_emer = ''</v>
       </c>
       <c r="P82" t="s">
         <v>566</v>
       </c>
       <c r="Q82" t="str">
         <f t="shared" si="19"/>
-        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["bit_emer"]}: {e}')</v>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["inv_emer"]}: {e}')</v>
       </c>
       <c r="R82" t="str">
         <f t="shared" si="20"/>
-        <v>bit_emer = ''</v>
+        <v>inv_emer = ''</v>
       </c>
     </row>
     <row r="83" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="B83" t="str">
-        <f t="shared" si="21"/>
-        <v>insp_bot.png</v>
+        <f t="shared" si="23"/>
+        <v>bit_emer.png</v>
       </c>
       <c r="C83" t="str">
-        <f t="shared" si="22"/>
-        <v>{{ insp_bot }}</v>
+        <f t="shared" si="24"/>
+        <v>{{ bit_emer }}</v>
       </c>
       <c r="D83">
         <v>190</v>
@@ -19760,62 +19770,62 @@
         <v>572</v>
       </c>
       <c r="G83" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>'ubicacion_bombero' : r_val['ubicacion_bombero'],</v>
       </c>
       <c r="H83" t="str">
         <f t="shared" si="13"/>
-        <v>'insp_bot': insp_bot,</v>
+        <v>'bit_emer': bit_emer,</v>
       </c>
       <c r="I83" t="s">
         <v>565</v>
       </c>
       <c r="J83" t="str">
         <f t="shared" si="14"/>
-        <v>img_path_insp_bot = os.path.join(IMAGES_PATH, r_val["insp_bot"])</v>
+        <v>img_path_bit_emer = os.path.join(IMAGES_PATH, r_val["bit_emer"])</v>
       </c>
       <c r="K83" t="str">
         <f t="shared" si="15"/>
-        <v>if os.path.exists(img_path_insp_bot):</v>
+        <v>if os.path.exists(img_path_bit_emer):</v>
       </c>
       <c r="L83" t="str">
         <f t="shared" si="16"/>
-        <v>insp_bot = InlineImage(docx_tpl, img_path_insp_bot, height=Mm(190))</v>
+        <v>bit_emer = InlineImage(docx_tpl, img_path_bit_emer, height=Mm(190))</v>
       </c>
       <c r="M83" t="s">
         <v>567</v>
       </c>
       <c r="N83" t="str">
         <f t="shared" si="17"/>
-        <v>print(f'Advertencia: No se encontró la imagen {r_val["insp_bot"]}')</v>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["bit_emer"]}')</v>
       </c>
       <c r="O83" t="str">
         <f t="shared" si="18"/>
-        <v>insp_bot = ''</v>
+        <v>bit_emer = ''</v>
       </c>
       <c r="P83" t="s">
         <v>566</v>
       </c>
       <c r="Q83" t="str">
         <f t="shared" si="19"/>
-        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["insp_bot"]}: {e}')</v>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["bit_emer"]}: {e}')</v>
       </c>
       <c r="R83" t="str">
         <f t="shared" si="20"/>
-        <v>insp_bot = ''</v>
+        <v>bit_emer = ''</v>
       </c>
     </row>
     <row r="84" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="B84" t="str">
-        <f t="shared" si="21"/>
-        <v>insp_ext.png</v>
+        <f t="shared" si="23"/>
+        <v>insp_bot.png</v>
       </c>
       <c r="C84" t="str">
-        <f t="shared" si="22"/>
-        <v>{{ insp_ext }}</v>
+        <f t="shared" si="24"/>
+        <v>{{ insp_bot }}</v>
       </c>
       <c r="D84">
         <v>190</v>
@@ -19827,62 +19837,62 @@
         <v>305</v>
       </c>
       <c r="G84" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>'detector_gas' : r_val['detector_gas'],</v>
       </c>
       <c r="H84" t="str">
         <f t="shared" si="13"/>
-        <v>'insp_ext': insp_ext,</v>
+        <v>'insp_bot': insp_bot,</v>
       </c>
       <c r="I84" t="s">
         <v>565</v>
       </c>
       <c r="J84" t="str">
         <f t="shared" si="14"/>
-        <v>img_path_insp_ext = os.path.join(IMAGES_PATH, r_val["insp_ext"])</v>
+        <v>img_path_insp_bot = os.path.join(IMAGES_PATH, r_val["insp_bot"])</v>
       </c>
       <c r="K84" t="str">
         <f t="shared" si="15"/>
-        <v>if os.path.exists(img_path_insp_ext):</v>
+        <v>if os.path.exists(img_path_insp_bot):</v>
       </c>
       <c r="L84" t="str">
         <f t="shared" si="16"/>
-        <v>insp_ext = InlineImage(docx_tpl, img_path_insp_ext, height=Mm(190))</v>
+        <v>insp_bot = InlineImage(docx_tpl, img_path_insp_bot, height=Mm(190))</v>
       </c>
       <c r="M84" t="s">
         <v>567</v>
       </c>
       <c r="N84" t="str">
         <f t="shared" si="17"/>
-        <v>print(f'Advertencia: No se encontró la imagen {r_val["insp_ext"]}')</v>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["insp_bot"]}')</v>
       </c>
       <c r="O84" t="str">
         <f t="shared" si="18"/>
-        <v>insp_ext = ''</v>
+        <v>insp_bot = ''</v>
       </c>
       <c r="P84" t="s">
         <v>566</v>
       </c>
       <c r="Q84" t="str">
         <f t="shared" si="19"/>
-        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["insp_ext"]}: {e}')</v>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["insp_bot"]}: {e}')</v>
       </c>
       <c r="R84" t="str">
         <f t="shared" si="20"/>
-        <v>insp_ext = ''</v>
+        <v>insp_bot = ''</v>
       </c>
     </row>
     <row r="85" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>734</v>
+        <v>730</v>
       </c>
       <c r="B85" t="str">
-        <f t="shared" si="21"/>
-        <v>insp_dh.png</v>
+        <f t="shared" si="23"/>
+        <v>insp_ext.png</v>
       </c>
       <c r="C85" t="str">
-        <f t="shared" si="22"/>
-        <v>{{ insp_dh }}</v>
+        <f t="shared" si="24"/>
+        <v>{{ insp_ext }}</v>
       </c>
       <c r="D85">
         <v>190</v>
@@ -19894,62 +19904,62 @@
         <v>576</v>
       </c>
       <c r="G85" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>'ubicación_gas' : r_val['ubicación_gas'],</v>
       </c>
       <c r="H85" t="str">
         <f t="shared" si="13"/>
-        <v>'insp_dh': insp_dh,</v>
+        <v>'insp_ext': insp_ext,</v>
       </c>
       <c r="I85" t="s">
         <v>565</v>
       </c>
       <c r="J85" t="str">
         <f t="shared" si="14"/>
-        <v>img_path_insp_dh = os.path.join(IMAGES_PATH, r_val["insp_dh"])</v>
+        <v>img_path_insp_ext = os.path.join(IMAGES_PATH, r_val["insp_ext"])</v>
       </c>
       <c r="K85" t="str">
         <f t="shared" si="15"/>
-        <v>if os.path.exists(img_path_insp_dh):</v>
+        <v>if os.path.exists(img_path_insp_ext):</v>
       </c>
       <c r="L85" t="str">
         <f t="shared" si="16"/>
-        <v>insp_dh = InlineImage(docx_tpl, img_path_insp_dh, height=Mm(190))</v>
+        <v>insp_ext = InlineImage(docx_tpl, img_path_insp_ext, height=Mm(190))</v>
       </c>
       <c r="M85" t="s">
         <v>567</v>
       </c>
       <c r="N85" t="str">
         <f t="shared" si="17"/>
-        <v>print(f'Advertencia: No se encontró la imagen {r_val["insp_dh"]}')</v>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["insp_ext"]}')</v>
       </c>
       <c r="O85" t="str">
         <f t="shared" si="18"/>
-        <v>insp_dh = ''</v>
+        <v>insp_ext = ''</v>
       </c>
       <c r="P85" t="s">
         <v>566</v>
       </c>
       <c r="Q85" t="str">
         <f t="shared" si="19"/>
-        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["insp_dh"]}: {e}')</v>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["insp_ext"]}: {e}')</v>
       </c>
       <c r="R85" t="str">
         <f t="shared" si="20"/>
-        <v>insp_dh = ''</v>
+        <v>insp_ext = ''</v>
       </c>
     </row>
     <row r="86" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="B86" t="str">
-        <f t="shared" si="21"/>
-        <v>insp_lamp.png</v>
+        <f t="shared" si="23"/>
+        <v>insp_dh.png</v>
       </c>
       <c r="C86" t="str">
-        <f t="shared" si="22"/>
-        <v>{{ insp_lamp }}</v>
+        <f t="shared" si="24"/>
+        <v>{{ insp_dh }}</v>
       </c>
       <c r="D86">
         <v>190</v>
@@ -19961,62 +19971,62 @@
         <v>306</v>
       </c>
       <c r="G86" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>'equipo_brigada' : r_val['equipo_brigada'],</v>
       </c>
       <c r="H86" t="str">
         <f t="shared" si="13"/>
-        <v>'insp_lamp': insp_lamp,</v>
+        <v>'insp_dh': insp_dh,</v>
       </c>
       <c r="I86" t="s">
         <v>565</v>
       </c>
       <c r="J86" t="str">
         <f t="shared" si="14"/>
-        <v>img_path_insp_lamp = os.path.join(IMAGES_PATH, r_val["insp_lamp"])</v>
+        <v>img_path_insp_dh = os.path.join(IMAGES_PATH, r_val["insp_dh"])</v>
       </c>
       <c r="K86" t="str">
         <f t="shared" si="15"/>
-        <v>if os.path.exists(img_path_insp_lamp):</v>
+        <v>if os.path.exists(img_path_insp_dh):</v>
       </c>
       <c r="L86" t="str">
         <f t="shared" si="16"/>
-        <v>insp_lamp = InlineImage(docx_tpl, img_path_insp_lamp, height=Mm(190))</v>
+        <v>insp_dh = InlineImage(docx_tpl, img_path_insp_dh, height=Mm(190))</v>
       </c>
       <c r="M86" t="s">
         <v>567</v>
       </c>
       <c r="N86" t="str">
         <f t="shared" si="17"/>
-        <v>print(f'Advertencia: No se encontró la imagen {r_val["insp_lamp"]}')</v>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["insp_dh"]}')</v>
       </c>
       <c r="O86" t="str">
         <f t="shared" si="18"/>
-        <v>insp_lamp = ''</v>
+        <v>insp_dh = ''</v>
       </c>
       <c r="P86" t="s">
         <v>566</v>
       </c>
       <c r="Q86" t="str">
         <f t="shared" si="19"/>
-        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["insp_lamp"]}: {e}')</v>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["insp_dh"]}: {e}')</v>
       </c>
       <c r="R86" t="str">
         <f t="shared" si="20"/>
-        <v>insp_lamp = ''</v>
+        <v>insp_dh = ''</v>
       </c>
     </row>
     <row r="87" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="B87" t="str">
-        <f t="shared" si="21"/>
-        <v>insp_alarm.png</v>
+        <f t="shared" si="23"/>
+        <v>insp_lamp.png</v>
       </c>
       <c r="C87" t="str">
-        <f t="shared" si="22"/>
-        <v>{{ insp_alarm }}</v>
+        <f t="shared" si="24"/>
+        <v>{{ insp_lamp }}</v>
       </c>
       <c r="D87">
         <v>190</v>
@@ -20028,62 +20038,62 @@
         <v>584</v>
       </c>
       <c r="G87" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>'ubicacion_brigada' : r_val['ubicacion_brigada'],</v>
       </c>
       <c r="H87" t="str">
         <f t="shared" si="13"/>
-        <v>'insp_alarm': insp_alarm,</v>
+        <v>'insp_lamp': insp_lamp,</v>
       </c>
       <c r="I87" t="s">
         <v>565</v>
       </c>
       <c r="J87" t="str">
         <f t="shared" si="14"/>
-        <v>img_path_insp_alarm = os.path.join(IMAGES_PATH, r_val["insp_alarm"])</v>
+        <v>img_path_insp_lamp = os.path.join(IMAGES_PATH, r_val["insp_lamp"])</v>
       </c>
       <c r="K87" t="str">
         <f t="shared" si="15"/>
-        <v>if os.path.exists(img_path_insp_alarm):</v>
+        <v>if os.path.exists(img_path_insp_lamp):</v>
       </c>
       <c r="L87" t="str">
         <f t="shared" si="16"/>
-        <v>insp_alarm = InlineImage(docx_tpl, img_path_insp_alarm, height=Mm(190))</v>
+        <v>insp_lamp = InlineImage(docx_tpl, img_path_insp_lamp, height=Mm(190))</v>
       </c>
       <c r="M87" t="s">
         <v>567</v>
       </c>
       <c r="N87" t="str">
         <f t="shared" si="17"/>
-        <v>print(f'Advertencia: No se encontró la imagen {r_val["insp_alarm"]}')</v>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["insp_lamp"]}')</v>
       </c>
       <c r="O87" t="str">
         <f t="shared" si="18"/>
-        <v>insp_alarm = ''</v>
+        <v>insp_lamp = ''</v>
       </c>
       <c r="P87" t="s">
         <v>566</v>
       </c>
       <c r="Q87" t="str">
         <f t="shared" si="19"/>
-        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["insp_alarm"]}: {e}')</v>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["insp_lamp"]}: {e}')</v>
       </c>
       <c r="R87" t="str">
         <f t="shared" si="20"/>
-        <v>insp_alarm = ''</v>
+        <v>insp_lamp = ''</v>
       </c>
     </row>
     <row r="88" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>731</v>
+        <v>736</v>
       </c>
       <c r="B88" t="str">
-        <f t="shared" si="21"/>
-        <v>ev_sim1.png</v>
+        <f t="shared" si="23"/>
+        <v>insp_alarm.png</v>
       </c>
       <c r="C88" t="str">
-        <f t="shared" si="22"/>
-        <v>{{ ev_sim1 }}</v>
+        <f t="shared" si="24"/>
+        <v>{{ insp_alarm }}</v>
       </c>
       <c r="D88">
         <v>190</v>
@@ -20095,62 +20105,62 @@
         <v>716</v>
       </c>
       <c r="G88" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>'ubiacion_brigadas' : r_val['ubiacion_brigadas'],</v>
       </c>
       <c r="H88" t="str">
         <f t="shared" si="13"/>
-        <v>'ev_sim1': ev_sim1,</v>
+        <v>'insp_alarm': insp_alarm,</v>
       </c>
       <c r="I88" t="s">
         <v>565</v>
       </c>
       <c r="J88" t="str">
         <f t="shared" si="14"/>
-        <v>img_path_ev_sim1 = os.path.join(IMAGES_PATH, r_val["ev_sim1"])</v>
+        <v>img_path_insp_alarm = os.path.join(IMAGES_PATH, r_val["insp_alarm"])</v>
       </c>
       <c r="K88" t="str">
         <f t="shared" si="15"/>
-        <v>if os.path.exists(img_path_ev_sim1):</v>
+        <v>if os.path.exists(img_path_insp_alarm):</v>
       </c>
       <c r="L88" t="str">
         <f t="shared" si="16"/>
-        <v>ev_sim1 = InlineImage(docx_tpl, img_path_ev_sim1, height=Mm(190))</v>
+        <v>insp_alarm = InlineImage(docx_tpl, img_path_insp_alarm, height=Mm(190))</v>
       </c>
       <c r="M88" t="s">
         <v>567</v>
       </c>
       <c r="N88" t="str">
         <f t="shared" si="17"/>
-        <v>print(f'Advertencia: No se encontró la imagen {r_val["ev_sim1"]}')</v>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["insp_alarm"]}')</v>
       </c>
       <c r="O88" t="str">
         <f t="shared" si="18"/>
-        <v>ev_sim1 = ''</v>
+        <v>insp_alarm = ''</v>
       </c>
       <c r="P88" t="s">
         <v>566</v>
       </c>
       <c r="Q88" t="str">
         <f t="shared" si="19"/>
-        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["ev_sim1"]}: {e}')</v>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["insp_alarm"]}: {e}')</v>
       </c>
       <c r="R88" t="str">
         <f t="shared" si="20"/>
-        <v>ev_sim1 = ''</v>
+        <v>insp_alarm = ''</v>
       </c>
     </row>
     <row r="89" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="B89" t="str">
-        <f t="shared" si="21"/>
-        <v>ev_sim2.png</v>
+        <f t="shared" si="23"/>
+        <v>ev_sim1.png</v>
       </c>
       <c r="C89" t="str">
-        <f t="shared" si="22"/>
-        <v>{{ ev_sim2 }}</v>
+        <f t="shared" si="24"/>
+        <v>{{ ev_sim1 }}</v>
       </c>
       <c r="D89">
         <v>190</v>
@@ -20162,62 +20172,62 @@
         <v>307</v>
       </c>
       <c r="G89" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>'lampara' : r_val['lampara'],</v>
       </c>
       <c r="H89" t="str">
         <f t="shared" si="13"/>
-        <v>'ev_sim2': ev_sim2,</v>
+        <v>'ev_sim1': ev_sim1,</v>
       </c>
       <c r="I89" t="s">
         <v>565</v>
       </c>
       <c r="J89" t="str">
         <f t="shared" si="14"/>
-        <v>img_path_ev_sim2 = os.path.join(IMAGES_PATH, r_val["ev_sim2"])</v>
+        <v>img_path_ev_sim1 = os.path.join(IMAGES_PATH, r_val["ev_sim1"])</v>
       </c>
       <c r="K89" t="str">
         <f t="shared" si="15"/>
-        <v>if os.path.exists(img_path_ev_sim2):</v>
+        <v>if os.path.exists(img_path_ev_sim1):</v>
       </c>
       <c r="L89" t="str">
         <f t="shared" si="16"/>
-        <v>ev_sim2 = InlineImage(docx_tpl, img_path_ev_sim2, height=Mm(190))</v>
+        <v>ev_sim1 = InlineImage(docx_tpl, img_path_ev_sim1, height=Mm(190))</v>
       </c>
       <c r="M89" t="s">
         <v>567</v>
       </c>
       <c r="N89" t="str">
         <f t="shared" si="17"/>
-        <v>print(f'Advertencia: No se encontró la imagen {r_val["ev_sim2"]}')</v>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["ev_sim1"]}')</v>
       </c>
       <c r="O89" t="str">
         <f t="shared" si="18"/>
-        <v>ev_sim2 = ''</v>
+        <v>ev_sim1 = ''</v>
       </c>
       <c r="P89" t="s">
         <v>566</v>
       </c>
       <c r="Q89" t="str">
         <f t="shared" si="19"/>
-        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["ev_sim2"]}: {e}')</v>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["ev_sim1"]}: {e}')</v>
       </c>
       <c r="R89" t="str">
         <f t="shared" si="20"/>
-        <v>ev_sim2 = ''</v>
+        <v>ev_sim1 = ''</v>
       </c>
     </row>
     <row r="90" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="B90" t="str">
-        <f t="shared" si="21"/>
-        <v>visitas.png</v>
+        <f t="shared" si="23"/>
+        <v>ev_sim2.png</v>
       </c>
       <c r="C90" t="str">
-        <f t="shared" si="22"/>
-        <v>{{ visitas }}</v>
+        <f t="shared" si="24"/>
+        <v>{{ ev_sim2 }}</v>
       </c>
       <c r="D90">
         <v>190</v>
@@ -20229,52 +20239,66 @@
         <v>568</v>
       </c>
       <c r="G90" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>'ubicacion_lampara' : r_val['ubicacion_lampara'],</v>
       </c>
       <c r="H90" t="str">
         <f t="shared" si="13"/>
-        <v>'visitas': visitas,</v>
+        <v>'ev_sim2': ev_sim2,</v>
       </c>
       <c r="I90" t="s">
         <v>565</v>
       </c>
       <c r="J90" t="str">
         <f t="shared" si="14"/>
-        <v>img_path_visitas = os.path.join(IMAGES_PATH, r_val["visitas"])</v>
+        <v>img_path_ev_sim2 = os.path.join(IMAGES_PATH, r_val["ev_sim2"])</v>
       </c>
       <c r="K90" t="str">
         <f t="shared" si="15"/>
-        <v>if os.path.exists(img_path_visitas):</v>
+        <v>if os.path.exists(img_path_ev_sim2):</v>
       </c>
       <c r="L90" t="str">
         <f t="shared" si="16"/>
-        <v>visitas = InlineImage(docx_tpl, img_path_visitas, height=Mm(190))</v>
+        <v>ev_sim2 = InlineImage(docx_tpl, img_path_ev_sim2, height=Mm(190))</v>
       </c>
       <c r="M90" t="s">
         <v>567</v>
       </c>
       <c r="N90" t="str">
         <f t="shared" si="17"/>
-        <v>print(f'Advertencia: No se encontró la imagen {r_val["visitas"]}')</v>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["ev_sim2"]}')</v>
       </c>
       <c r="O90" t="str">
         <f t="shared" si="18"/>
-        <v>visitas = ''</v>
+        <v>ev_sim2 = ''</v>
       </c>
       <c r="P90" t="s">
         <v>566</v>
       </c>
       <c r="Q90" t="str">
         <f t="shared" si="19"/>
-        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["visitas"]}: {e}')</v>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["ev_sim2"]}: {e}')</v>
       </c>
       <c r="R90" t="str">
         <f t="shared" si="20"/>
-        <v>visitas = ''</v>
+        <v>ev_sim2 = ''</v>
       </c>
     </row>
     <row r="91" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A91" t="s">
+        <v>733</v>
+      </c>
+      <c r="B91" t="str">
+        <f t="shared" si="23"/>
+        <v>visitas.png</v>
+      </c>
+      <c r="C91" t="str">
+        <f t="shared" si="24"/>
+        <v>{{ visitas }}</v>
+      </c>
+      <c r="D91">
+        <v>190</v>
+      </c>
       <c r="E91" t="s">
         <v>22</v>
       </c>
@@ -20282,7 +20306,7 @@
         <v>308</v>
       </c>
       <c r="G91" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>'baterias' : r_val['baterias'],</v>
       </c>
     </row>
@@ -20294,7 +20318,7 @@
         <v>578</v>
       </c>
       <c r="G92" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>'ubiacion_baterias' : r_val['ubiacion_baterias'],</v>
       </c>
     </row>
@@ -20306,7 +20330,7 @@
         <v>309</v>
       </c>
       <c r="G93" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>'tambo_arena' : r_val['tambo_arena'],</v>
       </c>
     </row>
@@ -20318,7 +20342,7 @@
         <v>570</v>
       </c>
       <c r="G94" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>'ubicacion_tambo' : r_val['ubicacion_tambo'],</v>
       </c>
     </row>
@@ -20330,7 +20354,7 @@
         <v>310</v>
       </c>
       <c r="G95" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>'tanques' : r_val['tanques'],</v>
       </c>
     </row>
@@ -20342,7 +20366,7 @@
         <v>311</v>
       </c>
       <c r="G96" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>'tanque_1' : r_val['tanque_1'],</v>
       </c>
     </row>
@@ -20354,7 +20378,7 @@
         <v>312</v>
       </c>
       <c r="G97" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>'tanque_2' : r_val['tanque_2'],</v>
       </c>
     </row>
@@ -20366,7 +20390,7 @@
         <v>313</v>
       </c>
       <c r="G98" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>'tanque_3' : r_val['tanque_3'],</v>
       </c>
     </row>
@@ -20378,7 +20402,7 @@
         <v>314</v>
       </c>
       <c r="G99" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>'dia' : r_val['dia'],</v>
       </c>
     </row>
@@ -20390,7 +20414,7 @@
         <v>315</v>
       </c>
       <c r="G100" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>'mes' : r_val['mes'],</v>
       </c>
     </row>
@@ -20402,7 +20426,7 @@
         <v>316</v>
       </c>
       <c r="G101" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>'anio' : r_val['anio'],</v>
       </c>
     </row>
@@ -20414,7 +20438,7 @@
         <v>317</v>
       </c>
       <c r="G102" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>'coordenadas' : r_val['coordenadas'],</v>
       </c>
     </row>
@@ -20426,7 +20450,7 @@
         <v>318</v>
       </c>
       <c r="G103" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>'norte' : r_val['norte'],</v>
       </c>
     </row>
@@ -20438,7 +20462,7 @@
         <v>319</v>
       </c>
       <c r="G104" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>'sur' : r_val['sur'],</v>
       </c>
     </row>
@@ -20450,7 +20474,7 @@
         <v>320</v>
       </c>
       <c r="G105" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>'este' : r_val['este'],</v>
       </c>
     </row>
@@ -20462,7 +20486,7 @@
         <v>321</v>
       </c>
       <c r="G106" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>'oeste' : r_val['oeste'],</v>
       </c>
     </row>
@@ -20474,7 +20498,7 @@
         <v>605</v>
       </c>
       <c r="G107" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>'ref_llegar' : r_val['ref_llegar'],</v>
       </c>
     </row>
@@ -20486,7 +20510,7 @@
         <v>322</v>
       </c>
       <c r="G108" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>'ley' : r_val['ley'],</v>
       </c>
     </row>
@@ -20498,7 +20522,7 @@
         <v>323</v>
       </c>
       <c r="G109" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>'reglamento' : r_val['reglamento'],</v>
       </c>
     </row>
@@ -20510,7 +20534,7 @@
         <v>694</v>
       </c>
       <c r="G110" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="25"/>
         <v>'m_dir' : r_val['m_dir'],</v>
       </c>
     </row>
@@ -20522,7 +20546,7 @@
         <v>324</v>
       </c>
       <c r="G111" t="str">
-        <f t="shared" ref="G111:G142" si="24">+_xlfn.CONCAT("'",E111,"' : r_val['",E111,"'],")</f>
+        <f t="shared" ref="G111:G142" si="26">+_xlfn.CONCAT("'",E111,"' : r_val['",E111,"'],")</f>
         <v>'coord_suplente' : r_val['coord_suplente'],</v>
       </c>
     </row>
@@ -20534,7 +20558,7 @@
         <v>695</v>
       </c>
       <c r="G112" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>'m_jef_caj' : r_val['m_jef_caj'],</v>
       </c>
     </row>
@@ -20546,7 +20570,7 @@
         <v>325</v>
       </c>
       <c r="G113" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>'evacuacion' : r_val['evacuacion'],</v>
       </c>
     </row>
@@ -20558,7 +20582,7 @@
         <v>596</v>
       </c>
       <c r="G114" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>'evac_puesto' : r_val['evac_puesto'],</v>
       </c>
     </row>
@@ -20570,7 +20594,7 @@
         <v>696</v>
       </c>
       <c r="G115" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>'m_evac' : r_val['m_evac'],</v>
       </c>
     </row>
@@ -20582,7 +20606,7 @@
         <v>326</v>
       </c>
       <c r="G116" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>'evac_suplente' : r_val['evac_suplente'],</v>
       </c>
     </row>
@@ -20594,7 +20618,7 @@
         <v>597</v>
       </c>
       <c r="G117" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>'supl_evac_pue' : r_val['supl_evac_pue'],</v>
       </c>
     </row>
@@ -20606,7 +20630,7 @@
         <v>697</v>
       </c>
       <c r="G118" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>'m_supl_evac' : r_val['m_supl_evac'],</v>
       </c>
     </row>
@@ -20618,7 +20642,7 @@
         <v>327</v>
       </c>
       <c r="G119" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>'incendios' : r_val['incendios'],</v>
       </c>
     </row>
@@ -20630,7 +20654,7 @@
         <v>598</v>
       </c>
       <c r="G120" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>'incen_puesto' : r_val['incen_puesto'],</v>
       </c>
     </row>
@@ -20642,7 +20666,7 @@
         <v>698</v>
       </c>
       <c r="G121" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>'m_inc' : r_val['m_inc'],</v>
       </c>
     </row>
@@ -20654,7 +20678,7 @@
         <v>328</v>
       </c>
       <c r="G122" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>'inc_suplente' : r_val['inc_suplente'],</v>
       </c>
     </row>
@@ -20666,7 +20690,7 @@
         <v>599</v>
       </c>
       <c r="G123" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>'supl_inc_puesto' : r_val['supl_inc_puesto'],</v>
       </c>
     </row>
@@ -20678,7 +20702,7 @@
         <v>699</v>
       </c>
       <c r="G124" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>'m_supl_inc' : r_val['m_supl_inc'],</v>
       </c>
     </row>
@@ -20690,7 +20714,7 @@
         <v>329</v>
       </c>
       <c r="G125" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>'primeros_auxilios' : r_val['primeros_auxilios'],</v>
       </c>
     </row>
@@ -20702,7 +20726,7 @@
         <v>600</v>
       </c>
       <c r="G126" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>'prim_aux_puesto' : r_val['prim_aux_puesto'],</v>
       </c>
     </row>
@@ -20714,7 +20738,7 @@
         <v>700</v>
       </c>
       <c r="G127" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>'m_prim_aux' : r_val['m_prim_aux'],</v>
       </c>
     </row>
@@ -20726,7 +20750,7 @@
         <v>330</v>
       </c>
       <c r="G128" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>'aux_suplente' : r_val['aux_suplente'],</v>
       </c>
     </row>
@@ -20738,7 +20762,7 @@
         <v>601</v>
       </c>
       <c r="G129" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>'supl_prim_aux_puesto' : r_val['supl_prim_aux_puesto'],</v>
       </c>
     </row>
@@ -20750,7 +20774,7 @@
         <v>701</v>
       </c>
       <c r="G130" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>'m_supl_paux' : r_val['m_supl_paux'],</v>
       </c>
     </row>
@@ -20762,7 +20786,7 @@
         <v>331</v>
       </c>
       <c r="G131" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>'busqueda' : r_val['busqueda'],</v>
       </c>
     </row>
@@ -20774,7 +20798,7 @@
         <v>602</v>
       </c>
       <c r="G132" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>'busq_puesto' : r_val['busq_puesto'],</v>
       </c>
     </row>
@@ -20786,7 +20810,7 @@
         <v>702</v>
       </c>
       <c r="G133" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>'m_busq' : r_val['m_busq'],</v>
       </c>
     </row>
@@ -20798,7 +20822,7 @@
         <v>332</v>
       </c>
       <c r="G134" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>'busq_suplente' : r_val['busq_suplente'],</v>
       </c>
     </row>
@@ -20810,7 +20834,7 @@
         <v>603</v>
       </c>
       <c r="G135" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>'supl_busq_puesto' : r_val['supl_busq_puesto'],</v>
       </c>
     </row>
@@ -20822,7 +20846,7 @@
         <v>703</v>
       </c>
       <c r="G136" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>'m_supl_busq' : r_val['m_supl_busq'],</v>
       </c>
     </row>
@@ -20834,7 +20858,7 @@
         <v>333</v>
       </c>
       <c r="G137" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>'descrip_gi' : r_val['descrip_gi'],</v>
       </c>
     </row>
@@ -20846,7 +20870,7 @@
         <v>334</v>
       </c>
       <c r="G138" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>'gas_inflamable' : r_val['gas_inflamable'],</v>
       </c>
     </row>
@@ -20858,7 +20882,7 @@
         <v>335</v>
       </c>
       <c r="G139" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>'valor_gi' : r_val['valor_gi'],</v>
       </c>
     </row>
@@ -20870,7 +20894,7 @@
         <v>336</v>
       </c>
       <c r="G140" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>'descrp_li' : r_val['descrp_li'],</v>
       </c>
     </row>
@@ -20882,7 +20906,7 @@
         <v>337</v>
       </c>
       <c r="G141" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>'liquido_inflamable' : r_val['liquido_inflamable'],</v>
       </c>
     </row>
@@ -20894,7 +20918,7 @@
         <v>338</v>
       </c>
       <c r="G142" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="26"/>
         <v>'valor_li' : r_val['valor_li'],</v>
       </c>
     </row>
@@ -20906,7 +20930,7 @@
         <v>339</v>
       </c>
       <c r="G143" t="str">
-        <f t="shared" ref="G143:G179" si="25">+_xlfn.CONCAT("'",E143,"' : r_val['",E143,"'],")</f>
+        <f t="shared" ref="G143:G179" si="27">+_xlfn.CONCAT("'",E143,"' : r_val['",E143,"'],")</f>
         <v>'descrip_lc' : r_val['descrip_lc'],</v>
       </c>
     </row>
@@ -20918,7 +20942,7 @@
         <v>340</v>
       </c>
       <c r="G144" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'liquido_combustible' : r_val['liquido_combustible'],</v>
       </c>
     </row>
@@ -20930,7 +20954,7 @@
         <v>341</v>
       </c>
       <c r="G145" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'valor_lc' : r_val['valor_lc'],</v>
       </c>
     </row>
@@ -20942,7 +20966,7 @@
         <v>342</v>
       </c>
       <c r="G146" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'descrip_sc' : r_val['descrip_sc'],</v>
       </c>
     </row>
@@ -20954,7 +20978,7 @@
         <v>343</v>
       </c>
       <c r="G147" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'solido_combusible' : r_val['solido_combusible'],</v>
       </c>
     </row>
@@ -20966,7 +20990,7 @@
         <v>344</v>
       </c>
       <c r="G148" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'valor_sc' : r_val['valor_sc'],</v>
       </c>
     </row>
@@ -20978,7 +21002,7 @@
         <v>345</v>
       </c>
       <c r="G149" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'tipo_riesgo' : r_val['tipo_riesgo'],</v>
       </c>
     </row>
@@ -20990,7 +21014,7 @@
         <v>664</v>
       </c>
       <c r="G150" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'nombre1' : r_val['nombre1'],</v>
       </c>
     </row>
@@ -21002,7 +21026,7 @@
         <v>665</v>
       </c>
       <c r="G151" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'puesto1' : r_val['puesto1'],</v>
       </c>
     </row>
@@ -21014,7 +21038,7 @@
         <v>666</v>
       </c>
       <c r="G152" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'m1' : r_val['m1'],</v>
       </c>
     </row>
@@ -21026,7 +21050,7 @@
         <v>667</v>
       </c>
       <c r="G153" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'nombre2' : r_val['nombre2'],</v>
       </c>
     </row>
@@ -21038,7 +21062,7 @@
         <v>668</v>
       </c>
       <c r="G154" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'puesto2' : r_val['puesto2'],</v>
       </c>
     </row>
@@ -21050,7 +21074,7 @@
         <v>669</v>
       </c>
       <c r="G155" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'m2' : r_val['m2'],</v>
       </c>
     </row>
@@ -21062,7 +21086,7 @@
         <v>670</v>
       </c>
       <c r="G156" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'nombre3' : r_val['nombre3'],</v>
       </c>
     </row>
@@ -21074,7 +21098,7 @@
         <v>671</v>
       </c>
       <c r="G157" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'puesto3' : r_val['puesto3'],</v>
       </c>
     </row>
@@ -21086,7 +21110,7 @@
         <v>672</v>
       </c>
       <c r="G158" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'m3' : r_val['m3'],</v>
       </c>
     </row>
@@ -21098,7 +21122,7 @@
         <v>673</v>
       </c>
       <c r="G159" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'nombre4' : r_val['nombre4'],</v>
       </c>
     </row>
@@ -21110,7 +21134,7 @@
         <v>674</v>
       </c>
       <c r="G160" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'puesto4' : r_val['puesto4'],</v>
       </c>
     </row>
@@ -21122,7 +21146,7 @@
         <v>675</v>
       </c>
       <c r="G161" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'m4' : r_val['m4'],</v>
       </c>
     </row>
@@ -21134,7 +21158,7 @@
         <v>676</v>
       </c>
       <c r="G162" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'nombre5' : r_val['nombre5'],</v>
       </c>
     </row>
@@ -21146,7 +21170,7 @@
         <v>677</v>
       </c>
       <c r="G163" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'puesto5' : r_val['puesto5'],</v>
       </c>
     </row>
@@ -21158,7 +21182,7 @@
         <v>678</v>
       </c>
       <c r="G164" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'m5' : r_val['m5'],</v>
       </c>
     </row>
@@ -21170,7 +21194,7 @@
         <v>679</v>
       </c>
       <c r="G165" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'nombre6' : r_val['nombre6'],</v>
       </c>
     </row>
@@ -21182,7 +21206,7 @@
         <v>680</v>
       </c>
       <c r="G166" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'puesto6' : r_val['puesto6'],</v>
       </c>
     </row>
@@ -21194,7 +21218,7 @@
         <v>681</v>
       </c>
       <c r="G167" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'m6' : r_val['m6'],</v>
       </c>
     </row>
@@ -21206,7 +21230,7 @@
         <v>682</v>
       </c>
       <c r="G168" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'nombre7' : r_val['nombre7'],</v>
       </c>
     </row>
@@ -21218,7 +21242,7 @@
         <v>683</v>
       </c>
       <c r="G169" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'puesto7' : r_val['puesto7'],</v>
       </c>
     </row>
@@ -21230,7 +21254,7 @@
         <v>684</v>
       </c>
       <c r="G170" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'m7' : r_val['m7'],</v>
       </c>
     </row>
@@ -21242,7 +21266,7 @@
         <v>685</v>
       </c>
       <c r="G171" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'nombre8' : r_val['nombre8'],</v>
       </c>
     </row>
@@ -21254,7 +21278,7 @@
         <v>686</v>
       </c>
       <c r="G172" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'puesto8' : r_val['puesto8'],</v>
       </c>
     </row>
@@ -21266,7 +21290,7 @@
         <v>687</v>
       </c>
       <c r="G173" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'m8' : r_val['m8'],</v>
       </c>
     </row>
@@ -21278,7 +21302,7 @@
         <v>688</v>
       </c>
       <c r="G174" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'nombre9' : r_val['nombre9'],</v>
       </c>
     </row>
@@ -21290,7 +21314,7 @@
         <v>689</v>
       </c>
       <c r="G175" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'puesto9' : r_val['puesto9'],</v>
       </c>
     </row>
@@ -21302,7 +21326,7 @@
         <v>690</v>
       </c>
       <c r="G176" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'m9' : r_val['m9'],</v>
       </c>
     </row>
@@ -21314,7 +21338,7 @@
         <v>691</v>
       </c>
       <c r="G177" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'nombre10' : r_val['nombre10'],</v>
       </c>
     </row>
@@ -21326,7 +21350,7 @@
         <v>692</v>
       </c>
       <c r="G178" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'puesto10' : r_val['puesto10'],</v>
       </c>
     </row>
@@ -21338,7 +21362,7 @@
         <v>693</v>
       </c>
       <c r="G179" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="27"/>
         <v>'m10' : r_val['m10'],</v>
       </c>
     </row>

</xml_diff>

<commit_message>
archivo BBVA1 info esencial
</commit_message>
<xml_diff>
--- a/Inputs/BD.xlsx
+++ b/Inputs/BD.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/078e1a455e5c02ce/Documentos/GitHub/Proyecto_PIPC/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2097" documentId="13_ncr:1_{7D3A426E-EC5E-453A-8CC7-F83B71F24F18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D11FA5CC-0D81-47A0-ADC8-AC915EA1CB9D}"/>
+  <xr:revisionPtr revIDLastSave="2113" documentId="13_ncr:1_{7D3A426E-EC5E-453A-8CC7-F83B71F24F18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B393A461-F338-4306-9288-2FEA4679A352}"/>
   <bookViews>
-    <workbookView xWindow="9972" yWindow="0" windowWidth="13056" windowHeight="8880" xr2:uid="{3F095A75-F066-4695-8672-8D4315F1EF23}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3F095A75-F066-4695-8672-8D4315F1EF23}"/>
   </bookViews>
   <sheets>
     <sheet name="BD" sheetId="1" r:id="rId1"/>
@@ -5668,9 +5668,6 @@
     <t>LAURA LILIANA CASTELLANOS MEDINA</t>
   </si>
   <si>
-    <t>CR 5020 PUEBLA SAN MANUEL</t>
-  </si>
-  <si>
     <t>CR 1521 PLAZA ARCANGELES</t>
   </si>
   <si>
@@ -5729,6 +5726,9 @@
   </si>
   <si>
     <t>FRENTE A TELEVISORA “IMAGEN TELEVISIÓN”</t>
+  </si>
+  <si>
+    <t>CR 520 PUEBLA SAN MANUEL</t>
   </si>
 </sst>
 </file>
@@ -6382,7 +6382,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp1.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Spin" dx="26" fmlaLink="$A$1" max="30000" min="1" page="10" val="13"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Spin" dx="26" fmlaLink="$A$1" max="30000" min="1" page="10" val="28"/>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6766,7 +6766,7 @@
   <sheetData>
     <row r="1" spans="1:281" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2">
-        <v>13</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:281" x14ac:dyDescent="0.3">
@@ -7587,31 +7587,31 @@
         <v>646</v>
       </c>
       <c r="JM2" t="s">
+        <v>1715</v>
+      </c>
+      <c r="JN2" t="s">
         <v>1716</v>
       </c>
-      <c r="JN2" t="s">
+      <c r="JO2" t="s">
         <v>1717</v>
       </c>
-      <c r="JO2" t="s">
+      <c r="JP2" t="s">
         <v>1718</v>
       </c>
-      <c r="JP2" t="s">
+      <c r="JQ2" t="s">
         <v>1719</v>
       </c>
-      <c r="JQ2" t="s">
+      <c r="JR2" t="s">
         <v>1720</v>
       </c>
-      <c r="JR2" t="s">
+      <c r="JS2" t="s">
         <v>1721</v>
       </c>
-      <c r="JS2" t="s">
+      <c r="JT2" t="s">
         <v>1722</v>
       </c>
-      <c r="JT2" t="s">
+      <c r="JU2" t="s">
         <v>1723</v>
-      </c>
-      <c r="JU2" t="s">
-        <v>1724</v>
       </c>
     </row>
     <row r="3" spans="1:281" x14ac:dyDescent="0.3">
@@ -11438,7 +11438,7 @@
         <v>72000</v>
       </c>
       <c r="P15" t="s">
-        <v>1725</v>
+        <v>1724</v>
       </c>
       <c r="V15">
         <v>832.26</v>
@@ -11605,19 +11605,19 @@
         <v>1343</v>
       </c>
       <c r="CZ15" t="s">
+        <v>1725</v>
+      </c>
+      <c r="DA15" t="s">
         <v>1726</v>
       </c>
-      <c r="DA15" t="s">
+      <c r="DB15" t="s">
         <v>1727</v>
-      </c>
-      <c r="DB15" t="s">
-        <v>1728</v>
       </c>
       <c r="DC15" t="s">
         <v>440</v>
       </c>
       <c r="DD15" t="s">
-        <v>1729</v>
+        <v>1728</v>
       </c>
       <c r="DE15" t="s">
         <v>442</v>
@@ -18972,7 +18972,7 @@
         <v>948</v>
       </c>
       <c r="D30" t="s">
-        <v>1709</v>
+        <v>1729</v>
       </c>
       <c r="E30" t="s">
         <v>845</v>
@@ -24475,7 +24475,7 @@
         <v>948</v>
       </c>
       <c r="D41" t="s">
-        <v>1710</v>
+        <v>1709</v>
       </c>
       <c r="E41" t="s">
         <v>845</v>
@@ -24487,13 +24487,13 @@
         <v>847</v>
       </c>
       <c r="I41" t="s">
-        <v>1711</v>
+        <v>1710</v>
       </c>
       <c r="J41">
         <v>6510</v>
       </c>
       <c r="L41" t="s">
-        <v>1712</v>
+        <v>1711</v>
       </c>
       <c r="M41" t="s">
         <v>1495</v>
@@ -24666,7 +24666,7 @@
         <v>2024</v>
       </c>
       <c r="CY41" t="s">
-        <v>1713</v>
+        <v>1712</v>
       </c>
       <c r="DE41" t="s">
         <v>442</v>
@@ -24985,7 +24985,7 @@
         <v>847</v>
       </c>
       <c r="I42" t="s">
-        <v>1714</v>
+        <v>1713</v>
       </c>
       <c r="J42">
         <v>101</v>
@@ -25104,7 +25104,7 @@
         <v>2024</v>
       </c>
       <c r="CY42" t="s">
-        <v>1715</v>
+        <v>1714</v>
       </c>
       <c r="DE42" t="s">
         <v>442</v>
@@ -30910,7 +30910,7 @@
     <row r="1" spans="1:248" x14ac:dyDescent="0.3">
       <c r="A1">
         <f>+BD!A1</f>
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="B1" t="s">
         <v>134</v>
@@ -31665,7 +31665,7 @@
       </c>
       <c r="D2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,4, FALSE)</f>
-        <v>CR 511 PUEBLA JUAREZ</v>
+        <v>CR 520 PUEBLA SAN MANUEL</v>
       </c>
       <c r="E2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,5, FALSE)</f>
@@ -31685,19 +31685,19 @@
       </c>
       <c r="I2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,9, FALSE)</f>
-        <v xml:space="preserve"> AV. JUAREZ</v>
+        <v>DIAGONAL ZARAGOZA</v>
       </c>
       <c r="J2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,10, FALSE)</f>
-        <v>1506</v>
-      </c>
-      <c r="K2">
+        <v>5128</v>
+      </c>
+      <c r="K2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,11, FALSE)</f>
-        <v>0</v>
+        <v>A</v>
       </c>
       <c r="L2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,12, FALSE)</f>
-        <v>CENTRO</v>
+        <v>JARDINES DE SAN MANUEL</v>
       </c>
       <c r="M2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,13, FALSE)</f>
@@ -31709,15 +31709,15 @@
       </c>
       <c r="O2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,15, FALSE)</f>
-        <v>72000</v>
-      </c>
-      <c r="P2" t="str">
+        <v>72570</v>
+      </c>
+      <c r="P2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,16, FALSE)</f>
-        <v>222 232 08 09</v>
-      </c>
-      <c r="Q2">
+        <v>2216671314</v>
+      </c>
+      <c r="Q2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,17, FALSE)</f>
-        <v>0</v>
+        <v>josecasiano.garcia@bbva.xom</v>
       </c>
       <c r="R2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,18, FALSE)</f>
@@ -31737,11 +31737,11 @@
       </c>
       <c r="V2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,22, FALSE)</f>
-        <v>832.26</v>
+        <v>0</v>
       </c>
       <c r="W2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,23, FALSE)</f>
-        <v>832.26</v>
+        <v>0</v>
       </c>
       <c r="X2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,24, FALSE)</f>
@@ -31769,7 +31769,7 @@
       </c>
       <c r="AD2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,30, FALSE)</f>
-        <v>10 CAJONES</v>
+        <v>5 CAJONES</v>
       </c>
       <c r="AE2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,31, FALSE)</f>
@@ -31777,11 +31777,11 @@
       </c>
       <c r="AF2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,32, FALSE)</f>
-        <v>MARIO ROJAS JURADO</v>
+        <v>NATALIA E. MARTINEZ ROJAS</v>
       </c>
       <c r="AG2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,33, FALSE)</f>
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="AH2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,34, FALSE)</f>
@@ -31789,11 +31789,11 @@
       </c>
       <c r="AI2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,35, FALSE)</f>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AJ2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,36, FALSE)</f>
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="AK2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,37, FALSE)</f>
@@ -31809,11 +31809,11 @@
       </c>
       <c r="AN2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,40, FALSE)</f>
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AO2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,41, FALSE)</f>
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="AP2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,42, FALSE)</f>
@@ -31825,11 +31825,11 @@
       </c>
       <c r="AR2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,44, FALSE)</f>
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="AS2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,45, FALSE)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AT2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,46, FALSE)</f>
@@ -31837,7 +31837,7 @@
       </c>
       <c r="AU2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,47, FALSE)</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AV2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,48, FALSE)</f>
@@ -31849,7 +31849,7 @@
       </c>
       <c r="AX2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,50, FALSE)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AY2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,51, FALSE)</f>
@@ -31877,7 +31877,7 @@
       </c>
       <c r="BE2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,57, FALSE)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BF2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,58, FALSE)</f>
@@ -31889,7 +31889,7 @@
       </c>
       <c r="BH2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,60, FALSE)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BI2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,61, FALSE)</f>
@@ -31897,7 +31897,7 @@
       </c>
       <c r="BJ2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,62, FALSE)</f>
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="BK2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,63, FALSE)</f>
@@ -31905,7 +31905,7 @@
       </c>
       <c r="BL2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,64, FALSE)</f>
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="BM2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,65, FALSE)</f>
@@ -31921,11 +31921,11 @@
       </c>
       <c r="BP2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,68, FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BQ2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,69, FALSE)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BR2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,70, FALSE)</f>
@@ -31933,11 +31933,11 @@
       </c>
       <c r="BS2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,71, FALSE)</f>
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="BT2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,72, FALSE)</f>
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="BU2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,73, FALSE)</f>
@@ -31961,7 +31961,7 @@
       </c>
       <c r="BZ2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,78, FALSE)</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="CA2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,79, FALSE)</f>
@@ -32049,7 +32049,7 @@
       </c>
       <c r="CV2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,100, FALSE)</f>
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="CW2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,101, FALSE)</f>
@@ -32061,27 +32061,27 @@
       </c>
       <c r="CY2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,103, FALSE)</f>
-        <v>19.047920704202305, -98.21059731923174</v>
-      </c>
-      <c r="CZ2" t="str">
+        <v>19.01635199500545, -98.19894850064507</v>
+      </c>
+      <c r="CZ2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,104, FALSE)</f>
-        <v>AVENIDA 5 PONIENTE</v>
-      </c>
-      <c r="DA2" t="str">
+        <v>0</v>
+      </c>
+      <c r="DA2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,105, FALSE)</f>
-        <v>AVENIDA JUÁREZ</v>
-      </c>
-      <c r="DB2" t="str">
+        <v>0</v>
+      </c>
+      <c r="DB2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,106, FALSE)</f>
-        <v>CALE 15 SUR</v>
-      </c>
-      <c r="DC2" t="str">
+        <v>0</v>
+      </c>
+      <c r="DC2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,107, FALSE)</f>
-        <v>LOCALES COMERCIALES</v>
-      </c>
-      <c r="DD2" t="str">
+        <v>0</v>
+      </c>
+      <c r="DD2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,108, FALSE)</f>
-        <v>FRENTE A TELEVISORA “IMAGEN TELEVISIÓN”</v>
+        <v>0</v>
       </c>
       <c r="DE2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,109, FALSE)</f>
@@ -32091,113 +32091,113 @@
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,110, FALSE)</f>
         <v>Reglamento de la Ley del Sistema Estatal de Protección Civil para el Estado Libre y Soberano de Puebla, publicado el 1 de julio de 1998.</v>
       </c>
-      <c r="DG2" t="str">
+      <c r="DG2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,111, FALSE)</f>
-        <v>MB09216</v>
+        <v>0</v>
       </c>
       <c r="DH2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,112, FALSE)</f>
-        <v>ROSARIO GONZALEZ VALLARTE</v>
+        <v>JOSE CACIANO GARCIA SANTIAGO</v>
       </c>
       <c r="DI2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,113, FALSE)</f>
-        <v>MI5545</v>
+        <v>MB77651</v>
       </c>
       <c r="DJ2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,114, FALSE)</f>
-        <v>DIEGO HERNANDEZ CARMONA</v>
+        <v>MIRIAM CORAL ZAYAGO MOJICA</v>
       </c>
       <c r="DK2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,115, FALSE)</f>
-        <v>ASESOR DIGITAL</v>
+        <v>BANQUERO POOL</v>
       </c>
       <c r="DL2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,116, FALSE)</f>
-        <v>MI28409</v>
+        <v>MB77868</v>
       </c>
       <c r="DM2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,117, FALSE)</f>
-        <v>PAOLA CUAUTLE AGUILAR</v>
+        <v>VICTORIA ALEJANDRA HERNANDEZ SOLIS</v>
       </c>
       <c r="DN2" s="5" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,118, FALSE)</f>
-        <v>CAJERO UNIVERSAL B</v>
+        <v>ASESOR DIGITAL</v>
       </c>
       <c r="DO2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,119, FALSE)</f>
-        <v>MB87913</v>
+        <v>MI22403</v>
       </c>
       <c r="DP2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,120, FALSE)</f>
-        <v>FERNANDO HERNANDEZ MARTINEZ</v>
+        <v>EDUARDO ARTURO ORTEGA QUINTERO</v>
       </c>
       <c r="DQ2" s="5" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,121, FALSE)</f>
-        <v>CAJERO UNIVERSAL B</v>
+        <v>ASESOR DIGITAL</v>
       </c>
       <c r="DR2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,122, FALSE)</f>
-        <v>M903801</v>
+        <v>MI23928</v>
       </c>
       <c r="DS2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,123, FALSE)</f>
-        <v>RAFAEL UGARTE OLIVER</v>
+        <v>MIGUEL ANGEL FONSECA GUTIERREZ</v>
       </c>
       <c r="DT2" s="5" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,124, FALSE)</f>
-        <v>CAJERO UNIVERSAL B</v>
+        <v>BANQUERO POOL</v>
       </c>
       <c r="DU2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,125, FALSE)</f>
-        <v>MB54486</v>
+        <v>MI10709</v>
       </c>
       <c r="DV2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,126, FALSE)</f>
-        <v>MARIA ANGELICA BALCAZAR ROMERO</v>
+        <v>GLADYS PEREZ SALAZAR</v>
       </c>
       <c r="DW2" s="5" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,127, FALSE)</f>
-        <v>BANQUERO JR</v>
+        <v>JEFE DE CAJA</v>
       </c>
       <c r="DX2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,128, FALSE)</f>
-        <v>MB44681</v>
+        <v>M821641</v>
       </c>
       <c r="DY2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,129, FALSE)</f>
-        <v>MARIA DE LOS ANGELES LARA MORALES</v>
+        <v>ANA LAURA FLORES SERRANO</v>
       </c>
       <c r="DZ2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,130, FALSE)</f>
-        <v>BANQUERO</v>
+        <v>CAJERO UNIVERSAL B</v>
       </c>
       <c r="EA2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,131, FALSE)</f>
-        <v>MB90635</v>
+        <v>M841691</v>
       </c>
       <c r="EB2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,132, FALSE)</f>
-        <v>JUDITH CHICO SARTILLO</v>
+        <v>VICTOR CONCEPCION SUAREZ FLORES</v>
       </c>
       <c r="EC2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,133, FALSE)</f>
-        <v>ASESOR DIGITAL</v>
+        <v>CAJERO UNIVERSAL B</v>
       </c>
       <c r="ED2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,134, FALSE)</f>
-        <v>MI17688</v>
-      </c>
-      <c r="EE2" t="str">
+        <v>MB95251</v>
+      </c>
+      <c r="EE2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,135, FALSE)</f>
-        <v>HECTOR ELIAS COYOTL SANCHEZ</v>
-      </c>
-      <c r="EF2" t="str">
+        <v>0</v>
+      </c>
+      <c r="EF2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,136, FALSE)</f>
-        <v>ASESOR DIGITAL</v>
-      </c>
-      <c r="EG2" t="str">
+        <v>0</v>
+      </c>
+      <c r="EG2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,137, FALSE)</f>
-        <v>MI21700</v>
+        <v>0</v>
       </c>
       <c r="EH2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,138, FALSE)</f>
@@ -32241,39 +32241,39 @@
       </c>
       <c r="ER2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,148, FALSE)</f>
-        <v>960</v>
+        <v>0</v>
       </c>
       <c r="ES2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,149, FALSE)</f>
-        <v>6.4000000000000001E-2</v>
+        <v>0</v>
       </c>
       <c r="ET2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,150, FALSE)</f>
         <v>ORDINARIO</v>
       </c>
-      <c r="EU2" t="str">
+      <c r="EU2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,151, FALSE)</f>
-        <v>MARTHA PATRICIA SALGADO FLORES</v>
-      </c>
-      <c r="EV2" t="str">
+        <v>0</v>
+      </c>
+      <c r="EV2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,152, FALSE)</f>
-        <v>CAJERO UNIVERSAL B</v>
-      </c>
-      <c r="EW2" t="str">
+        <v>0</v>
+      </c>
+      <c r="EW2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,153, FALSE)</f>
-        <v>MB97571</v>
-      </c>
-      <c r="EX2" t="str">
+        <v>0</v>
+      </c>
+      <c r="EX2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,154, FALSE)</f>
-        <v>MONICA VIDAL HERANANDEZ</v>
-      </c>
-      <c r="EY2" t="str">
+        <v>0</v>
+      </c>
+      <c r="EY2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,155, FALSE)</f>
-        <v>CAJERO UNIVERSAL</v>
-      </c>
-      <c r="EZ2" t="str">
+        <v>0</v>
+      </c>
+      <c r="EZ2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,156, FALSE)</f>
-        <v>MB47232</v>
+        <v>0</v>
       </c>
       <c r="FA2" t="s">
         <v>81</v>

</xml_diff>

<commit_message>
cambio mod_estruc por registro_perito
</commit_message>
<xml_diff>
--- a/Inputs/BD.xlsx
+++ b/Inputs/BD.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/078e1a455e5c02ce/Documentos/GitHub/Proyecto_PIPC/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2113" documentId="13_ncr:1_{7D3A426E-EC5E-453A-8CC7-F83B71F24F18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B393A461-F338-4306-9288-2FEA4679A352}"/>
+  <xr:revisionPtr revIDLastSave="2647" documentId="13_ncr:1_{7D3A426E-EC5E-453A-8CC7-F83B71F24F18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{49319CD6-1B47-4B95-9381-CCE56D53938A}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3F095A75-F066-4695-8672-8D4315F1EF23}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{3F095A75-F066-4695-8672-8D4315F1EF23}"/>
   </bookViews>
   <sheets>
     <sheet name="BD" sheetId="1" r:id="rId1"/>
@@ -539,7 +539,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5519" uniqueCount="1730">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5524" uniqueCount="1735">
   <si>
     <t>dia</t>
   </si>
@@ -5729,6 +5729,21 @@
   </si>
   <si>
     <t>CR 520 PUEBLA SAN MANUEL</t>
+  </si>
+  <si>
+    <t>registro_perito</t>
+  </si>
+  <si>
+    <t>no_registro</t>
+  </si>
+  <si>
+    <t>NÚMERO DE REGISTRO</t>
+  </si>
+  <si>
+    <t>DMPC/018/2024</t>
+  </si>
+  <si>
+    <t>28 DE SEPTIEMBRE DE 2021</t>
   </si>
 </sst>
 </file>
@@ -6382,7 +6397,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp1.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Spin" dx="26" fmlaLink="$A$1" max="30000" min="1" page="10" val="28"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Spin" dx="26" fmlaLink="$A$1" max="30000" min="1" page="10" val="38"/>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6766,7 +6781,7 @@
   <sheetData>
     <row r="1" spans="1:281" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:281" x14ac:dyDescent="0.3">
@@ -6828,10 +6843,10 @@
         <v>151</v>
       </c>
       <c r="T2" t="s">
-        <v>152</v>
+        <v>1730</v>
       </c>
       <c r="U2" t="s">
-        <v>153</v>
+        <v>1731</v>
       </c>
       <c r="V2" t="s">
         <v>154</v>
@@ -24009,6 +24024,24 @@
       </c>
       <c r="Q40" s="3" t="s">
         <v>1586</v>
+      </c>
+      <c r="R40">
+        <v>3</v>
+      </c>
+      <c r="S40" t="s">
+        <v>1734</v>
+      </c>
+      <c r="T40" t="s">
+        <v>1732</v>
+      </c>
+      <c r="U40" t="s">
+        <v>1733</v>
+      </c>
+      <c r="V40">
+        <v>300</v>
+      </c>
+      <c r="W40">
+        <v>300</v>
       </c>
       <c r="X40">
         <v>1</v>
@@ -30910,7 +30943,7 @@
     <row r="1" spans="1:248" x14ac:dyDescent="0.3">
       <c r="A1">
         <f>+BD!A1</f>
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="B1" t="s">
         <v>134</v>
@@ -30967,10 +31000,10 @@
         <v>151</v>
       </c>
       <c r="T1" t="s">
-        <v>152</v>
+        <v>1730</v>
       </c>
       <c r="U1" t="s">
-        <v>153</v>
+        <v>1731</v>
       </c>
       <c r="V1" t="s">
         <v>154</v>
@@ -31665,7 +31698,7 @@
       </c>
       <c r="D2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,4, FALSE)</f>
-        <v>CR 520 PUEBLA SAN MANUEL</v>
+        <v>CR 1888 PLAZA KENTRO SAN ANDRES CHOLULA</v>
       </c>
       <c r="E2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,5, FALSE)</f>
@@ -31685,23 +31718,23 @@
       </c>
       <c r="I2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,9, FALSE)</f>
-        <v>DIAGONAL ZARAGOZA</v>
+        <v>BOULEVARD ATLIXCAYOTL</v>
       </c>
       <c r="J2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,10, FALSE)</f>
-        <v>5128</v>
+        <v>3432</v>
       </c>
       <c r="K2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,11, FALSE)</f>
-        <v>A</v>
+        <v>LOCAL 18, 19, 20, 21</v>
       </c>
       <c r="L2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,12, FALSE)</f>
-        <v>JARDINES DE SAN MANUEL</v>
+        <v>RESERVA TERRITORIAL ATLIXCAYOTL</v>
       </c>
       <c r="M2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,13, FALSE)</f>
-        <v>PUEBLA</v>
+        <v>SAN ANDRES CHOLULA</v>
       </c>
       <c r="N2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,14, FALSE)</f>
@@ -31709,39 +31742,39 @@
       </c>
       <c r="O2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,15, FALSE)</f>
-        <v>72570</v>
+        <v>72825</v>
       </c>
       <c r="P2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,16, FALSE)</f>
-        <v>2216671314</v>
+        <v>2226894860</v>
       </c>
       <c r="Q2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,17, FALSE)</f>
-        <v>josecasiano.garcia@bbva.xom</v>
+        <v>mariamercedes.ramirez@bbva.com</v>
       </c>
       <c r="R2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,18, FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="S2">
+        <v>3</v>
+      </c>
+      <c r="S2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,19, FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="T2">
+        <v>28 DE SEPTIEMBRE DE 2021</v>
+      </c>
+      <c r="T2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,20, FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="U2">
+        <v>NÚMERO DE REGISTRO</v>
+      </c>
+      <c r="U2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,21, FALSE)</f>
-        <v>0</v>
+        <v>DMPC/018/2024</v>
       </c>
       <c r="V2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,22, FALSE)</f>
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="W2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,23, FALSE)</f>
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="X2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,24, FALSE)</f>
@@ -31769,7 +31802,7 @@
       </c>
       <c r="AD2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,30, FALSE)</f>
-        <v>5 CAJONES</v>
+        <v>10 CAJONES</v>
       </c>
       <c r="AE2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,31, FALSE)</f>
@@ -31777,7 +31810,7 @@
       </c>
       <c r="AF2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,32, FALSE)</f>
-        <v>NATALIA E. MARTINEZ ROJAS</v>
+        <v>NANCY KAREN CASCO GONZALEZ</v>
       </c>
       <c r="AG2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,33, FALSE)</f>
@@ -31789,11 +31822,11 @@
       </c>
       <c r="AI2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,35, FALSE)</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AJ2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,36, FALSE)</f>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="AK2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,37, FALSE)</f>
@@ -31825,11 +31858,11 @@
       </c>
       <c r="AR2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,44, FALSE)</f>
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="AS2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,45, FALSE)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AT2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,46, FALSE)</f>
@@ -31837,7 +31870,7 @@
       </c>
       <c r="AU2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,47, FALSE)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AV2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,48, FALSE)</f>
@@ -31849,7 +31882,7 @@
       </c>
       <c r="AX2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,50, FALSE)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AY2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,51, FALSE)</f>
@@ -31877,7 +31910,7 @@
       </c>
       <c r="BE2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,57, FALSE)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BF2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,58, FALSE)</f>
@@ -31889,7 +31922,7 @@
       </c>
       <c r="BH2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,60, FALSE)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BI2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,61, FALSE)</f>
@@ -31897,7 +31930,7 @@
       </c>
       <c r="BJ2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,62, FALSE)</f>
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="BK2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,63, FALSE)</f>
@@ -31905,7 +31938,7 @@
       </c>
       <c r="BL2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,64, FALSE)</f>
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="BM2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,65, FALSE)</f>
@@ -31913,11 +31946,11 @@
       </c>
       <c r="BN2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,66, FALSE)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BO2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,67, FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BP2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,68, FALSE)</f>
@@ -31925,11 +31958,11 @@
       </c>
       <c r="BQ2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,69, FALSE)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="BR2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,70, FALSE)</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="BS2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,71, FALSE)</f>
@@ -31961,7 +31994,7 @@
       </c>
       <c r="BZ2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,78, FALSE)</f>
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="CA2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,79, FALSE)</f>
@@ -32049,7 +32082,7 @@
       </c>
       <c r="CV2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,100, FALSE)</f>
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="CW2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,101, FALSE)</f>
@@ -32061,7 +32094,7 @@
       </c>
       <c r="CY2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,103, FALSE)</f>
-        <v>19.01635199500545, -98.19894850064507</v>
+        <v>19.016349983466032, -98.25408282595988</v>
       </c>
       <c r="CZ2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,104, FALSE)</f>
@@ -32091,113 +32124,113 @@
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,110, FALSE)</f>
         <v>Reglamento de la Ley del Sistema Estatal de Protección Civil para el Estado Libre y Soberano de Puebla, publicado el 1 de julio de 1998.</v>
       </c>
-      <c r="DG2">
+      <c r="DG2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,111, FALSE)</f>
-        <v>0</v>
+        <v>MB67587</v>
       </c>
       <c r="DH2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,112, FALSE)</f>
-        <v>JOSE CACIANO GARCIA SANTIAGO</v>
+        <v>MARIA MERCEDES RAMIREZ H</v>
       </c>
       <c r="DI2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,113, FALSE)</f>
-        <v>MB77651</v>
+        <v>MB56662</v>
       </c>
       <c r="DJ2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,114, FALSE)</f>
-        <v>MIRIAM CORAL ZAYAGO MOJICA</v>
+        <v>JAZMIN VALENCIA DE LA CRUZ</v>
       </c>
       <c r="DK2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,115, FALSE)</f>
-        <v>BANQUERO POOL</v>
+        <v>ASESOR DIGITAL</v>
       </c>
       <c r="DL2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,116, FALSE)</f>
-        <v>MB77868</v>
+        <v>MI20213</v>
       </c>
       <c r="DM2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,117, FALSE)</f>
-        <v>VICTORIA ALEJANDRA HERNANDEZ SOLIS</v>
+        <v>JULIO GABRIEL CORTES CABRERA</v>
       </c>
       <c r="DN2" s="5" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,118, FALSE)</f>
-        <v>ASESOR DIGITAL</v>
+        <v>BANQUERO JR</v>
       </c>
       <c r="DO2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,119, FALSE)</f>
-        <v>MI22403</v>
+        <v>MI05034</v>
       </c>
       <c r="DP2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,120, FALSE)</f>
-        <v>EDUARDO ARTURO ORTEGA QUINTERO</v>
+        <v>YUNIS FLORES ANGON</v>
       </c>
       <c r="DQ2" s="5" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,121, FALSE)</f>
-        <v>ASESOR DIGITAL</v>
+        <v>CAJERO UNIVERSAL B</v>
       </c>
       <c r="DR2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,122, FALSE)</f>
-        <v>MI23928</v>
+        <v>MB88363</v>
       </c>
       <c r="DS2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,123, FALSE)</f>
-        <v>MIGUEL ANGEL FONSECA GUTIERREZ</v>
+        <v>ABIGAIL VICTORIANO HERNANDEZ</v>
       </c>
       <c r="DT2" s="5" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,124, FALSE)</f>
-        <v>BANQUERO POOL</v>
+        <v>CAJERO UNIVERSAL B</v>
       </c>
       <c r="DU2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,125, FALSE)</f>
-        <v>MI10709</v>
+        <v>MB86803</v>
       </c>
       <c r="DV2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,126, FALSE)</f>
-        <v>GLADYS PEREZ SALAZAR</v>
+        <v>KATIA XIMENA CANO RODRIGUEZ</v>
       </c>
       <c r="DW2" s="5" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,127, FALSE)</f>
-        <v>JEFE DE CAJA</v>
+        <v>ASESOR DIGITAL</v>
       </c>
       <c r="DX2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,128, FALSE)</f>
-        <v>M821641</v>
+        <v>MI22288</v>
       </c>
       <c r="DY2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,129, FALSE)</f>
-        <v>ANA LAURA FLORES SERRANO</v>
+        <v>KATIA XIMENA CANO RODRIGUEZ</v>
       </c>
       <c r="DZ2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,130, FALSE)</f>
-        <v>CAJERO UNIVERSAL B</v>
+        <v>ASESOR DIGITAL</v>
       </c>
       <c r="EA2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,131, FALSE)</f>
-        <v>M841691</v>
+        <v>MI22288</v>
       </c>
       <c r="EB2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,132, FALSE)</f>
-        <v>VICTOR CONCEPCION SUAREZ FLORES</v>
+        <v>MARIA LETICIA GONZALEZ SANCHEZ</v>
       </c>
       <c r="EC2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,133, FALSE)</f>
-        <v>CAJERO UNIVERSAL B</v>
+        <v>CAJERO UNIVERSAL A</v>
       </c>
       <c r="ED2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,134, FALSE)</f>
-        <v>MB95251</v>
-      </c>
-      <c r="EE2">
+        <v>M813725</v>
+      </c>
+      <c r="EE2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,135, FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="EF2">
+        <v>DAMAYANTI RODRIGUEZ CORDOBA</v>
+      </c>
+      <c r="EF2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,136, FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="EG2">
+        <v>BANQUERO JR</v>
+      </c>
+      <c r="EG2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,137, FALSE)</f>
-        <v>0</v>
+        <v>MI22132</v>
       </c>
       <c r="EH2">
         <f>VLOOKUP($A$1,BD!$A$3:$HC$210,138, FALSE)</f>
@@ -32561,7 +32594,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4A8EE80-4440-4B18-8DA6-6D8F054BB32D}">
-  <dimension ref="C1:V179"/>
+  <dimension ref="C1:V181"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="3:22" x14ac:dyDescent="0.3">
@@ -39605,7 +39638,7 @@
         <v>332</v>
       </c>
       <c r="K143" t="str">
-        <f t="shared" ref="K143:K179" si="34">+_xlfn.CONCAT("'",I143,"' : r_val['",I143,"'],")</f>
+        <f t="shared" ref="K143:K181" si="34">+_xlfn.CONCAT("'",I143,"' : r_val['",I143,"'],")</f>
         <v>'descrip_lc' : r_val['descrip_lc'],</v>
       </c>
     </row>
@@ -40039,6 +40072,32 @@
       <c r="K179" t="str">
         <f t="shared" si="34"/>
         <v>'m10' : r_val['m10'],</v>
+      </c>
+    </row>
+    <row r="180" spans="9:11" x14ac:dyDescent="0.3">
+      <c r="I180" t="s">
+        <v>1730</v>
+      </c>
+      <c r="J180" t="str">
+        <f>+_xlfn.CONCAT("{{ ",I180," }}")</f>
+        <v>{{ registro_perito }}</v>
+      </c>
+      <c r="K180" t="str">
+        <f t="shared" si="34"/>
+        <v>'registro_perito' : r_val['registro_perito'],</v>
+      </c>
+    </row>
+    <row r="181" spans="9:11" x14ac:dyDescent="0.3">
+      <c r="I181" t="s">
+        <v>1731</v>
+      </c>
+      <c r="J181" t="str">
+        <f>+_xlfn.CONCAT("{{ ",I181," }}")</f>
+        <v>{{ no_registro }}</v>
+      </c>
+      <c r="K181" t="str">
+        <f t="shared" si="34"/>
+        <v>'no_registro' : r_val['no_registro'],</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se agrega imagen 'corresp1'
</commit_message>
<xml_diff>
--- a/Inputs/BD.xlsx
+++ b/Inputs/BD.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/078e1a455e5c02ce/Documentos/GitHub/Proyecto_PIPC/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2861" documentId="13_ncr:1_{7D3A426E-EC5E-453A-8CC7-F83B71F24F18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DBE3CA1D-ADA2-4AD1-BDDC-5B0B8442EB46}"/>
+  <xr:revisionPtr revIDLastSave="2872" documentId="13_ncr:1_{7D3A426E-EC5E-453A-8CC7-F83B71F24F18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{13ABC23B-9C10-4F43-BB9C-F9DD185C515F}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{3F095A75-F066-4695-8672-8D4315F1EF23}"/>
   </bookViews>
@@ -539,7 +539,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5674" uniqueCount="1761">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5680" uniqueCount="1762">
   <si>
     <t>dia</t>
   </si>
@@ -5822,6 +5822,9 @@
   </si>
   <si>
     <t>layout.png</t>
+  </si>
+  <si>
+    <t>corresp1</t>
   </si>
 </sst>
 </file>
@@ -31909,10 +31912,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76893F01-97EA-43A4-9AE2-ED099B9448DD}">
-  <dimension ref="A1:JA2"/>
+  <dimension ref="A1:JB2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:261" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:262" x14ac:dyDescent="0.3">
       <c r="A1">
         <f>+BD!A1</f>
         <v>38</v>
@@ -32697,8 +32700,11 @@
       <c r="JA1" t="s">
         <v>949</v>
       </c>
+      <c r="JB1" t="s">
+        <v>1761</v>
+      </c>
     </row>
-    <row r="2" spans="1:261" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:262" x14ac:dyDescent="0.3">
       <c r="B2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HP$210,2, FALSE)</f>
         <v>BBVA</v>
@@ -33646,6 +33652,10 @@
       </c>
       <c r="JA2" t="s">
         <v>950</v>
+      </c>
+      <c r="JB2" t="str">
+        <f>+_xlfn.CONCAT(JB1,".png")</f>
+        <v>corresp1.png</v>
       </c>
     </row>
   </sheetData>
@@ -38484,7 +38494,7 @@
         <v>'sismo_incendio' : r_val['sismo_incendio'],</v>
       </c>
       <c r="M67" t="str">
-        <f t="shared" ref="M67:M92" si="13">+_xlfn.CONCAT("'",E67,"': ",E67,",")</f>
+        <f t="shared" ref="M67:M93" si="13">+_xlfn.CONCAT("'",E67,"': ",E67,",")</f>
         <v>'plano': plano,</v>
       </c>
       <c r="N67" t="s">
@@ -40285,37 +40295,37 @@
         <v>558</v>
       </c>
       <c r="O91" t="str">
-        <f t="shared" ref="O91:O92" si="26">+_xlfn.CONCAT("img_path_",E91," = os.path.join(IMAGES_PATH, r_val[""",E91,"""])")</f>
+        <f t="shared" ref="O91:O93" si="26">+_xlfn.CONCAT("img_path_",E91," = os.path.join(IMAGES_PATH, r_val[""",E91,"""])")</f>
         <v>img_path_visitas = os.path.join(IMAGES_PATH, r_val["visitas"])</v>
       </c>
       <c r="P91" t="str">
-        <f t="shared" ref="P91:P92" si="27">+_xlfn.CONCAT("if os.path.exists(img_path_",E91,"):")</f>
+        <f t="shared" ref="P91:P93" si="27">+_xlfn.CONCAT("if os.path.exists(img_path_",E91,"):")</f>
         <v>if os.path.exists(img_path_visitas):</v>
       </c>
       <c r="Q91" t="str">
-        <f t="shared" ref="Q91:Q92" si="28">+_xlfn.CONCAT(E91," = InlineImage(docx_tpl, img_path_",E91,", height=Mm(",H91,"))")</f>
+        <f t="shared" ref="Q91:Q93" si="28">+_xlfn.CONCAT(E91," = InlineImage(docx_tpl, img_path_",E91,", height=Mm(",H91,"))")</f>
         <v>visitas = InlineImage(docx_tpl, img_path_visitas, height=Mm(155))</v>
       </c>
       <c r="R91" t="s">
         <v>560</v>
       </c>
       <c r="S91" t="str">
-        <f t="shared" ref="S91:S92" si="29">+_xlfn.CONCAT("print(f'Advertencia: No se encontró la imagen {r_val[""",E91,"""]}')")</f>
+        <f t="shared" ref="S91:S93" si="29">+_xlfn.CONCAT("print(f'Advertencia: No se encontró la imagen {r_val[""",E91,"""]}')")</f>
         <v>print(f'Advertencia: No se encontró la imagen {r_val["visitas"]}')</v>
       </c>
       <c r="T91" t="str">
-        <f t="shared" ref="T91:T92" si="30">+_xlfn.CONCAT(E91," = ''")</f>
+        <f t="shared" ref="T91:T93" si="30">+_xlfn.CONCAT(E91," = ''")</f>
         <v>visitas = ''</v>
       </c>
       <c r="U91" t="s">
         <v>559</v>
       </c>
       <c r="V91" t="str">
-        <f t="shared" ref="V91:V92" si="31">+_xlfn.CONCAT("print(f'Advertencia: No se pudo cargar la imagen {r_val[""",E91,"""]}: {e}')")</f>
+        <f t="shared" ref="V91:V93" si="31">+_xlfn.CONCAT("print(f'Advertencia: No se pudo cargar la imagen {r_val[""",E91,"""]}: {e}')")</f>
         <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["visitas"]}: {e}')</v>
       </c>
       <c r="W91" t="str">
-        <f t="shared" ref="W91:W92" si="32">+_xlfn.CONCAT(E91," = ''")</f>
+        <f t="shared" ref="W91:W93" si="32">+_xlfn.CONCAT(E91," = ''")</f>
         <v>visitas = ''</v>
       </c>
     </row>
@@ -40394,6 +40404,23 @@
       </c>
     </row>
     <row r="93" spans="3:23" x14ac:dyDescent="0.3">
+      <c r="E93" t="s">
+        <v>1761</v>
+      </c>
+      <c r="F93" t="str">
+        <f>+_xlfn.CONCAT(E93,".png")</f>
+        <v>corresp1.png</v>
+      </c>
+      <c r="G93" t="str">
+        <f>+_xlfn.CONCAT("{{ ",E93," }}")</f>
+        <v>{{ corresp1 }}</v>
+      </c>
+      <c r="H93">
+        <v>155</v>
+      </c>
+      <c r="I93" t="s">
+        <v>1758</v>
+      </c>
       <c r="J93" t="s">
         <v>23</v>
       </c>
@@ -40403,6 +40430,47 @@
       <c r="L93" t="str">
         <f t="shared" si="25"/>
         <v>'tambo_arena' : r_val['tambo_arena'],</v>
+      </c>
+      <c r="M93" t="str">
+        <f t="shared" si="13"/>
+        <v>'corresp1': corresp1,</v>
+      </c>
+      <c r="N93" t="s">
+        <v>558</v>
+      </c>
+      <c r="O93" t="str">
+        <f t="shared" si="26"/>
+        <v>img_path_corresp1 = os.path.join(IMAGES_PATH, r_val["corresp1"])</v>
+      </c>
+      <c r="P93" t="str">
+        <f t="shared" si="27"/>
+        <v>if os.path.exists(img_path_corresp1):</v>
+      </c>
+      <c r="Q93" s="1" t="str">
+        <f>+_xlfn.CONCAT(E93," = InlineImage(docx_tpl, img_path_",E93,", ",I93,"=Mm(",H93,"))")</f>
+        <v>corresp1 = InlineImage(docx_tpl, img_path_corresp1, width=Mm(155))</v>
+      </c>
+      <c r="R93" t="s">
+        <v>560</v>
+      </c>
+      <c r="S93" t="str">
+        <f t="shared" si="29"/>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["corresp1"]}')</v>
+      </c>
+      <c r="T93" t="str">
+        <f t="shared" si="30"/>
+        <v>corresp1 = ''</v>
+      </c>
+      <c r="U93" t="s">
+        <v>559</v>
+      </c>
+      <c r="V93" t="str">
+        <f t="shared" si="31"/>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["corresp1"]}: {e}')</v>
+      </c>
+      <c r="W93" t="str">
+        <f t="shared" si="32"/>
+        <v>corresp1 = ''</v>
       </c>
     </row>
     <row r="94" spans="3:23" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Se agregan imagenes para pipc BBVA
</commit_message>
<xml_diff>
--- a/Inputs/BD.xlsx
+++ b/Inputs/BD.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/078e1a455e5c02ce/Documentos/GitHub/Proyecto_PIPC/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2872" documentId="13_ncr:1_{7D3A426E-EC5E-453A-8CC7-F83B71F24F18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{13ABC23B-9C10-4F43-BB9C-F9DD185C515F}"/>
+  <xr:revisionPtr revIDLastSave="2913" documentId="13_ncr:1_{7D3A426E-EC5E-453A-8CC7-F83B71F24F18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{13B4B3A0-B833-4C48-85B8-DDDF8DA6B11D}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{3F095A75-F066-4695-8672-8D4315F1EF23}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3F095A75-F066-4695-8672-8D4315F1EF23}"/>
   </bookViews>
   <sheets>
     <sheet name="BD" sheetId="1" r:id="rId1"/>
@@ -539,7 +539,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5680" uniqueCount="1762">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5783" uniqueCount="1785">
   <si>
     <t>dia</t>
   </si>
@@ -5825,6 +5825,75 @@
   </si>
   <si>
     <t>corresp1</t>
+  </si>
+  <si>
+    <t>corresp2</t>
+  </si>
+  <si>
+    <t>corresp3</t>
+  </si>
+  <si>
+    <t>carta_respon</t>
+  </si>
+  <si>
+    <t>registro1</t>
+  </si>
+  <si>
+    <t>registro2</t>
+  </si>
+  <si>
+    <t>ries_circ</t>
+  </si>
+  <si>
+    <t>mapa_ext</t>
+  </si>
+  <si>
+    <t>rec_ext</t>
+  </si>
+  <si>
+    <t>mayor_ries</t>
+  </si>
+  <si>
+    <t>menor_ries</t>
+  </si>
+  <si>
+    <t>zona_evac</t>
+  </si>
+  <si>
+    <t>corresp1.png</t>
+  </si>
+  <si>
+    <t>corresp2.png</t>
+  </si>
+  <si>
+    <t>corresp3.png</t>
+  </si>
+  <si>
+    <t>carta_respon.png</t>
+  </si>
+  <si>
+    <t>registro1.png</t>
+  </si>
+  <si>
+    <t>registro2.png</t>
+  </si>
+  <si>
+    <t>ries_circ.png</t>
+  </si>
+  <si>
+    <t>mapa_ext.png</t>
+  </si>
+  <si>
+    <t>rec_ext.png</t>
+  </si>
+  <si>
+    <t>mayor_ries.png</t>
+  </si>
+  <si>
+    <t>menor_ries.png</t>
+  </si>
+  <si>
+    <t>zona_evac.png</t>
   </si>
 </sst>
 </file>
@@ -6865,15 +6934,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE6A0106-4EDF-4D58-B8A9-1C9CC54D9FE0}">
-  <dimension ref="A1:KH201"/>
+  <dimension ref="A1:KT201"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:294" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:306" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2">
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:294" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:306" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>133</v>
       </c>
@@ -7658,106 +7727,142 @@
         <v>949</v>
       </c>
       <c r="JB2" t="s">
+        <v>1761</v>
+      </c>
+      <c r="JC2" t="s">
+        <v>1762</v>
+      </c>
+      <c r="JD2" t="s">
+        <v>1763</v>
+      </c>
+      <c r="JE2" t="s">
+        <v>1764</v>
+      </c>
+      <c r="JF2" t="s">
+        <v>1765</v>
+      </c>
+      <c r="JG2" t="s">
+        <v>1766</v>
+      </c>
+      <c r="JH2" t="s">
+        <v>1767</v>
+      </c>
+      <c r="JI2" t="s">
+        <v>1768</v>
+      </c>
+      <c r="JJ2" t="s">
+        <v>1769</v>
+      </c>
+      <c r="JK2" t="s">
+        <v>1770</v>
+      </c>
+      <c r="JL2" t="s">
+        <v>1771</v>
+      </c>
+      <c r="JM2" t="s">
+        <v>1772</v>
+      </c>
+      <c r="JN2" t="s">
         <v>621</v>
       </c>
-      <c r="JC2" t="s">
+      <c r="JO2" t="s">
         <v>622</v>
       </c>
-      <c r="JD2" t="s">
+      <c r="JP2" t="s">
         <v>639</v>
       </c>
-      <c r="JE2" t="s">
+      <c r="JQ2" t="s">
         <v>623</v>
       </c>
-      <c r="JF2" t="s">
+      <c r="JR2" t="s">
         <v>624</v>
       </c>
-      <c r="JG2" t="s">
+      <c r="JS2" t="s">
         <v>640</v>
       </c>
-      <c r="JH2" t="s">
+      <c r="JT2" t="s">
         <v>625</v>
       </c>
-      <c r="JI2" t="s">
+      <c r="JU2" t="s">
         <v>626</v>
       </c>
-      <c r="JJ2" t="s">
+      <c r="JV2" t="s">
         <v>641</v>
       </c>
-      <c r="JK2" t="s">
+      <c r="JW2" t="s">
         <v>627</v>
       </c>
-      <c r="JL2" t="s">
+      <c r="JX2" t="s">
         <v>628</v>
       </c>
-      <c r="JM2" t="s">
+      <c r="JY2" t="s">
         <v>642</v>
       </c>
-      <c r="JN2" t="s">
+      <c r="JZ2" t="s">
         <v>629</v>
       </c>
-      <c r="JO2" t="s">
+      <c r="KA2" t="s">
         <v>630</v>
       </c>
-      <c r="JP2" t="s">
+      <c r="KB2" t="s">
         <v>643</v>
       </c>
-      <c r="JQ2" t="s">
+      <c r="KC2" t="s">
         <v>631</v>
       </c>
-      <c r="JR2" t="s">
+      <c r="KD2" t="s">
         <v>632</v>
       </c>
-      <c r="JS2" t="s">
+      <c r="KE2" t="s">
         <v>644</v>
       </c>
-      <c r="JT2" t="s">
+      <c r="KF2" t="s">
         <v>633</v>
       </c>
-      <c r="JU2" t="s">
+      <c r="KG2" t="s">
         <v>634</v>
       </c>
-      <c r="JV2" t="s">
+      <c r="KH2" t="s">
         <v>645</v>
       </c>
-      <c r="JW2" t="s">
+      <c r="KI2" t="s">
         <v>635</v>
       </c>
-      <c r="JX2" t="s">
+      <c r="KJ2" t="s">
         <v>636</v>
       </c>
-      <c r="JY2" t="s">
+      <c r="KK2" t="s">
         <v>646</v>
       </c>
-      <c r="JZ2" t="s">
+      <c r="KL2" t="s">
         <v>1715</v>
       </c>
-      <c r="KA2" t="s">
+      <c r="KM2" t="s">
         <v>1716</v>
       </c>
-      <c r="KB2" t="s">
+      <c r="KN2" t="s">
         <v>1717</v>
       </c>
-      <c r="KC2" t="s">
+      <c r="KO2" t="s">
         <v>1718</v>
       </c>
-      <c r="KD2" t="s">
+      <c r="KP2" t="s">
         <v>1719</v>
       </c>
-      <c r="KE2" t="s">
+      <c r="KQ2" t="s">
         <v>1720</v>
       </c>
-      <c r="KF2" t="s">
+      <c r="KR2" t="s">
         <v>1721</v>
       </c>
-      <c r="KG2" t="s">
+      <c r="KS2" t="s">
         <v>1722</v>
       </c>
-      <c r="KH2" t="s">
+      <c r="KT2" t="s">
         <v>1723</v>
       </c>
     </row>
-    <row r="3" spans="1:294" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:306" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
@@ -8040,7 +8145,7 @@
         <v>ORDINARIO</v>
       </c>
     </row>
-    <row r="4" spans="1:294" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:306" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2</v>
       </c>
@@ -8317,7 +8422,7 @@
         <v>ORDINARIO</v>
       </c>
     </row>
-    <row r="5" spans="1:294" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:306" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>3</v>
       </c>
@@ -8600,7 +8705,7 @@
         <v>ORDINARIO</v>
       </c>
     </row>
-    <row r="6" spans="1:294" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:306" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>4</v>
       </c>
@@ -8877,7 +8982,7 @@
         <v>ORDINARIO</v>
       </c>
     </row>
-    <row r="7" spans="1:294" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:306" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>5</v>
       </c>
@@ -9151,7 +9256,7 @@
         <v>ORDINARIO</v>
       </c>
     </row>
-    <row r="8" spans="1:294" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:306" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>6</v>
       </c>
@@ -9461,7 +9566,7 @@
         <v>ALTO</v>
       </c>
     </row>
-    <row r="9" spans="1:294" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:306" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>7</v>
       </c>
@@ -9744,7 +9849,7 @@
         <v>ALTO</v>
       </c>
     </row>
-    <row r="10" spans="1:294" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:306" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>8</v>
       </c>
@@ -10057,7 +10162,7 @@
         <v>ALTO</v>
       </c>
     </row>
-    <row r="11" spans="1:294" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:306" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>9</v>
       </c>
@@ -10379,7 +10484,7 @@
         <v>ALTO</v>
       </c>
     </row>
-    <row r="12" spans="1:294" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:306" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>10</v>
       </c>
@@ -10680,7 +10785,7 @@
         <v>ALTO</v>
       </c>
     </row>
-    <row r="13" spans="1:294" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:306" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>11</v>
       </c>
@@ -10978,7 +11083,7 @@
         <v>ALTO</v>
       </c>
     </row>
-    <row r="14" spans="1:294" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:306" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>12</v>
       </c>
@@ -11491,107 +11596,107 @@
       <c r="JA14" t="s">
         <v>843</v>
       </c>
-      <c r="JB14" t="s">
+      <c r="JN14" t="s">
         <v>890</v>
       </c>
-      <c r="JC14" t="s">
+      <c r="JO14" t="s">
         <v>877</v>
       </c>
-      <c r="JD14" t="s">
+      <c r="JP14" t="s">
         <v>891</v>
       </c>
-      <c r="JE14" t="s">
+      <c r="JQ14" t="s">
         <v>892</v>
       </c>
-      <c r="JF14" t="s">
+      <c r="JR14" t="s">
         <v>877</v>
       </c>
-      <c r="JG14" t="s">
+      <c r="JS14" t="s">
         <v>893</v>
       </c>
-      <c r="JH14" t="s">
+      <c r="JT14" t="s">
         <v>894</v>
       </c>
-      <c r="JI14" t="s">
+      <c r="JU14" t="s">
         <v>865</v>
       </c>
-      <c r="JJ14" t="s">
+      <c r="JV14" t="s">
         <v>895</v>
       </c>
-      <c r="JK14" t="s">
+      <c r="JW14" t="s">
         <v>896</v>
-      </c>
-      <c r="JL14" t="s">
-        <v>868</v>
-      </c>
-      <c r="JM14" t="s">
-        <v>897</v>
-      </c>
-      <c r="JN14" t="s">
-        <v>898</v>
-      </c>
-      <c r="JO14" t="s">
-        <v>868</v>
-      </c>
-      <c r="JP14" t="s">
-        <v>899</v>
-      </c>
-      <c r="JQ14" t="s">
-        <v>900</v>
-      </c>
-      <c r="JR14" t="s">
-        <v>868</v>
-      </c>
-      <c r="JS14" t="s">
-        <v>901</v>
-      </c>
-      <c r="JT14" t="s">
-        <v>902</v>
-      </c>
-      <c r="JU14" t="s">
-        <v>868</v>
-      </c>
-      <c r="JV14" t="s">
-        <v>903</v>
-      </c>
-      <c r="JW14" t="s">
-        <v>904</v>
       </c>
       <c r="JX14" t="s">
         <v>868</v>
       </c>
       <c r="JY14" t="s">
-        <v>905</v>
+        <v>897</v>
       </c>
       <c r="JZ14" t="s">
-        <v>906</v>
+        <v>898</v>
       </c>
       <c r="KA14" t="s">
         <v>868</v>
       </c>
       <c r="KB14" t="s">
+        <v>899</v>
+      </c>
+      <c r="KC14" t="s">
+        <v>900</v>
+      </c>
+      <c r="KD14" t="s">
+        <v>868</v>
+      </c>
+      <c r="KE14" t="s">
+        <v>901</v>
+      </c>
+      <c r="KF14" t="s">
+        <v>902</v>
+      </c>
+      <c r="KG14" t="s">
+        <v>868</v>
+      </c>
+      <c r="KH14" t="s">
+        <v>903</v>
+      </c>
+      <c r="KI14" t="s">
+        <v>904</v>
+      </c>
+      <c r="KJ14" t="s">
+        <v>868</v>
+      </c>
+      <c r="KK14" t="s">
+        <v>905</v>
+      </c>
+      <c r="KL14" t="s">
+        <v>906</v>
+      </c>
+      <c r="KM14" t="s">
+        <v>868</v>
+      </c>
+      <c r="KN14" t="s">
         <v>907</v>
       </c>
-      <c r="KC14" t="s">
+      <c r="KO14" t="s">
         <v>908</v>
       </c>
-      <c r="KD14" t="s">
+      <c r="KP14" t="s">
         <v>874</v>
       </c>
-      <c r="KE14" t="s">
+      <c r="KQ14" t="s">
         <v>909</v>
       </c>
-      <c r="KF14" t="s">
+      <c r="KR14" t="s">
         <v>910</v>
       </c>
-      <c r="KG14" t="s">
+      <c r="KS14" t="s">
         <v>874</v>
       </c>
-      <c r="KH14" t="s">
+      <c r="KT14" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="15" spans="1:294" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:306" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>13</v>
       </c>
@@ -12136,35 +12241,35 @@
       <c r="JA15" t="s">
         <v>843</v>
       </c>
-      <c r="JB15" t="s">
+      <c r="JN15" t="s">
         <v>939</v>
       </c>
-      <c r="JC15" t="s">
+      <c r="JO15" t="s">
         <v>868</v>
       </c>
-      <c r="JD15" t="s">
+      <c r="JP15" t="s">
         <v>940</v>
       </c>
-      <c r="JE15" t="s">
+      <c r="JQ15" t="s">
         <v>941</v>
       </c>
-      <c r="JF15" t="s">
+      <c r="JR15" t="s">
         <v>868</v>
       </c>
-      <c r="JG15" t="s">
+      <c r="JS15" t="s">
         <v>942</v>
       </c>
-      <c r="JH15" t="s">
+      <c r="JT15" t="s">
         <v>943</v>
       </c>
-      <c r="JI15" t="s">
+      <c r="JU15" t="s">
         <v>871</v>
       </c>
-      <c r="JJ15" t="s">
+      <c r="JV15" t="s">
         <v>944</v>
       </c>
     </row>
-    <row r="16" spans="1:294" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:306" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>14</v>
       </c>
@@ -12650,7 +12755,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="17" spans="1:267" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:279" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>15</v>
       </c>
@@ -13141,7 +13246,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="18" spans="1:267" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:279" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>16</v>
       </c>
@@ -13640,7 +13745,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="19" spans="1:267" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:279" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>17</v>
       </c>
@@ -14157,7 +14262,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="20" spans="1:267" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:279" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>18</v>
       </c>
@@ -14672,17 +14777,17 @@
       <c r="JA20" t="s">
         <v>843</v>
       </c>
-      <c r="JB20" t="s">
+      <c r="JN20" t="s">
         <v>1085</v>
       </c>
-      <c r="JC20" t="s">
+      <c r="JO20" t="s">
         <v>868</v>
       </c>
-      <c r="JD20" t="s">
+      <c r="JP20" t="s">
         <v>1086</v>
       </c>
     </row>
-    <row r="21" spans="1:267" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:279" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>19</v>
       </c>
@@ -15144,7 +15249,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="22" spans="1:267" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:279" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>20</v>
       </c>
@@ -15646,7 +15751,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="23" spans="1:267" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:279" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>21</v>
       </c>
@@ -16162,7 +16267,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="24" spans="1:267" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:279" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>22</v>
       </c>
@@ -16684,7 +16789,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="25" spans="1:267" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:279" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>23</v>
       </c>
@@ -17177,7 +17282,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="26" spans="1:267" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:279" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>24</v>
       </c>
@@ -17677,7 +17782,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="27" spans="1:267" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:279" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>25</v>
       </c>
@@ -18167,7 +18272,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="28" spans="1:267" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:279" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>26</v>
       </c>
@@ -18679,7 +18784,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="29" spans="1:267" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:279" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>27</v>
       </c>
@@ -19202,23 +19307,23 @@
       <c r="JA29" t="s">
         <v>843</v>
       </c>
-      <c r="JB29" t="s">
+      <c r="JN29" t="s">
         <v>1309</v>
       </c>
-      <c r="JC29" t="s">
+      <c r="JO29" t="s">
         <v>874</v>
       </c>
-      <c r="JE29" t="s">
+      <c r="JQ29" t="s">
         <v>1310</v>
       </c>
-      <c r="JF29" t="s">
+      <c r="JR29" t="s">
         <v>874</v>
       </c>
-      <c r="JG29" t="s">
+      <c r="JS29" t="s">
         <v>1311</v>
       </c>
     </row>
-    <row r="30" spans="1:267" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:279" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>28</v>
       </c>
@@ -19709,7 +19814,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="31" spans="1:267" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:279" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>29</v>
       </c>
@@ -20212,7 +20317,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="32" spans="1:267" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:279" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>30</v>
       </c>
@@ -20715,7 +20820,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="33" spans="1:279" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:291" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>31</v>
       </c>
@@ -21196,7 +21301,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="34" spans="1:279" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:291" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>32</v>
       </c>
@@ -21685,7 +21790,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="35" spans="1:279" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:291" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>33</v>
       </c>
@@ -22188,7 +22293,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="36" spans="1:279" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:291" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>34</v>
       </c>
@@ -22692,7 +22797,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="37" spans="1:279" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:291" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>35</v>
       </c>
@@ -23189,7 +23294,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="38" spans="1:279" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:291" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>36</v>
       </c>
@@ -23685,7 +23790,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="39" spans="1:279" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:291" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>37</v>
       </c>
@@ -24208,62 +24313,62 @@
       <c r="JA39" t="s">
         <v>843</v>
       </c>
-      <c r="JB39" t="s">
+      <c r="JN39" t="s">
         <v>1572</v>
       </c>
-      <c r="JC39" t="s">
+      <c r="JO39" t="s">
         <v>868</v>
       </c>
-      <c r="JD39" t="s">
+      <c r="JP39" t="s">
         <v>1573</v>
       </c>
-      <c r="JE39" t="s">
+      <c r="JQ39" t="s">
         <v>1574</v>
-      </c>
-      <c r="JF39" t="s">
-        <v>868</v>
-      </c>
-      <c r="JG39" t="s">
-        <v>1575</v>
-      </c>
-      <c r="JH39" t="s">
-        <v>1576</v>
-      </c>
-      <c r="JI39" t="s">
-        <v>884</v>
-      </c>
-      <c r="JJ39" t="s">
-        <v>1577</v>
-      </c>
-      <c r="JK39" t="s">
-        <v>1578</v>
-      </c>
-      <c r="JL39" t="s">
-        <v>868</v>
-      </c>
-      <c r="JM39" t="s">
-        <v>1579</v>
-      </c>
-      <c r="JN39" t="s">
-        <v>1580</v>
-      </c>
-      <c r="JO39" t="s">
-        <v>1230</v>
-      </c>
-      <c r="JP39" t="s">
-        <v>1581</v>
-      </c>
-      <c r="JQ39" t="s">
-        <v>1582</v>
       </c>
       <c r="JR39" t="s">
         <v>868</v>
       </c>
       <c r="JS39" t="s">
+        <v>1575</v>
+      </c>
+      <c r="JT39" t="s">
+        <v>1576</v>
+      </c>
+      <c r="JU39" t="s">
+        <v>884</v>
+      </c>
+      <c r="JV39" t="s">
+        <v>1577</v>
+      </c>
+      <c r="JW39" t="s">
+        <v>1578</v>
+      </c>
+      <c r="JX39" t="s">
+        <v>868</v>
+      </c>
+      <c r="JY39" t="s">
+        <v>1579</v>
+      </c>
+      <c r="JZ39" t="s">
+        <v>1580</v>
+      </c>
+      <c r="KA39" t="s">
+        <v>1230</v>
+      </c>
+      <c r="KB39" t="s">
+        <v>1581</v>
+      </c>
+      <c r="KC39" t="s">
+        <v>1582</v>
+      </c>
+      <c r="KD39" t="s">
+        <v>868</v>
+      </c>
+      <c r="KE39" t="s">
         <v>1583</v>
       </c>
     </row>
-    <row r="40" spans="1:279" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:291" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>38</v>
       </c>
@@ -24840,7 +24945,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="41" spans="1:279" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:291" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>39</v>
       </c>
@@ -25345,7 +25450,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="42" spans="1:279" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:291" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>40</v>
       </c>
@@ -25801,26 +25906,26 @@
       <c r="JA42" t="s">
         <v>843</v>
       </c>
-      <c r="JB42" t="s">
+      <c r="JN42" t="s">
         <v>1650</v>
       </c>
-      <c r="JC42" t="s">
+      <c r="JO42" t="s">
         <v>1321</v>
       </c>
-      <c r="JD42" t="s">
+      <c r="JP42" t="s">
         <v>1651</v>
       </c>
-      <c r="JE42" t="s">
+      <c r="JQ42" t="s">
         <v>1652</v>
       </c>
-      <c r="JF42" t="s">
+      <c r="JR42" t="s">
         <v>874</v>
       </c>
-      <c r="JG42" t="s">
+      <c r="JS42" t="s">
         <v>1653</v>
       </c>
     </row>
-    <row r="43" spans="1:279" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:291" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>41</v>
       </c>
@@ -25857,7 +25962,7 @@
         <v>ORDINARIO</v>
       </c>
     </row>
-    <row r="44" spans="1:279" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:291" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>42</v>
       </c>
@@ -25894,7 +25999,7 @@
         <v>ORDINARIO</v>
       </c>
     </row>
-    <row r="45" spans="1:279" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:291" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>43</v>
       </c>
@@ -25931,7 +26036,7 @@
         <v>ORDINARIO</v>
       </c>
     </row>
-    <row r="46" spans="1:279" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:291" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>44</v>
       </c>
@@ -25968,7 +26073,7 @@
         <v>ORDINARIO</v>
       </c>
     </row>
-    <row r="47" spans="1:279" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:291" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>45</v>
       </c>
@@ -26005,7 +26110,7 @@
         <v>ORDINARIO</v>
       </c>
     </row>
-    <row r="48" spans="1:279" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:291" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>46</v>
       </c>
@@ -31829,12 +31934,12 @@
       <formula>$A40=$A$1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="JB2:KH2">
+  <conditionalFormatting sqref="JN2:KT2">
     <cfRule type="expression" dxfId="1" priority="151">
       <formula>#REF!=$A$1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="JB14:KH42">
+  <conditionalFormatting sqref="JN14:KT42">
     <cfRule type="expression" dxfId="0" priority="152">
       <formula>$A14=$A$1</formula>
     </cfRule>
@@ -31912,10 +32017,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76893F01-97EA-43A4-9AE2-ED099B9448DD}">
-  <dimension ref="A1:JB2"/>
+  <dimension ref="A1:JM2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:262" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:273" x14ac:dyDescent="0.3">
       <c r="A1">
         <f>+BD!A1</f>
         <v>38</v>
@@ -32703,8 +32808,41 @@
       <c r="JB1" t="s">
         <v>1761</v>
       </c>
+      <c r="JC1" t="s">
+        <v>1762</v>
+      </c>
+      <c r="JD1" t="s">
+        <v>1763</v>
+      </c>
+      <c r="JE1" t="s">
+        <v>1764</v>
+      </c>
+      <c r="JF1" t="s">
+        <v>1765</v>
+      </c>
+      <c r="JG1" t="s">
+        <v>1766</v>
+      </c>
+      <c r="JH1" t="s">
+        <v>1767</v>
+      </c>
+      <c r="JI1" t="s">
+        <v>1768</v>
+      </c>
+      <c r="JJ1" t="s">
+        <v>1769</v>
+      </c>
+      <c r="JK1" t="s">
+        <v>1770</v>
+      </c>
+      <c r="JL1" t="s">
+        <v>1771</v>
+      </c>
+      <c r="JM1" t="s">
+        <v>1772</v>
+      </c>
     </row>
-    <row r="2" spans="1:262" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:273" x14ac:dyDescent="0.3">
       <c r="B2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$HP$210,2, FALSE)</f>
         <v>BBVA</v>
@@ -33653,9 +33791,41 @@
       <c r="JA2" t="s">
         <v>950</v>
       </c>
-      <c r="JB2" t="str">
-        <f>+_xlfn.CONCAT(JB1,".png")</f>
-        <v>corresp1.png</v>
+      <c r="JB2" t="s">
+        <v>1773</v>
+      </c>
+      <c r="JC2" t="s">
+        <v>1774</v>
+      </c>
+      <c r="JD2" t="s">
+        <v>1775</v>
+      </c>
+      <c r="JE2" t="s">
+        <v>1776</v>
+      </c>
+      <c r="JF2" t="s">
+        <v>1777</v>
+      </c>
+      <c r="JG2" t="s">
+        <v>1778</v>
+      </c>
+      <c r="JH2" t="s">
+        <v>1779</v>
+      </c>
+      <c r="JI2" t="s">
+        <v>1780</v>
+      </c>
+      <c r="JJ2" t="s">
+        <v>1781</v>
+      </c>
+      <c r="JK2" t="s">
+        <v>1782</v>
+      </c>
+      <c r="JL2" t="s">
+        <v>1783</v>
+      </c>
+      <c r="JM2" t="s">
+        <v>1784</v>
       </c>
     </row>
   </sheetData>
@@ -38494,7 +38664,7 @@
         <v>'sismo_incendio' : r_val['sismo_incendio'],</v>
       </c>
       <c r="M67" t="str">
-        <f t="shared" ref="M67:M93" si="13">+_xlfn.CONCAT("'",E67,"': ",E67,",")</f>
+        <f t="shared" ref="M67:M104" si="13">+_xlfn.CONCAT("'",E67,"': ",E67,",")</f>
         <v>'plano': plano,</v>
       </c>
       <c r="N67" t="s">
@@ -40303,7 +40473,7 @@
         <v>if os.path.exists(img_path_visitas):</v>
       </c>
       <c r="Q91" t="str">
-        <f t="shared" ref="Q91:Q93" si="28">+_xlfn.CONCAT(E91," = InlineImage(docx_tpl, img_path_",E91,", height=Mm(",H91,"))")</f>
+        <f t="shared" ref="Q91:Q92" si="28">+_xlfn.CONCAT(E91," = InlineImage(docx_tpl, img_path_",E91,", height=Mm(",H91,"))")</f>
         <v>visitas = InlineImage(docx_tpl, img_path_visitas, height=Mm(155))</v>
       </c>
       <c r="R91" t="s">
@@ -40404,6 +40574,9 @@
       </c>
     </row>
     <row r="93" spans="3:23" x14ac:dyDescent="0.3">
+      <c r="C93" t="s">
+        <v>843</v>
+      </c>
       <c r="E93" t="s">
         <v>1761</v>
       </c>
@@ -40474,6 +40647,26 @@
       </c>
     </row>
     <row r="94" spans="3:23" x14ac:dyDescent="0.3">
+      <c r="C94" t="s">
+        <v>843</v>
+      </c>
+      <c r="E94" t="s">
+        <v>1762</v>
+      </c>
+      <c r="F94" t="str">
+        <f t="shared" ref="F94:F104" si="33">+_xlfn.CONCAT(E94,".png")</f>
+        <v>corresp2.png</v>
+      </c>
+      <c r="G94" t="str">
+        <f t="shared" ref="G94:G104" si="34">+_xlfn.CONCAT("{{ ",E94," }}")</f>
+        <v>{{ corresp2 }}</v>
+      </c>
+      <c r="H94">
+        <v>155</v>
+      </c>
+      <c r="I94" t="s">
+        <v>1758</v>
+      </c>
       <c r="J94" t="s">
         <v>564</v>
       </c>
@@ -40484,8 +40677,69 @@
         <f t="shared" si="25"/>
         <v>'ubicacion_tambo' : r_val['ubicacion_tambo'],</v>
       </c>
+      <c r="M94" t="str">
+        <f t="shared" si="13"/>
+        <v>'corresp2': corresp2,</v>
+      </c>
+      <c r="N94" t="s">
+        <v>558</v>
+      </c>
+      <c r="O94" t="str">
+        <f t="shared" ref="O94:O104" si="35">+_xlfn.CONCAT("img_path_",E94," = os.path.join(IMAGES_PATH, r_val[""",E94,"""])")</f>
+        <v>img_path_corresp2 = os.path.join(IMAGES_PATH, r_val["corresp2"])</v>
+      </c>
+      <c r="P94" t="str">
+        <f t="shared" ref="P94:P104" si="36">+_xlfn.CONCAT("if os.path.exists(img_path_",E94,"):")</f>
+        <v>if os.path.exists(img_path_corresp2):</v>
+      </c>
+      <c r="Q94" t="str">
+        <f t="shared" ref="Q94:Q104" si="37">+_xlfn.CONCAT(E94," = InlineImage(docx_tpl, img_path_",E94,", ",I94,"=Mm(",H94,"))")</f>
+        <v>corresp2 = InlineImage(docx_tpl, img_path_corresp2, width=Mm(155))</v>
+      </c>
+      <c r="R94" t="s">
+        <v>560</v>
+      </c>
+      <c r="S94" t="str">
+        <f t="shared" ref="S94:S104" si="38">+_xlfn.CONCAT("print(f'Advertencia: No se encontró la imagen {r_val[""",E94,"""]}')")</f>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["corresp2"]}')</v>
+      </c>
+      <c r="T94" t="str">
+        <f t="shared" ref="T94:T104" si="39">+_xlfn.CONCAT(E94," = ''")</f>
+        <v>corresp2 = ''</v>
+      </c>
+      <c r="U94" t="s">
+        <v>559</v>
+      </c>
+      <c r="V94" t="str">
+        <f t="shared" ref="V94:V104" si="40">+_xlfn.CONCAT("print(f'Advertencia: No se pudo cargar la imagen {r_val[""",E94,"""]}: {e}')")</f>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["corresp2"]}: {e}')</v>
+      </c>
+      <c r="W94" t="str">
+        <f t="shared" ref="W94:W104" si="41">+_xlfn.CONCAT(E94," = ''")</f>
+        <v>corresp2 = ''</v>
+      </c>
     </row>
     <row r="95" spans="3:23" x14ac:dyDescent="0.3">
+      <c r="C95" t="s">
+        <v>843</v>
+      </c>
+      <c r="E95" t="s">
+        <v>1763</v>
+      </c>
+      <c r="F95" t="str">
+        <f t="shared" si="33"/>
+        <v>corresp3.png</v>
+      </c>
+      <c r="G95" t="str">
+        <f t="shared" si="34"/>
+        <v>{{ corresp3 }}</v>
+      </c>
+      <c r="H95">
+        <v>155</v>
+      </c>
+      <c r="I95" t="s">
+        <v>1758</v>
+      </c>
       <c r="J95" t="s">
         <v>191</v>
       </c>
@@ -40496,8 +40750,69 @@
         <f t="shared" si="25"/>
         <v>'tanques' : r_val['tanques'],</v>
       </c>
+      <c r="M95" t="str">
+        <f t="shared" si="13"/>
+        <v>'corresp3': corresp3,</v>
+      </c>
+      <c r="N95" t="s">
+        <v>558</v>
+      </c>
+      <c r="O95" t="str">
+        <f t="shared" si="35"/>
+        <v>img_path_corresp3 = os.path.join(IMAGES_PATH, r_val["corresp3"])</v>
+      </c>
+      <c r="P95" t="str">
+        <f t="shared" si="36"/>
+        <v>if os.path.exists(img_path_corresp3):</v>
+      </c>
+      <c r="Q95" t="str">
+        <f t="shared" si="37"/>
+        <v>corresp3 = InlineImage(docx_tpl, img_path_corresp3, width=Mm(155))</v>
+      </c>
+      <c r="R95" t="s">
+        <v>560</v>
+      </c>
+      <c r="S95" t="str">
+        <f t="shared" si="38"/>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["corresp3"]}')</v>
+      </c>
+      <c r="T95" t="str">
+        <f t="shared" si="39"/>
+        <v>corresp3 = ''</v>
+      </c>
+      <c r="U95" t="s">
+        <v>559</v>
+      </c>
+      <c r="V95" t="str">
+        <f t="shared" si="40"/>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["corresp3"]}: {e}')</v>
+      </c>
+      <c r="W95" t="str">
+        <f t="shared" si="41"/>
+        <v>corresp3 = ''</v>
+      </c>
     </row>
     <row r="96" spans="3:23" x14ac:dyDescent="0.3">
+      <c r="C96" t="s">
+        <v>843</v>
+      </c>
+      <c r="E96" t="s">
+        <v>1764</v>
+      </c>
+      <c r="F96" t="str">
+        <f t="shared" si="33"/>
+        <v>carta_respon.png</v>
+      </c>
+      <c r="G96" t="str">
+        <f t="shared" si="34"/>
+        <v>{{ carta_respon }}</v>
+      </c>
+      <c r="H96">
+        <v>155</v>
+      </c>
+      <c r="I96" t="s">
+        <v>1758</v>
+      </c>
       <c r="J96" t="s">
         <v>192</v>
       </c>
@@ -40508,8 +40823,69 @@
         <f t="shared" si="25"/>
         <v>'tanque_1' : r_val['tanque_1'],</v>
       </c>
+      <c r="M96" t="str">
+        <f t="shared" si="13"/>
+        <v>'carta_respon': carta_respon,</v>
+      </c>
+      <c r="N96" t="s">
+        <v>558</v>
+      </c>
+      <c r="O96" t="str">
+        <f t="shared" si="35"/>
+        <v>img_path_carta_respon = os.path.join(IMAGES_PATH, r_val["carta_respon"])</v>
+      </c>
+      <c r="P96" t="str">
+        <f t="shared" si="36"/>
+        <v>if os.path.exists(img_path_carta_respon):</v>
+      </c>
+      <c r="Q96" t="str">
+        <f t="shared" si="37"/>
+        <v>carta_respon = InlineImage(docx_tpl, img_path_carta_respon, width=Mm(155))</v>
+      </c>
+      <c r="R96" t="s">
+        <v>560</v>
+      </c>
+      <c r="S96" t="str">
+        <f t="shared" si="38"/>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["carta_respon"]}')</v>
+      </c>
+      <c r="T96" t="str">
+        <f t="shared" si="39"/>
+        <v>carta_respon = ''</v>
+      </c>
+      <c r="U96" t="s">
+        <v>559</v>
+      </c>
+      <c r="V96" t="str">
+        <f t="shared" si="40"/>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["carta_respon"]}: {e}')</v>
+      </c>
+      <c r="W96" t="str">
+        <f t="shared" si="41"/>
+        <v>carta_respon = ''</v>
+      </c>
     </row>
-    <row r="97" spans="10:12" x14ac:dyDescent="0.3">
+    <row r="97" spans="3:23" x14ac:dyDescent="0.3">
+      <c r="C97" t="s">
+        <v>843</v>
+      </c>
+      <c r="E97" t="s">
+        <v>1765</v>
+      </c>
+      <c r="F97" t="str">
+        <f t="shared" si="33"/>
+        <v>registro1.png</v>
+      </c>
+      <c r="G97" t="str">
+        <f t="shared" si="34"/>
+        <v>{{ registro1 }}</v>
+      </c>
+      <c r="H97">
+        <v>155</v>
+      </c>
+      <c r="I97" t="s">
+        <v>1758</v>
+      </c>
       <c r="J97" t="s">
         <v>193</v>
       </c>
@@ -40520,8 +40896,69 @@
         <f t="shared" si="25"/>
         <v>'tanque_2' : r_val['tanque_2'],</v>
       </c>
+      <c r="M97" t="str">
+        <f t="shared" si="13"/>
+        <v>'registro1': registro1,</v>
+      </c>
+      <c r="N97" t="s">
+        <v>558</v>
+      </c>
+      <c r="O97" t="str">
+        <f t="shared" si="35"/>
+        <v>img_path_registro1 = os.path.join(IMAGES_PATH, r_val["registro1"])</v>
+      </c>
+      <c r="P97" t="str">
+        <f t="shared" si="36"/>
+        <v>if os.path.exists(img_path_registro1):</v>
+      </c>
+      <c r="Q97" t="str">
+        <f t="shared" si="37"/>
+        <v>registro1 = InlineImage(docx_tpl, img_path_registro1, width=Mm(155))</v>
+      </c>
+      <c r="R97" t="s">
+        <v>560</v>
+      </c>
+      <c r="S97" t="str">
+        <f t="shared" si="38"/>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["registro1"]}')</v>
+      </c>
+      <c r="T97" t="str">
+        <f t="shared" si="39"/>
+        <v>registro1 = ''</v>
+      </c>
+      <c r="U97" t="s">
+        <v>559</v>
+      </c>
+      <c r="V97" t="str">
+        <f t="shared" si="40"/>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["registro1"]}: {e}')</v>
+      </c>
+      <c r="W97" t="str">
+        <f t="shared" si="41"/>
+        <v>registro1 = ''</v>
+      </c>
     </row>
-    <row r="98" spans="10:12" x14ac:dyDescent="0.3">
+    <row r="98" spans="3:23" x14ac:dyDescent="0.3">
+      <c r="C98" t="s">
+        <v>843</v>
+      </c>
+      <c r="E98" t="s">
+        <v>1766</v>
+      </c>
+      <c r="F98" t="str">
+        <f t="shared" si="33"/>
+        <v>registro2.png</v>
+      </c>
+      <c r="G98" t="str">
+        <f t="shared" si="34"/>
+        <v>{{ registro2 }}</v>
+      </c>
+      <c r="H98">
+        <v>155</v>
+      </c>
+      <c r="I98" t="s">
+        <v>1758</v>
+      </c>
       <c r="J98" t="s">
         <v>194</v>
       </c>
@@ -40532,8 +40969,69 @@
         <f t="shared" si="25"/>
         <v>'tanque_3' : r_val['tanque_3'],</v>
       </c>
+      <c r="M98" t="str">
+        <f t="shared" si="13"/>
+        <v>'registro2': registro2,</v>
+      </c>
+      <c r="N98" t="s">
+        <v>558</v>
+      </c>
+      <c r="O98" t="str">
+        <f t="shared" si="35"/>
+        <v>img_path_registro2 = os.path.join(IMAGES_PATH, r_val["registro2"])</v>
+      </c>
+      <c r="P98" t="str">
+        <f t="shared" si="36"/>
+        <v>if os.path.exists(img_path_registro2):</v>
+      </c>
+      <c r="Q98" t="str">
+        <f t="shared" si="37"/>
+        <v>registro2 = InlineImage(docx_tpl, img_path_registro2, width=Mm(155))</v>
+      </c>
+      <c r="R98" t="s">
+        <v>560</v>
+      </c>
+      <c r="S98" t="str">
+        <f t="shared" si="38"/>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["registro2"]}')</v>
+      </c>
+      <c r="T98" t="str">
+        <f t="shared" si="39"/>
+        <v>registro2 = ''</v>
+      </c>
+      <c r="U98" t="s">
+        <v>559</v>
+      </c>
+      <c r="V98" t="str">
+        <f t="shared" si="40"/>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["registro2"]}: {e}')</v>
+      </c>
+      <c r="W98" t="str">
+        <f t="shared" si="41"/>
+        <v>registro2 = ''</v>
+      </c>
     </row>
-    <row r="99" spans="10:12" x14ac:dyDescent="0.3">
+    <row r="99" spans="3:23" x14ac:dyDescent="0.3">
+      <c r="C99" t="s">
+        <v>843</v>
+      </c>
+      <c r="E99" t="s">
+        <v>1767</v>
+      </c>
+      <c r="F99" t="str">
+        <f t="shared" si="33"/>
+        <v>ries_circ.png</v>
+      </c>
+      <c r="G99" t="str">
+        <f t="shared" si="34"/>
+        <v>{{ ries_circ }}</v>
+      </c>
+      <c r="H99">
+        <v>155</v>
+      </c>
+      <c r="I99" t="s">
+        <v>1758</v>
+      </c>
       <c r="J99" t="s">
         <v>0</v>
       </c>
@@ -40544,8 +41042,69 @@
         <f t="shared" si="25"/>
         <v>'dia' : r_val['dia'],</v>
       </c>
+      <c r="M99" t="str">
+        <f t="shared" si="13"/>
+        <v>'ries_circ': ries_circ,</v>
+      </c>
+      <c r="N99" t="s">
+        <v>558</v>
+      </c>
+      <c r="O99" t="str">
+        <f t="shared" si="35"/>
+        <v>img_path_ries_circ = os.path.join(IMAGES_PATH, r_val["ries_circ"])</v>
+      </c>
+      <c r="P99" t="str">
+        <f t="shared" si="36"/>
+        <v>if os.path.exists(img_path_ries_circ):</v>
+      </c>
+      <c r="Q99" t="str">
+        <f t="shared" si="37"/>
+        <v>ries_circ = InlineImage(docx_tpl, img_path_ries_circ, width=Mm(155))</v>
+      </c>
+      <c r="R99" t="s">
+        <v>560</v>
+      </c>
+      <c r="S99" t="str">
+        <f t="shared" si="38"/>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["ries_circ"]}')</v>
+      </c>
+      <c r="T99" t="str">
+        <f t="shared" si="39"/>
+        <v>ries_circ = ''</v>
+      </c>
+      <c r="U99" t="s">
+        <v>559</v>
+      </c>
+      <c r="V99" t="str">
+        <f t="shared" si="40"/>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["ries_circ"]}: {e}')</v>
+      </c>
+      <c r="W99" t="str">
+        <f t="shared" si="41"/>
+        <v>ries_circ = ''</v>
+      </c>
     </row>
-    <row r="100" spans="10:12" x14ac:dyDescent="0.3">
+    <row r="100" spans="3:23" x14ac:dyDescent="0.3">
+      <c r="C100" t="s">
+        <v>843</v>
+      </c>
+      <c r="E100" t="s">
+        <v>1768</v>
+      </c>
+      <c r="F100" t="str">
+        <f t="shared" si="33"/>
+        <v>mapa_ext.png</v>
+      </c>
+      <c r="G100" t="str">
+        <f t="shared" si="34"/>
+        <v>{{ mapa_ext }}</v>
+      </c>
+      <c r="H100">
+        <v>155</v>
+      </c>
+      <c r="I100" t="s">
+        <v>1758</v>
+      </c>
       <c r="J100" t="s">
         <v>1</v>
       </c>
@@ -40556,8 +41115,69 @@
         <f t="shared" si="25"/>
         <v>'mes' : r_val['mes'],</v>
       </c>
+      <c r="M100" t="str">
+        <f t="shared" si="13"/>
+        <v>'mapa_ext': mapa_ext,</v>
+      </c>
+      <c r="N100" t="s">
+        <v>558</v>
+      </c>
+      <c r="O100" t="str">
+        <f t="shared" si="35"/>
+        <v>img_path_mapa_ext = os.path.join(IMAGES_PATH, r_val["mapa_ext"])</v>
+      </c>
+      <c r="P100" t="str">
+        <f t="shared" si="36"/>
+        <v>if os.path.exists(img_path_mapa_ext):</v>
+      </c>
+      <c r="Q100" t="str">
+        <f t="shared" si="37"/>
+        <v>mapa_ext = InlineImage(docx_tpl, img_path_mapa_ext, width=Mm(155))</v>
+      </c>
+      <c r="R100" t="s">
+        <v>560</v>
+      </c>
+      <c r="S100" t="str">
+        <f t="shared" si="38"/>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["mapa_ext"]}')</v>
+      </c>
+      <c r="T100" t="str">
+        <f t="shared" si="39"/>
+        <v>mapa_ext = ''</v>
+      </c>
+      <c r="U100" t="s">
+        <v>559</v>
+      </c>
+      <c r="V100" t="str">
+        <f t="shared" si="40"/>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["mapa_ext"]}: {e}')</v>
+      </c>
+      <c r="W100" t="str">
+        <f t="shared" si="41"/>
+        <v>mapa_ext = ''</v>
+      </c>
     </row>
-    <row r="101" spans="10:12" x14ac:dyDescent="0.3">
+    <row r="101" spans="3:23" x14ac:dyDescent="0.3">
+      <c r="C101" t="s">
+        <v>843</v>
+      </c>
+      <c r="E101" t="s">
+        <v>1769</v>
+      </c>
+      <c r="F101" t="str">
+        <f t="shared" si="33"/>
+        <v>rec_ext.png</v>
+      </c>
+      <c r="G101" t="str">
+        <f t="shared" si="34"/>
+        <v>{{ rec_ext }}</v>
+      </c>
+      <c r="H101">
+        <v>155</v>
+      </c>
+      <c r="I101" t="s">
+        <v>1758</v>
+      </c>
       <c r="J101" t="s">
         <v>2</v>
       </c>
@@ -40568,8 +41188,69 @@
         <f t="shared" si="25"/>
         <v>'anio' : r_val['anio'],</v>
       </c>
+      <c r="M101" t="str">
+        <f t="shared" si="13"/>
+        <v>'rec_ext': rec_ext,</v>
+      </c>
+      <c r="N101" t="s">
+        <v>558</v>
+      </c>
+      <c r="O101" t="str">
+        <f t="shared" si="35"/>
+        <v>img_path_rec_ext = os.path.join(IMAGES_PATH, r_val["rec_ext"])</v>
+      </c>
+      <c r="P101" t="str">
+        <f t="shared" si="36"/>
+        <v>if os.path.exists(img_path_rec_ext):</v>
+      </c>
+      <c r="Q101" t="str">
+        <f t="shared" si="37"/>
+        <v>rec_ext = InlineImage(docx_tpl, img_path_rec_ext, width=Mm(155))</v>
+      </c>
+      <c r="R101" t="s">
+        <v>560</v>
+      </c>
+      <c r="S101" t="str">
+        <f t="shared" si="38"/>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["rec_ext"]}')</v>
+      </c>
+      <c r="T101" t="str">
+        <f t="shared" si="39"/>
+        <v>rec_ext = ''</v>
+      </c>
+      <c r="U101" t="s">
+        <v>559</v>
+      </c>
+      <c r="V101" t="str">
+        <f t="shared" si="40"/>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["rec_ext"]}: {e}')</v>
+      </c>
+      <c r="W101" t="str">
+        <f t="shared" si="41"/>
+        <v>rec_ext = ''</v>
+      </c>
     </row>
-    <row r="102" spans="10:12" x14ac:dyDescent="0.3">
+    <row r="102" spans="3:23" x14ac:dyDescent="0.3">
+      <c r="C102" t="s">
+        <v>843</v>
+      </c>
+      <c r="E102" t="s">
+        <v>1770</v>
+      </c>
+      <c r="F102" t="str">
+        <f t="shared" si="33"/>
+        <v>mayor_ries.png</v>
+      </c>
+      <c r="G102" t="str">
+        <f t="shared" si="34"/>
+        <v>{{ mayor_ries }}</v>
+      </c>
+      <c r="H102">
+        <v>155</v>
+      </c>
+      <c r="I102" t="s">
+        <v>1758</v>
+      </c>
       <c r="J102" t="s">
         <v>195</v>
       </c>
@@ -40580,8 +41261,69 @@
         <f t="shared" si="25"/>
         <v>'coordenadas' : r_val['coordenadas'],</v>
       </c>
+      <c r="M102" t="str">
+        <f t="shared" si="13"/>
+        <v>'mayor_ries': mayor_ries,</v>
+      </c>
+      <c r="N102" t="s">
+        <v>558</v>
+      </c>
+      <c r="O102" t="str">
+        <f t="shared" si="35"/>
+        <v>img_path_mayor_ries = os.path.join(IMAGES_PATH, r_val["mayor_ries"])</v>
+      </c>
+      <c r="P102" t="str">
+        <f t="shared" si="36"/>
+        <v>if os.path.exists(img_path_mayor_ries):</v>
+      </c>
+      <c r="Q102" t="str">
+        <f t="shared" si="37"/>
+        <v>mayor_ries = InlineImage(docx_tpl, img_path_mayor_ries, width=Mm(155))</v>
+      </c>
+      <c r="R102" t="s">
+        <v>560</v>
+      </c>
+      <c r="S102" t="str">
+        <f t="shared" si="38"/>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["mayor_ries"]}')</v>
+      </c>
+      <c r="T102" t="str">
+        <f t="shared" si="39"/>
+        <v>mayor_ries = ''</v>
+      </c>
+      <c r="U102" t="s">
+        <v>559</v>
+      </c>
+      <c r="V102" t="str">
+        <f t="shared" si="40"/>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["mayor_ries"]}: {e}')</v>
+      </c>
+      <c r="W102" t="str">
+        <f t="shared" si="41"/>
+        <v>mayor_ries = ''</v>
+      </c>
     </row>
-    <row r="103" spans="10:12" x14ac:dyDescent="0.3">
+    <row r="103" spans="3:23" x14ac:dyDescent="0.3">
+      <c r="C103" t="s">
+        <v>843</v>
+      </c>
+      <c r="E103" t="s">
+        <v>1771</v>
+      </c>
+      <c r="F103" t="str">
+        <f t="shared" si="33"/>
+        <v>menor_ries.png</v>
+      </c>
+      <c r="G103" t="str">
+        <f t="shared" si="34"/>
+        <v>{{ menor_ries }}</v>
+      </c>
+      <c r="H103">
+        <v>155</v>
+      </c>
+      <c r="I103" t="s">
+        <v>1758</v>
+      </c>
       <c r="J103" t="s">
         <v>196</v>
       </c>
@@ -40592,8 +41334,69 @@
         <f t="shared" si="25"/>
         <v>'norte' : r_val['norte'],</v>
       </c>
+      <c r="M103" t="str">
+        <f t="shared" si="13"/>
+        <v>'menor_ries': menor_ries,</v>
+      </c>
+      <c r="N103" t="s">
+        <v>558</v>
+      </c>
+      <c r="O103" t="str">
+        <f t="shared" si="35"/>
+        <v>img_path_menor_ries = os.path.join(IMAGES_PATH, r_val["menor_ries"])</v>
+      </c>
+      <c r="P103" t="str">
+        <f t="shared" si="36"/>
+        <v>if os.path.exists(img_path_menor_ries):</v>
+      </c>
+      <c r="Q103" t="str">
+        <f t="shared" si="37"/>
+        <v>menor_ries = InlineImage(docx_tpl, img_path_menor_ries, width=Mm(155))</v>
+      </c>
+      <c r="R103" t="s">
+        <v>560</v>
+      </c>
+      <c r="S103" t="str">
+        <f t="shared" si="38"/>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["menor_ries"]}')</v>
+      </c>
+      <c r="T103" t="str">
+        <f t="shared" si="39"/>
+        <v>menor_ries = ''</v>
+      </c>
+      <c r="U103" t="s">
+        <v>559</v>
+      </c>
+      <c r="V103" t="str">
+        <f t="shared" si="40"/>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["menor_ries"]}: {e}')</v>
+      </c>
+      <c r="W103" t="str">
+        <f t="shared" si="41"/>
+        <v>menor_ries = ''</v>
+      </c>
     </row>
-    <row r="104" spans="10:12" x14ac:dyDescent="0.3">
+    <row r="104" spans="3:23" x14ac:dyDescent="0.3">
+      <c r="C104" t="s">
+        <v>843</v>
+      </c>
+      <c r="E104" t="s">
+        <v>1772</v>
+      </c>
+      <c r="F104" t="str">
+        <f t="shared" si="33"/>
+        <v>zona_evac.png</v>
+      </c>
+      <c r="G104" t="str">
+        <f t="shared" si="34"/>
+        <v>{{ zona_evac }}</v>
+      </c>
+      <c r="H104">
+        <v>155</v>
+      </c>
+      <c r="I104" t="s">
+        <v>1758</v>
+      </c>
       <c r="J104" t="s">
         <v>197</v>
       </c>
@@ -40604,8 +41407,52 @@
         <f t="shared" si="25"/>
         <v>'sur' : r_val['sur'],</v>
       </c>
+      <c r="M104" t="str">
+        <f t="shared" si="13"/>
+        <v>'zona_evac': zona_evac,</v>
+      </c>
+      <c r="N104" t="s">
+        <v>558</v>
+      </c>
+      <c r="O104" t="str">
+        <f t="shared" si="35"/>
+        <v>img_path_zona_evac = os.path.join(IMAGES_PATH, r_val["zona_evac"])</v>
+      </c>
+      <c r="P104" t="str">
+        <f t="shared" si="36"/>
+        <v>if os.path.exists(img_path_zona_evac):</v>
+      </c>
+      <c r="Q104" t="str">
+        <f t="shared" si="37"/>
+        <v>zona_evac = InlineImage(docx_tpl, img_path_zona_evac, width=Mm(155))</v>
+      </c>
+      <c r="R104" t="s">
+        <v>560</v>
+      </c>
+      <c r="S104" t="str">
+        <f t="shared" si="38"/>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["zona_evac"]}')</v>
+      </c>
+      <c r="T104" t="str">
+        <f t="shared" si="39"/>
+        <v>zona_evac = ''</v>
+      </c>
+      <c r="U104" t="s">
+        <v>559</v>
+      </c>
+      <c r="V104" t="str">
+        <f t="shared" si="40"/>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["zona_evac"]}: {e}')</v>
+      </c>
+      <c r="W104" t="str">
+        <f t="shared" si="41"/>
+        <v>zona_evac = ''</v>
+      </c>
     </row>
-    <row r="105" spans="10:12" x14ac:dyDescent="0.3">
+    <row r="105" spans="3:23" x14ac:dyDescent="0.3">
+      <c r="C105" t="s">
+        <v>843</v>
+      </c>
       <c r="J105" t="s">
         <v>198</v>
       </c>
@@ -40617,7 +41464,7 @@
         <v>'este' : r_val['este'],</v>
       </c>
     </row>
-    <row r="106" spans="10:12" x14ac:dyDescent="0.3">
+    <row r="106" spans="3:23" x14ac:dyDescent="0.3">
       <c r="J106" t="s">
         <v>199</v>
       </c>
@@ -40629,7 +41476,7 @@
         <v>'oeste' : r_val['oeste'],</v>
       </c>
     </row>
-    <row r="107" spans="10:12" x14ac:dyDescent="0.3">
+    <row r="107" spans="3:23" x14ac:dyDescent="0.3">
       <c r="J107" t="s">
         <v>597</v>
       </c>
@@ -40641,7 +41488,7 @@
         <v>'ref_llegar' : r_val['ref_llegar'],</v>
       </c>
     </row>
-    <row r="108" spans="10:12" x14ac:dyDescent="0.3">
+    <row r="108" spans="3:23" x14ac:dyDescent="0.3">
       <c r="J108" t="s">
         <v>200</v>
       </c>
@@ -40653,7 +41500,7 @@
         <v>'ley' : r_val['ley'],</v>
       </c>
     </row>
-    <row r="109" spans="10:12" x14ac:dyDescent="0.3">
+    <row r="109" spans="3:23" x14ac:dyDescent="0.3">
       <c r="J109" t="s">
         <v>201</v>
       </c>
@@ -40665,7 +41512,7 @@
         <v>'reglamento' : r_val['reglamento'],</v>
       </c>
     </row>
-    <row r="110" spans="10:12" x14ac:dyDescent="0.3">
+    <row r="110" spans="3:23" x14ac:dyDescent="0.3">
       <c r="J110" t="s">
         <v>647</v>
       </c>
@@ -40677,7 +41524,7 @@
         <v>'m_dir' : r_val['m_dir'],</v>
       </c>
     </row>
-    <row r="111" spans="10:12" x14ac:dyDescent="0.3">
+    <row r="111" spans="3:23" x14ac:dyDescent="0.3">
       <c r="J111" t="s">
         <v>202</v>
       </c>
@@ -40685,11 +41532,11 @@
         <v>317</v>
       </c>
       <c r="L111" t="str">
-        <f t="shared" ref="L111:L142" si="33">+_xlfn.CONCAT("'",J111,"' : r_val['",J111,"'],")</f>
+        <f t="shared" ref="L111:L142" si="42">+_xlfn.CONCAT("'",J111,"' : r_val['",J111,"'],")</f>
         <v>'coord_suplente' : r_val['coord_suplente'],</v>
       </c>
     </row>
-    <row r="112" spans="10:12" x14ac:dyDescent="0.3">
+    <row r="112" spans="3:23" x14ac:dyDescent="0.3">
       <c r="J112" t="s">
         <v>648</v>
       </c>
@@ -40697,7 +41544,7 @@
         <v>688</v>
       </c>
       <c r="L112" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="42"/>
         <v>'m_jef_caj' : r_val['m_jef_caj'],</v>
       </c>
     </row>
@@ -40709,7 +41556,7 @@
         <v>318</v>
       </c>
       <c r="L113" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="42"/>
         <v>'evacuacion' : r_val['evacuacion'],</v>
       </c>
     </row>
@@ -40721,7 +41568,7 @@
         <v>589</v>
       </c>
       <c r="L114" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="42"/>
         <v>'evac_puesto' : r_val['evac_puesto'],</v>
       </c>
     </row>
@@ -40733,7 +41580,7 @@
         <v>689</v>
       </c>
       <c r="L115" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="42"/>
         <v>'m_evac' : r_val['m_evac'],</v>
       </c>
     </row>
@@ -40745,7 +41592,7 @@
         <v>319</v>
       </c>
       <c r="L116" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="42"/>
         <v>'evac_suplente' : r_val['evac_suplente'],</v>
       </c>
     </row>
@@ -40757,7 +41604,7 @@
         <v>590</v>
       </c>
       <c r="L117" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="42"/>
         <v>'supl_evac_pue' : r_val['supl_evac_pue'],</v>
       </c>
     </row>
@@ -40769,7 +41616,7 @@
         <v>690</v>
       </c>
       <c r="L118" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="42"/>
         <v>'m_supl_evac' : r_val['m_supl_evac'],</v>
       </c>
     </row>
@@ -40781,7 +41628,7 @@
         <v>320</v>
       </c>
       <c r="L119" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="42"/>
         <v>'incendios' : r_val['incendios'],</v>
       </c>
     </row>
@@ -40793,7 +41640,7 @@
         <v>591</v>
       </c>
       <c r="L120" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="42"/>
         <v>'incen_puesto' : r_val['incen_puesto'],</v>
       </c>
     </row>
@@ -40805,7 +41652,7 @@
         <v>691</v>
       </c>
       <c r="L121" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="42"/>
         <v>'m_inc' : r_val['m_inc'],</v>
       </c>
     </row>
@@ -40817,7 +41664,7 @@
         <v>321</v>
       </c>
       <c r="L122" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="42"/>
         <v>'inc_suplente' : r_val['inc_suplente'],</v>
       </c>
     </row>
@@ -40829,7 +41676,7 @@
         <v>592</v>
       </c>
       <c r="L123" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="42"/>
         <v>'supl_inc_puesto' : r_val['supl_inc_puesto'],</v>
       </c>
     </row>
@@ -40841,7 +41688,7 @@
         <v>692</v>
       </c>
       <c r="L124" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="42"/>
         <v>'m_supl_inc' : r_val['m_supl_inc'],</v>
       </c>
     </row>
@@ -40853,7 +41700,7 @@
         <v>322</v>
       </c>
       <c r="L125" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="42"/>
         <v>'primeros_auxilios' : r_val['primeros_auxilios'],</v>
       </c>
     </row>
@@ -40865,7 +41712,7 @@
         <v>593</v>
       </c>
       <c r="L126" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="42"/>
         <v>'prim_aux_puesto' : r_val['prim_aux_puesto'],</v>
       </c>
     </row>
@@ -40877,7 +41724,7 @@
         <v>693</v>
       </c>
       <c r="L127" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="42"/>
         <v>'m_prim_aux' : r_val['m_prim_aux'],</v>
       </c>
     </row>
@@ -40889,7 +41736,7 @@
         <v>323</v>
       </c>
       <c r="L128" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="42"/>
         <v>'aux_suplente' : r_val['aux_suplente'],</v>
       </c>
     </row>
@@ -40901,7 +41748,7 @@
         <v>594</v>
       </c>
       <c r="L129" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="42"/>
         <v>'supl_prim_aux_puesto' : r_val['supl_prim_aux_puesto'],</v>
       </c>
     </row>
@@ -40913,7 +41760,7 @@
         <v>694</v>
       </c>
       <c r="L130" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="42"/>
         <v>'m_supl_paux' : r_val['m_supl_paux'],</v>
       </c>
     </row>
@@ -40925,7 +41772,7 @@
         <v>324</v>
       </c>
       <c r="L131" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="42"/>
         <v>'busqueda' : r_val['busqueda'],</v>
       </c>
     </row>
@@ -40937,7 +41784,7 @@
         <v>595</v>
       </c>
       <c r="L132" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="42"/>
         <v>'busq_puesto' : r_val['busq_puesto'],</v>
       </c>
     </row>
@@ -40949,7 +41796,7 @@
         <v>695</v>
       </c>
       <c r="L133" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="42"/>
         <v>'m_busq' : r_val['m_busq'],</v>
       </c>
     </row>
@@ -40961,7 +41808,7 @@
         <v>325</v>
       </c>
       <c r="L134" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="42"/>
         <v>'busq_suplente' : r_val['busq_suplente'],</v>
       </c>
     </row>
@@ -40973,7 +41820,7 @@
         <v>596</v>
       </c>
       <c r="L135" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="42"/>
         <v>'supl_busq_puesto' : r_val['supl_busq_puesto'],</v>
       </c>
     </row>
@@ -40985,7 +41832,7 @@
         <v>696</v>
       </c>
       <c r="L136" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="42"/>
         <v>'m_supl_busq' : r_val['m_supl_busq'],</v>
       </c>
     </row>
@@ -40997,7 +41844,7 @@
         <v>326</v>
       </c>
       <c r="L137" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="42"/>
         <v>'descrip_gi' : r_val['descrip_gi'],</v>
       </c>
     </row>
@@ -41009,7 +41856,7 @@
         <v>327</v>
       </c>
       <c r="L138" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="42"/>
         <v>'gas_inflamable' : r_val['gas_inflamable'],</v>
       </c>
     </row>
@@ -41021,7 +41868,7 @@
         <v>328</v>
       </c>
       <c r="L139" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="42"/>
         <v>'valor_gi' : r_val['valor_gi'],</v>
       </c>
     </row>
@@ -41033,7 +41880,7 @@
         <v>329</v>
       </c>
       <c r="L140" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="42"/>
         <v>'descrp_li' : r_val['descrp_li'],</v>
       </c>
     </row>
@@ -41045,7 +41892,7 @@
         <v>330</v>
       </c>
       <c r="L141" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="42"/>
         <v>'liquido_inflamable' : r_val['liquido_inflamable'],</v>
       </c>
     </row>
@@ -41057,7 +41904,7 @@
         <v>331</v>
       </c>
       <c r="L142" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="42"/>
         <v>'valor_li' : r_val['valor_li'],</v>
       </c>
     </row>
@@ -41069,7 +41916,7 @@
         <v>332</v>
       </c>
       <c r="L143" t="str">
-        <f t="shared" ref="L143:L181" si="34">+_xlfn.CONCAT("'",J143,"' : r_val['",J143,"'],")</f>
+        <f t="shared" ref="L143:L181" si="43">+_xlfn.CONCAT("'",J143,"' : r_val['",J143,"'],")</f>
         <v>'descrip_lc' : r_val['descrip_lc'],</v>
       </c>
     </row>
@@ -41081,7 +41928,7 @@
         <v>333</v>
       </c>
       <c r="L144" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'liquido_combustible' : r_val['liquido_combustible'],</v>
       </c>
     </row>
@@ -41093,7 +41940,7 @@
         <v>334</v>
       </c>
       <c r="L145" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'valor_lc' : r_val['valor_lc'],</v>
       </c>
     </row>
@@ -41105,7 +41952,7 @@
         <v>335</v>
       </c>
       <c r="L146" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'descrip_sc' : r_val['descrip_sc'],</v>
       </c>
     </row>
@@ -41117,7 +41964,7 @@
         <v>336</v>
       </c>
       <c r="L147" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'solido_combusible' : r_val['solido_combusible'],</v>
       </c>
     </row>
@@ -41129,7 +41976,7 @@
         <v>337</v>
       </c>
       <c r="L148" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'valor_sc' : r_val['valor_sc'],</v>
       </c>
     </row>
@@ -41141,7 +41988,7 @@
         <v>338</v>
       </c>
       <c r="L149" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'tipo_riesgo' : r_val['tipo_riesgo'],</v>
       </c>
     </row>
@@ -41153,7 +42000,7 @@
         <v>657</v>
       </c>
       <c r="L150" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'nombre1' : r_val['nombre1'],</v>
       </c>
     </row>
@@ -41165,7 +42012,7 @@
         <v>658</v>
       </c>
       <c r="L151" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'puesto1' : r_val['puesto1'],</v>
       </c>
     </row>
@@ -41177,7 +42024,7 @@
         <v>659</v>
       </c>
       <c r="L152" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'m1' : r_val['m1'],</v>
       </c>
     </row>
@@ -41189,7 +42036,7 @@
         <v>660</v>
       </c>
       <c r="L153" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'nombre2' : r_val['nombre2'],</v>
       </c>
     </row>
@@ -41201,7 +42048,7 @@
         <v>661</v>
       </c>
       <c r="L154" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'puesto2' : r_val['puesto2'],</v>
       </c>
     </row>
@@ -41213,7 +42060,7 @@
         <v>662</v>
       </c>
       <c r="L155" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'m2' : r_val['m2'],</v>
       </c>
     </row>
@@ -41225,7 +42072,7 @@
         <v>663</v>
       </c>
       <c r="L156" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'nombre3' : r_val['nombre3'],</v>
       </c>
     </row>
@@ -41237,7 +42084,7 @@
         <v>664</v>
       </c>
       <c r="L157" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'puesto3' : r_val['puesto3'],</v>
       </c>
     </row>
@@ -41249,7 +42096,7 @@
         <v>665</v>
       </c>
       <c r="L158" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'m3' : r_val['m3'],</v>
       </c>
     </row>
@@ -41261,7 +42108,7 @@
         <v>666</v>
       </c>
       <c r="L159" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'nombre4' : r_val['nombre4'],</v>
       </c>
     </row>
@@ -41273,7 +42120,7 @@
         <v>667</v>
       </c>
       <c r="L160" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'puesto4' : r_val['puesto4'],</v>
       </c>
     </row>
@@ -41285,7 +42132,7 @@
         <v>668</v>
       </c>
       <c r="L161" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'m4' : r_val['m4'],</v>
       </c>
     </row>
@@ -41297,7 +42144,7 @@
         <v>669</v>
       </c>
       <c r="L162" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'nombre5' : r_val['nombre5'],</v>
       </c>
     </row>
@@ -41309,7 +42156,7 @@
         <v>670</v>
       </c>
       <c r="L163" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'puesto5' : r_val['puesto5'],</v>
       </c>
     </row>
@@ -41321,7 +42168,7 @@
         <v>671</v>
       </c>
       <c r="L164" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'m5' : r_val['m5'],</v>
       </c>
     </row>
@@ -41333,7 +42180,7 @@
         <v>672</v>
       </c>
       <c r="L165" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'nombre6' : r_val['nombre6'],</v>
       </c>
     </row>
@@ -41345,7 +42192,7 @@
         <v>673</v>
       </c>
       <c r="L166" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'puesto6' : r_val['puesto6'],</v>
       </c>
     </row>
@@ -41357,7 +42204,7 @@
         <v>674</v>
       </c>
       <c r="L167" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'m6' : r_val['m6'],</v>
       </c>
     </row>
@@ -41369,7 +42216,7 @@
         <v>675</v>
       </c>
       <c r="L168" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'nombre7' : r_val['nombre7'],</v>
       </c>
     </row>
@@ -41381,7 +42228,7 @@
         <v>676</v>
       </c>
       <c r="L169" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'puesto7' : r_val['puesto7'],</v>
       </c>
     </row>
@@ -41393,7 +42240,7 @@
         <v>677</v>
       </c>
       <c r="L170" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'m7' : r_val['m7'],</v>
       </c>
     </row>
@@ -41405,7 +42252,7 @@
         <v>678</v>
       </c>
       <c r="L171" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'nombre8' : r_val['nombre8'],</v>
       </c>
     </row>
@@ -41417,7 +42264,7 @@
         <v>679</v>
       </c>
       <c r="L172" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'puesto8' : r_val['puesto8'],</v>
       </c>
     </row>
@@ -41429,7 +42276,7 @@
         <v>680</v>
       </c>
       <c r="L173" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'m8' : r_val['m8'],</v>
       </c>
     </row>
@@ -41441,7 +42288,7 @@
         <v>681</v>
       </c>
       <c r="L174" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'nombre9' : r_val['nombre9'],</v>
       </c>
     </row>
@@ -41453,7 +42300,7 @@
         <v>682</v>
       </c>
       <c r="L175" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'puesto9' : r_val['puesto9'],</v>
       </c>
     </row>
@@ -41465,7 +42312,7 @@
         <v>683</v>
       </c>
       <c r="L176" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'m9' : r_val['m9'],</v>
       </c>
     </row>
@@ -41477,7 +42324,7 @@
         <v>684</v>
       </c>
       <c r="L177" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'nombre10' : r_val['nombre10'],</v>
       </c>
     </row>
@@ -41489,7 +42336,7 @@
         <v>685</v>
       </c>
       <c r="L178" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'puesto10' : r_val['puesto10'],</v>
       </c>
     </row>
@@ -41501,7 +42348,7 @@
         <v>686</v>
       </c>
       <c r="L179" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'m10' : r_val['m10'],</v>
       </c>
     </row>
@@ -41514,7 +42361,7 @@
         <v>{{ registro_perito }}</v>
       </c>
       <c r="L180" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'registro_perito' : r_val['registro_perito'],</v>
       </c>
     </row>
@@ -41527,7 +42374,7 @@
         <v>{{ no_registro }}</v>
       </c>
       <c r="L181" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="43"/>
         <v>'no_registro' : r_val['no_registro'],</v>
       </c>
     </row>
@@ -41536,11 +42383,11 @@
         <v>1735</v>
       </c>
       <c r="K182" t="str">
-        <f t="shared" ref="K182:K183" si="35">+_xlfn.CONCAT("{{ ",J182," }}")</f>
+        <f t="shared" ref="K182:K183" si="44">+_xlfn.CONCAT("{{ ",J182," }}")</f>
         <v>{{ dh_int }}</v>
       </c>
       <c r="L182" t="str">
-        <f t="shared" ref="L182:L183" si="36">+_xlfn.CONCAT("'",J182,"' : r_val['",J182,"'],")</f>
+        <f t="shared" ref="L182:L183" si="45">+_xlfn.CONCAT("'",J182,"' : r_val['",J182,"'],")</f>
         <v>'dh_int' : r_val['dh_int'],</v>
       </c>
     </row>
@@ -41549,11 +42396,11 @@
         <v>1736</v>
       </c>
       <c r="K183" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="44"/>
         <v>{{ dh_ext }}</v>
       </c>
       <c r="L183" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="45"/>
         <v>'dh_ext' : r_val['dh_ext'],</v>
       </c>
     </row>
@@ -41562,11 +42409,11 @@
         <v>1737</v>
       </c>
       <c r="K184" t="str">
-        <f t="shared" ref="K184" si="37">+_xlfn.CONCAT("{{ ",J184," }}")</f>
+        <f t="shared" ref="K184" si="46">+_xlfn.CONCAT("{{ ",J184," }}")</f>
         <v>{{ detectores_ext }}</v>
       </c>
       <c r="L184" t="str">
-        <f t="shared" ref="L184" si="38">+_xlfn.CONCAT("'",J184,"' : r_val['",J184,"'],")</f>
+        <f t="shared" ref="L184" si="47">+_xlfn.CONCAT("'",J184,"' : r_val['",J184,"'],")</f>
         <v>'detectores_ext' : r_val['detectores_ext'],</v>
       </c>
     </row>
@@ -41575,11 +42422,11 @@
         <v>1738</v>
       </c>
       <c r="K185" t="str">
-        <f t="shared" ref="K185" si="39">+_xlfn.CONCAT("{{ ",J185," }}")</f>
+        <f t="shared" ref="K185" si="48">+_xlfn.CONCAT("{{ ",J185," }}")</f>
         <v>{{ coord_sup_puesto }}</v>
       </c>
       <c r="L185" t="str">
-        <f t="shared" ref="L185" si="40">+_xlfn.CONCAT("'",J185,"' : r_val['",J185,"'],")</f>
+        <f t="shared" ref="L185" si="49">+_xlfn.CONCAT("'",J185,"' : r_val['",J185,"'],")</f>
         <v>'coord_sup_puesto' : r_val['coord_sup_puesto'],</v>
       </c>
     </row>
@@ -41588,11 +42435,11 @@
         <v>1744</v>
       </c>
       <c r="K186" t="str">
-        <f t="shared" ref="K186:K189" si="41">+_xlfn.CONCAT("{{ ",J186," }}")</f>
+        <f t="shared" ref="K186:K189" si="50">+_xlfn.CONCAT("{{ ",J186," }}")</f>
         <v>{{ riesgo1 }}</v>
       </c>
       <c r="L186" t="str">
-        <f t="shared" ref="L186:L189" si="42">+_xlfn.CONCAT("'",J186,"' : r_val['",J186,"'],")</f>
+        <f t="shared" ref="L186:L189" si="51">+_xlfn.CONCAT("'",J186,"' : r_val['",J186,"'],")</f>
         <v>'riesgo1' : r_val['riesgo1'],</v>
       </c>
     </row>
@@ -41601,11 +42448,11 @@
         <v>1745</v>
       </c>
       <c r="K187" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="50"/>
         <v>{{ riesgo2 }}</v>
       </c>
       <c r="L187" t="str">
-        <f t="shared" si="42"/>
+        <f t="shared" si="51"/>
         <v>'riesgo2' : r_val['riesgo2'],</v>
       </c>
     </row>
@@ -41614,11 +42461,11 @@
         <v>1746</v>
       </c>
       <c r="K188" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="50"/>
         <v>{{ riesgo3 }}</v>
       </c>
       <c r="L188" t="str">
-        <f t="shared" si="42"/>
+        <f t="shared" si="51"/>
         <v>'riesgo3' : r_val['riesgo3'],</v>
       </c>
     </row>
@@ -41627,11 +42474,11 @@
         <v>1747</v>
       </c>
       <c r="K189" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="50"/>
         <v>{{ riesgo4 }}</v>
       </c>
       <c r="L189" t="str">
-        <f t="shared" si="42"/>
+        <f t="shared" si="51"/>
         <v>'riesgo4' : r_val['riesgo4'],</v>
       </c>
     </row>
@@ -41640,11 +42487,11 @@
         <v>1751</v>
       </c>
       <c r="K190" t="str">
-        <f t="shared" ref="K190" si="43">+_xlfn.CONCAT("{{ ",J190," }}")</f>
+        <f t="shared" ref="K190" si="52">+_xlfn.CONCAT("{{ ",J190," }}")</f>
         <v>{{ valor_gri }}</v>
       </c>
       <c r="L190" t="str">
-        <f t="shared" ref="L190" si="44">+_xlfn.CONCAT("'",J190,"' : r_val['",J190,"'],")</f>
+        <f t="shared" ref="L190" si="53">+_xlfn.CONCAT("'",J190,"' : r_val['",J190,"'],")</f>
         <v>'valor_gri' : r_val['valor_gri'],</v>
       </c>
     </row>
@@ -41653,11 +42500,11 @@
         <v>1752</v>
       </c>
       <c r="K191" t="str">
-        <f t="shared" ref="K191:K194" si="45">+_xlfn.CONCAT("{{ ",J191," }}")</f>
+        <f t="shared" ref="K191:K194" si="54">+_xlfn.CONCAT("{{ ",J191," }}")</f>
         <v>{{ medidas_ries1 }}</v>
       </c>
       <c r="L191" t="str">
-        <f t="shared" ref="L191:L194" si="46">+_xlfn.CONCAT("'",J191,"' : r_val['",J191,"'],")</f>
+        <f t="shared" ref="L191:L194" si="55">+_xlfn.CONCAT("'",J191,"' : r_val['",J191,"'],")</f>
         <v>'medidas_ries1' : r_val['medidas_ries1'],</v>
       </c>
     </row>
@@ -41666,11 +42513,11 @@
         <v>1753</v>
       </c>
       <c r="K192" t="str">
-        <f t="shared" si="45"/>
+        <f t="shared" si="54"/>
         <v>{{ medidas_ries2 }}</v>
       </c>
       <c r="L192" t="str">
-        <f t="shared" si="46"/>
+        <f t="shared" si="55"/>
         <v>'medidas_ries2' : r_val['medidas_ries2'],</v>
       </c>
     </row>
@@ -41679,11 +42526,11 @@
         <v>1754</v>
       </c>
       <c r="K193" t="str">
-        <f t="shared" si="45"/>
+        <f t="shared" si="54"/>
         <v>{{ medidas_ries3 }}</v>
       </c>
       <c r="L193" t="str">
-        <f t="shared" si="46"/>
+        <f t="shared" si="55"/>
         <v>'medidas_ries3' : r_val['medidas_ries3'],</v>
       </c>
     </row>
@@ -41692,11 +42539,11 @@
         <v>1755</v>
       </c>
       <c r="K194" t="str">
-        <f t="shared" si="45"/>
+        <f t="shared" si="54"/>
         <v>{{ medidas_ries4 }}</v>
       </c>
       <c r="L194" t="str">
-        <f t="shared" si="46"/>
+        <f t="shared" si="55"/>
         <v>'medidas_ries4' : r_val['medidas_ries4'],</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Se agregan fotos de evalucion simulacro y acta UIPC
</commit_message>
<xml_diff>
--- a/Inputs/BD.xlsx
+++ b/Inputs/BD.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/078e1a455e5c02ce/Documentos/GitHub/Proyecto_PIPC/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6242" documentId="13_ncr:1_{7D3A426E-EC5E-453A-8CC7-F83B71F24F18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A6FA3155-E44A-4DE4-96B9-E887838E4F64}"/>
+  <xr:revisionPtr revIDLastSave="6316" documentId="13_ncr:1_{7D3A426E-EC5E-453A-8CC7-F83B71F24F18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2B58571F-D84D-438F-B359-A07494472925}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3F095A75-F066-4695-8672-8D4315F1EF23}"/>
   </bookViews>
@@ -563,7 +563,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7062" uniqueCount="2149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7178" uniqueCount="2175">
   <si>
     <t>dia</t>
   </si>
@@ -7010,6 +7010,84 @@
   </si>
   <si>
     <t>layout12</t>
+  </si>
+  <si>
+    <t>ev_sim (3).png</t>
+  </si>
+  <si>
+    <t>ev_sim (4).png</t>
+  </si>
+  <si>
+    <t>ev_sim (5).png</t>
+  </si>
+  <si>
+    <t>ev_sim (6).png</t>
+  </si>
+  <si>
+    <t>acta3</t>
+  </si>
+  <si>
+    <t>acta4</t>
+  </si>
+  <si>
+    <t>ev_sim3</t>
+  </si>
+  <si>
+    <t>ev_sim4</t>
+  </si>
+  <si>
+    <t>ev_sim5</t>
+  </si>
+  <si>
+    <t>ev_sim6</t>
+  </si>
+  <si>
+    <t>ev_sim7</t>
+  </si>
+  <si>
+    <t>ev_sim8</t>
+  </si>
+  <si>
+    <t>layout (1).png</t>
+  </si>
+  <si>
+    <t>layout (2).png</t>
+  </si>
+  <si>
+    <t>layout (3).png</t>
+  </si>
+  <si>
+    <t>layout (4).png</t>
+  </si>
+  <si>
+    <t>layout (5).png</t>
+  </si>
+  <si>
+    <t>layout (6).png</t>
+  </si>
+  <si>
+    <t>layout (7).png</t>
+  </si>
+  <si>
+    <t>layout (8).png</t>
+  </si>
+  <si>
+    <t>layout (9).png</t>
+  </si>
+  <si>
+    <t>layout (10).png</t>
+  </si>
+  <si>
+    <t>layout (11).png</t>
+  </si>
+  <si>
+    <t>layout (12).png</t>
+  </si>
+  <si>
+    <t>ev_sim (7).png</t>
+  </si>
+  <si>
+    <t>ev_sim (8).png</t>
   </si>
 </sst>
 </file>
@@ -7632,7 +7710,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp1.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Spin" dx="26" fmlaLink="$A$1" max="30000" min="1" page="10" val="57"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Spin" dx="26" fmlaLink="$A$1" max="30000" min="1" page="10" val="53"/>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8027,7 +8105,7 @@
   <sheetData>
     <row r="1" spans="1:322" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="DS1" t="s">
         <v>1969</v>
@@ -38717,13 +38795,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76893F01-97EA-43A4-9AE2-ED099B9448DD}">
-  <dimension ref="A1:KD2"/>
+  <dimension ref="A1:KX2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:290" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:310" x14ac:dyDescent="0.3">
       <c r="A1">
         <f>+BD!A1</f>
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B1" t="s">
         <v>134</v>
@@ -39592,8 +39670,68 @@
       <c r="KD1" t="s">
         <v>2135</v>
       </c>
+      <c r="KE1" t="s">
+        <v>2137</v>
+      </c>
+      <c r="KF1" t="s">
+        <v>2138</v>
+      </c>
+      <c r="KG1" t="s">
+        <v>2139</v>
+      </c>
+      <c r="KH1" t="s">
+        <v>2140</v>
+      </c>
+      <c r="KI1" t="s">
+        <v>2141</v>
+      </c>
+      <c r="KJ1" t="s">
+        <v>2142</v>
+      </c>
+      <c r="KK1" t="s">
+        <v>2143</v>
+      </c>
+      <c r="KL1" t="s">
+        <v>2144</v>
+      </c>
+      <c r="KM1" t="s">
+        <v>2145</v>
+      </c>
+      <c r="KN1" t="s">
+        <v>2146</v>
+      </c>
+      <c r="KO1" t="s">
+        <v>2147</v>
+      </c>
+      <c r="KP1" t="s">
+        <v>2148</v>
+      </c>
+      <c r="KQ1" t="s">
+        <v>2155</v>
+      </c>
+      <c r="KR1" t="s">
+        <v>2156</v>
+      </c>
+      <c r="KS1" t="s">
+        <v>2157</v>
+      </c>
+      <c r="KT1" t="s">
+        <v>2158</v>
+      </c>
+      <c r="KU1" t="s">
+        <v>2159</v>
+      </c>
+      <c r="KV1" t="s">
+        <v>2160</v>
+      </c>
+      <c r="KW1" t="s">
+        <v>2153</v>
+      </c>
+      <c r="KX1" t="s">
+        <v>2154</v>
+      </c>
     </row>
-    <row r="2" spans="1:290" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:310" x14ac:dyDescent="0.3">
       <c r="B2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,2, FALSE)</f>
         <v>GENERAL</v>
@@ -39604,15 +39742,15 @@
       </c>
       <c r="D2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,4, FALSE)</f>
-        <v>COMPLEJO MIXCOATL</v>
+        <v>COMPLEJO AZTLAN</v>
       </c>
       <c r="E2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,5, FALSE)</f>
-        <v>UVP810305C29</v>
+        <v>UVP810305C25</v>
       </c>
       <c r="F2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,6, FALSE)</f>
-        <v>COMPLEJO MIXCOATL</v>
+        <v>COMPLEJO AZTLAN</v>
       </c>
       <c r="G2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,7, FALSE)</f>
@@ -39624,11 +39762,11 @@
       </c>
       <c r="I2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,9, FALSE)</f>
-        <v>PRIVADA JACARANDAS</v>
+        <v>5 SUR</v>
       </c>
       <c r="J2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,10, FALSE)</f>
-        <v>327</v>
+        <v>5906</v>
       </c>
       <c r="K2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,11, FALSE)</f>
@@ -39660,15 +39798,15 @@
       </c>
       <c r="R2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,18, FALSE)</f>
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="S2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,19, FALSE)</f>
-        <v>7 DE SEPTIEMBRE DE 2021</v>
+        <v>6 DE DICIEMBRE DE 2010</v>
       </c>
       <c r="T2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,20, FALSE)</f>
-        <v>NOE MORA RAMIREZ</v>
+        <v>JORGE MANUEL ISLAS GOWER</v>
       </c>
       <c r="U2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,21, FALSE)</f>
@@ -39676,31 +39814,31 @@
       </c>
       <c r="V2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,22, FALSE)</f>
-        <v>496</v>
+        <v>2485</v>
       </c>
       <c r="W2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,23, FALSE)</f>
-        <v>298.74</v>
+        <v>4639.5200000000004</v>
       </c>
       <c r="X2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,24, FALSE)</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Y2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,25, FALSE)</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Z2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,26, FALSE)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AA2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,27, FALSE)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AB2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,28, FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,29, FALSE)</f>
@@ -39708,7 +39846,7 @@
       </c>
       <c r="AD2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,30, FALSE)</f>
-        <v>0 CAJONES</v>
+        <v>6 CAJONES</v>
       </c>
       <c r="AE2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,31, FALSE)</f>
@@ -39716,11 +39854,11 @@
       </c>
       <c r="AF2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,32, FALSE)</f>
-        <v>ISABEL MARÍA CORTES CUELLAR</v>
+        <v>MODESTO ALFONSO HERNÁNDEZ ORTIZ</v>
       </c>
       <c r="AG2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,33, FALSE)</f>
-        <v>6</v>
+        <v>70</v>
       </c>
       <c r="AH2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,34, FALSE)</f>
@@ -39728,11 +39866,11 @@
       </c>
       <c r="AI2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,35, FALSE)</f>
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="AJ2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,36, FALSE)</f>
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="AK2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,37, FALSE)</f>
@@ -39748,11 +39886,11 @@
       </c>
       <c r="AN2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,40, FALSE)</f>
-        <v>55</v>
+        <v>500</v>
       </c>
       <c r="AO2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,41, FALSE)</f>
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="AP2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,42, FALSE)</f>
@@ -39764,19 +39902,19 @@
       </c>
       <c r="AR2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,44, FALSE)</f>
-        <v>23</v>
+        <v>92</v>
       </c>
       <c r="AS2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,45, FALSE)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AT2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,46, FALSE)</f>
-        <v>PREFECTURA</v>
+        <v>RECEPCION, BIBLIOTECA, CAI, CAPS</v>
       </c>
       <c r="AU2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,47, FALSE)</f>
-        <v>9</v>
+        <v>39</v>
       </c>
       <c r="AV2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,48, FALSE)</f>
@@ -39784,11 +39922,11 @@
       </c>
       <c r="AW2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,49, FALSE)</f>
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="AX2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,50, FALSE)</f>
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="AY2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,51, FALSE)</f>
@@ -39824,7 +39962,7 @@
       </c>
       <c r="BG2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,59, FALSE)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BH2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,60, FALSE)</f>
@@ -39832,7 +39970,7 @@
       </c>
       <c r="BI2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,61, FALSE)</f>
-        <v>DIRECCION</v>
+        <v>COORDINACION, VIGILANCIA, CONTROL EXTERNO</v>
       </c>
       <c r="BJ2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,62, FALSE)</f>
@@ -39844,23 +39982,23 @@
       </c>
       <c r="BL2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,64, FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="BM2">
+        <v>5</v>
+      </c>
+      <c r="BM2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,65, FALSE)</f>
-        <v>0</v>
+        <v>OFICINAS</v>
       </c>
       <c r="BN2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,66, FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="BO2">
+        <v>1</v>
+      </c>
+      <c r="BO2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,67, FALSE)</f>
-        <v>0</v>
+        <v>GABINETE</v>
       </c>
       <c r="BP2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,68, FALSE)</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="BQ2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,69, FALSE)</f>
@@ -39868,7 +40006,7 @@
       </c>
       <c r="BR2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,70, FALSE)</f>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BS2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,71, FALSE)</f>
@@ -39876,11 +40014,11 @@
       </c>
       <c r="BT2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,72, FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="BU2">
+        <v>2</v>
+      </c>
+      <c r="BU2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,73, FALSE)</f>
-        <v>0</v>
+        <v>GABINETE</v>
       </c>
       <c r="BV2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,74, FALSE)</f>
@@ -39888,23 +40026,23 @@
       </c>
       <c r="BW2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,75, FALSE)</f>
-        <v>GABINETE</v>
+        <v>COORDINACION</v>
       </c>
       <c r="BX2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,76, FALSE)</f>
-        <v>3</v>
-      </c>
-      <c r="BY2" t="str">
+        <v>0</v>
+      </c>
+      <c r="BY2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,77, FALSE)</f>
-        <v>GABINETE</v>
+        <v>0</v>
       </c>
       <c r="BZ2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,78, FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="CA2">
+        <v>1</v>
+      </c>
+      <c r="CA2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,79, FALSE)</f>
-        <v>0</v>
+        <v>GABINETE</v>
       </c>
       <c r="CB2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,80, FALSE)</f>
@@ -39916,15 +40054,15 @@
       </c>
       <c r="CD2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,82, FALSE)</f>
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="CE2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,83, FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CF2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,84, FALSE)</f>
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="CG2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,85, FALSE)</f>
@@ -39932,27 +40070,27 @@
       </c>
       <c r="CH2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,86, FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CI2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,87, FALSE)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="CJ2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,88, FALSE)</f>
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="CK2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,89, FALSE)</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="CL2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,90, FALSE)</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="CM2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,91, FALSE)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="CN2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,92, FALSE)</f>
@@ -39976,11 +40114,11 @@
       </c>
       <c r="CS2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,97, FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="CT2">
+        <v>9</v>
+      </c>
+      <c r="CT2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,98, FALSE)</f>
-        <v>0</v>
+        <v>AREA COMÚN</v>
       </c>
       <c r="CU2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,99, FALSE)</f>
@@ -40016,7 +40154,7 @@
       </c>
       <c r="DC2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,107, FALSE)</f>
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="DD2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,108, FALSE)</f>
@@ -40024,11 +40162,11 @@
       </c>
       <c r="DE2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,109, FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="DF2">
+        <v>11</v>
+      </c>
+      <c r="DF2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,110, FALSE)</f>
-        <v>0</v>
+        <v>AREA COMÚN</v>
       </c>
       <c r="DG2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,111, FALSE)</f>
@@ -40108,15 +40246,15 @@
       </c>
       <c r="DZ2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,130, FALSE)</f>
-        <v>19.020492484141947, -98.21580700217788</v>
+        <v>19.017749517200585, -98.2183180754988</v>
       </c>
       <c r="EA2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,131, FALSE)</f>
-        <v>CASA HABITACIÓN</v>
+        <v>TAQUERIA</v>
       </c>
       <c r="EB2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,132, FALSE)</f>
-        <v>CASAS HABITACION</v>
+        <v>UVP TEOCALLI</v>
       </c>
       <c r="EC2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,133, FALSE)</f>
@@ -40124,7 +40262,7 @@
       </c>
       <c r="ED2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,134, FALSE)</f>
-        <v>CASA HABITACION</v>
+        <v>PARQUE EL ELEFANTE</v>
       </c>
       <c r="EE2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,135, FALSE)</f>
@@ -40252,15 +40390,15 @@
       </c>
       <c r="FJ2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,166, FALSE)</f>
-        <v>GAS LP</v>
+        <v>GAS LP Y GAS NATURAL</v>
       </c>
       <c r="FK2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,167, FALSE)</f>
-        <v>20</v>
+        <v>20480</v>
       </c>
       <c r="FL2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,168, FALSE)</f>
-        <v>6.6666666666666671E-3</v>
+        <v>6.8266666666666671</v>
       </c>
       <c r="FM2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,169, FALSE)</f>
@@ -40292,19 +40430,19 @@
       </c>
       <c r="FT2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,176, FALSE)</f>
-        <v>360</v>
+        <v>4200</v>
       </c>
       <c r="FU2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,177, FALSE)</f>
-        <v>2.4E-2</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="FV2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,178, FALSE)</f>
-        <v>3.0666666666666668E-2</v>
+        <v>7.1066666666666674</v>
       </c>
       <c r="FW2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,179, FALSE)</f>
-        <v>ORDINARIO</v>
+        <v>ALTO</v>
       </c>
       <c r="FX2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,180, FALSE)</f>
@@ -40644,6 +40782,68 @@
       </c>
       <c r="KD2" t="s">
         <v>2136</v>
+      </c>
+      <c r="KE2" t="s">
+        <v>2161</v>
+      </c>
+      <c r="KF2" t="s">
+        <v>2162</v>
+      </c>
+      <c r="KG2" t="s">
+        <v>2163</v>
+      </c>
+      <c r="KH2" t="s">
+        <v>2164</v>
+      </c>
+      <c r="KI2" t="s">
+        <v>2165</v>
+      </c>
+      <c r="KJ2" t="s">
+        <v>2166</v>
+      </c>
+      <c r="KK2" t="s">
+        <v>2167</v>
+      </c>
+      <c r="KL2" t="s">
+        <v>2168</v>
+      </c>
+      <c r="KM2" t="s">
+        <v>2169</v>
+      </c>
+      <c r="KN2" t="s">
+        <v>2170</v>
+      </c>
+      <c r="KO2" t="s">
+        <v>2171</v>
+      </c>
+      <c r="KP2" t="s">
+        <v>2172</v>
+      </c>
+      <c r="KQ2" t="s">
+        <v>2149</v>
+      </c>
+      <c r="KR2" t="s">
+        <v>2150</v>
+      </c>
+      <c r="KS2" t="s">
+        <v>2151</v>
+      </c>
+      <c r="KT2" t="s">
+        <v>2152</v>
+      </c>
+      <c r="KU2" t="s">
+        <v>2173</v>
+      </c>
+      <c r="KV2" t="s">
+        <v>2174</v>
+      </c>
+      <c r="KW2" t="str">
+        <f>+_xlfn.CONCAT(KW1,".png")</f>
+        <v>acta3.png</v>
+      </c>
+      <c r="KX2" t="str">
+        <f>+_xlfn.CONCAT(KX1,".png")</f>
+        <v>acta4.png</v>
       </c>
     </row>
   </sheetData>
@@ -47685,7 +47885,7 @@
         <v>1759</v>
       </c>
       <c r="F94" t="str">
-        <f t="shared" ref="F94:F107" si="33">+_xlfn.CONCAT(E94,".png")</f>
+        <f t="shared" ref="F94:F105" si="33">+_xlfn.CONCAT(E94,".png")</f>
         <v>corresp2.png</v>
       </c>
       <c r="G94" t="str">
@@ -48557,12 +48757,14 @@
       </c>
     </row>
     <row r="106" spans="2:23" x14ac:dyDescent="0.3">
+      <c r="B106" t="s">
+        <v>1898</v>
+      </c>
       <c r="E106" t="s">
         <v>2137</v>
       </c>
-      <c r="F106" t="str">
-        <f t="shared" si="33"/>
-        <v>layout1.png</v>
+      <c r="F106" t="s">
+        <v>2161</v>
       </c>
       <c r="G106" t="str">
         <f t="shared" si="34"/>
@@ -48627,12 +48829,14 @@
       </c>
     </row>
     <row r="107" spans="2:23" x14ac:dyDescent="0.3">
+      <c r="B107" t="s">
+        <v>1898</v>
+      </c>
       <c r="E107" t="s">
         <v>2138</v>
       </c>
-      <c r="F107" t="str">
-        <f t="shared" si="33"/>
-        <v>layout2.png</v>
+      <c r="F107" t="s">
+        <v>2162</v>
       </c>
       <c r="G107" t="str">
         <f t="shared" si="34"/>
@@ -48697,15 +48901,17 @@
       </c>
     </row>
     <row r="108" spans="2:23" x14ac:dyDescent="0.3">
+      <c r="B108" t="s">
+        <v>1898</v>
+      </c>
       <c r="E108" t="s">
         <v>2139</v>
       </c>
-      <c r="F108" t="str">
-        <f t="shared" ref="F108:F117" si="57">+_xlfn.CONCAT(E108,".png")</f>
-        <v>layout3.png</v>
+      <c r="F108" t="s">
+        <v>2163</v>
       </c>
       <c r="G108" t="str">
-        <f t="shared" ref="G108:G117" si="58">+_xlfn.CONCAT("{{ ",E108," }}")</f>
+        <f t="shared" ref="G108:G118" si="57">+_xlfn.CONCAT("{{ ",E108," }}")</f>
         <v>{{ layout3 }}</v>
       </c>
       <c r="H108">
@@ -48767,15 +48973,17 @@
       </c>
     </row>
     <row r="109" spans="2:23" x14ac:dyDescent="0.3">
+      <c r="B109" t="s">
+        <v>1898</v>
+      </c>
       <c r="E109" t="s">
         <v>2140</v>
       </c>
-      <c r="F109" t="str">
+      <c r="F109" t="s">
+        <v>2164</v>
+      </c>
+      <c r="G109" t="str">
         <f t="shared" si="57"/>
-        <v>layout4.png</v>
-      </c>
-      <c r="G109" t="str">
-        <f t="shared" si="58"/>
         <v>{{ layout4 }}</v>
       </c>
       <c r="H109">
@@ -48837,15 +49045,17 @@
       </c>
     </row>
     <row r="110" spans="2:23" x14ac:dyDescent="0.3">
+      <c r="B110" t="s">
+        <v>1898</v>
+      </c>
       <c r="E110" t="s">
         <v>2141</v>
       </c>
-      <c r="F110" t="str">
+      <c r="F110" t="s">
+        <v>2165</v>
+      </c>
+      <c r="G110" t="str">
         <f t="shared" si="57"/>
-        <v>layout5.png</v>
-      </c>
-      <c r="G110" t="str">
-        <f t="shared" si="58"/>
         <v>{{ layout5 }}</v>
       </c>
       <c r="H110">
@@ -48907,15 +49117,17 @@
       </c>
     </row>
     <row r="111" spans="2:23" x14ac:dyDescent="0.3">
+      <c r="B111" t="s">
+        <v>1898</v>
+      </c>
       <c r="E111" t="s">
         <v>2142</v>
       </c>
-      <c r="F111" t="str">
+      <c r="F111" t="s">
+        <v>2166</v>
+      </c>
+      <c r="G111" t="str">
         <f t="shared" si="57"/>
-        <v>layout6.png</v>
-      </c>
-      <c r="G111" t="str">
-        <f t="shared" si="58"/>
         <v>{{ layout6 }}</v>
       </c>
       <c r="H111">
@@ -48931,7 +49143,7 @@
         <v>317</v>
       </c>
       <c r="L111" t="str">
-        <f t="shared" ref="L111:L142" si="59">+_xlfn.CONCAT("'",J111,"' : r_val['",J111,"'],")</f>
+        <f t="shared" ref="L111:L142" si="58">+_xlfn.CONCAT("'",J111,"' : r_val['",J111,"'],")</f>
         <v>'coord_suplente' : r_val['coord_suplente'],</v>
       </c>
       <c r="M111" t="str">
@@ -48977,15 +49189,17 @@
       </c>
     </row>
     <row r="112" spans="2:23" x14ac:dyDescent="0.3">
+      <c r="B112" t="s">
+        <v>1898</v>
+      </c>
       <c r="E112" t="s">
         <v>2143</v>
       </c>
-      <c r="F112" t="str">
+      <c r="F112" t="s">
+        <v>2167</v>
+      </c>
+      <c r="G112" t="str">
         <f t="shared" si="57"/>
-        <v>layout7.png</v>
-      </c>
-      <c r="G112" t="str">
-        <f t="shared" si="58"/>
         <v>{{ layout7 }}</v>
       </c>
       <c r="H112">
@@ -49001,7 +49215,7 @@
         <v>687</v>
       </c>
       <c r="L112" t="str">
-        <f t="shared" si="59"/>
+        <f t="shared" si="58"/>
         <v>'m_jef_caj' : r_val['m_jef_caj'],</v>
       </c>
       <c r="M112" t="str">
@@ -49046,16 +49260,18 @@
         <v>layout7 = ''</v>
       </c>
     </row>
-    <row r="113" spans="5:23" x14ac:dyDescent="0.3">
+    <row r="113" spans="2:23" x14ac:dyDescent="0.3">
+      <c r="B113" t="s">
+        <v>1898</v>
+      </c>
       <c r="E113" t="s">
         <v>2144</v>
       </c>
-      <c r="F113" t="str">
+      <c r="F113" t="s">
+        <v>2168</v>
+      </c>
+      <c r="G113" t="str">
         <f t="shared" si="57"/>
-        <v>layout8.png</v>
-      </c>
-      <c r="G113" t="str">
-        <f t="shared" si="58"/>
         <v>{{ layout8 }}</v>
       </c>
       <c r="H113">
@@ -49071,7 +49287,7 @@
         <v>318</v>
       </c>
       <c r="L113" t="str">
-        <f t="shared" si="59"/>
+        <f t="shared" si="58"/>
         <v>'evacuacion' : r_val['evacuacion'],</v>
       </c>
       <c r="M113" t="str">
@@ -49116,16 +49332,18 @@
         <v>layout8 = ''</v>
       </c>
     </row>
-    <row r="114" spans="5:23" x14ac:dyDescent="0.3">
+    <row r="114" spans="2:23" x14ac:dyDescent="0.3">
+      <c r="B114" t="s">
+        <v>1898</v>
+      </c>
       <c r="E114" t="s">
         <v>2145</v>
       </c>
-      <c r="F114" t="str">
+      <c r="F114" t="s">
+        <v>2169</v>
+      </c>
+      <c r="G114" t="str">
         <f t="shared" si="57"/>
-        <v>layout9.png</v>
-      </c>
-      <c r="G114" t="str">
-        <f t="shared" si="58"/>
         <v>{{ layout9 }}</v>
       </c>
       <c r="H114">
@@ -49141,7 +49359,7 @@
         <v>588</v>
       </c>
       <c r="L114" t="str">
-        <f t="shared" si="59"/>
+        <f t="shared" si="58"/>
         <v>'evac_puesto' : r_val['evac_puesto'],</v>
       </c>
       <c r="M114" t="str">
@@ -49186,16 +49404,18 @@
         <v>layout9 = ''</v>
       </c>
     </row>
-    <row r="115" spans="5:23" x14ac:dyDescent="0.3">
+    <row r="115" spans="2:23" x14ac:dyDescent="0.3">
+      <c r="B115" t="s">
+        <v>1898</v>
+      </c>
       <c r="E115" t="s">
         <v>2146</v>
       </c>
-      <c r="F115" t="str">
+      <c r="F115" t="s">
+        <v>2170</v>
+      </c>
+      <c r="G115" t="str">
         <f t="shared" si="57"/>
-        <v>layout10.png</v>
-      </c>
-      <c r="G115" t="str">
-        <f t="shared" si="58"/>
         <v>{{ layout10 }}</v>
       </c>
       <c r="H115">
@@ -49211,7 +49431,7 @@
         <v>688</v>
       </c>
       <c r="L115" t="str">
-        <f t="shared" si="59"/>
+        <f t="shared" si="58"/>
         <v>'m_evac' : r_val['m_evac'],</v>
       </c>
       <c r="M115" t="str">
@@ -49256,16 +49476,18 @@
         <v>layout10 = ''</v>
       </c>
     </row>
-    <row r="116" spans="5:23" x14ac:dyDescent="0.3">
+    <row r="116" spans="2:23" x14ac:dyDescent="0.3">
+      <c r="B116" t="s">
+        <v>1898</v>
+      </c>
       <c r="E116" t="s">
         <v>2147</v>
       </c>
-      <c r="F116" t="str">
+      <c r="F116" t="s">
+        <v>2171</v>
+      </c>
+      <c r="G116" t="str">
         <f t="shared" si="57"/>
-        <v>layout11.png</v>
-      </c>
-      <c r="G116" t="str">
-        <f t="shared" si="58"/>
         <v>{{ layout11 }}</v>
       </c>
       <c r="H116">
@@ -49281,7 +49503,7 @@
         <v>319</v>
       </c>
       <c r="L116" t="str">
-        <f t="shared" si="59"/>
+        <f t="shared" si="58"/>
         <v>'evac_suplente' : r_val['evac_suplente'],</v>
       </c>
       <c r="M116" t="str">
@@ -49326,16 +49548,18 @@
         <v>layout11 = ''</v>
       </c>
     </row>
-    <row r="117" spans="5:23" x14ac:dyDescent="0.3">
+    <row r="117" spans="2:23" x14ac:dyDescent="0.3">
+      <c r="B117" t="s">
+        <v>1898</v>
+      </c>
       <c r="E117" t="s">
         <v>2148</v>
       </c>
-      <c r="F117" t="str">
+      <c r="F117" t="s">
+        <v>2172</v>
+      </c>
+      <c r="G117" t="str">
         <f t="shared" si="57"/>
-        <v>layout12.png</v>
-      </c>
-      <c r="G117" t="str">
-        <f t="shared" si="58"/>
         <v>{{ layout12 }}</v>
       </c>
       <c r="H117">
@@ -49351,7 +49575,7 @@
         <v>589</v>
       </c>
       <c r="L117" t="str">
-        <f t="shared" si="59"/>
+        <f t="shared" si="58"/>
         <v>'supl_evac_pue' : r_val['supl_evac_pue'],</v>
       </c>
       <c r="M117" t="str">
@@ -49396,7 +49620,26 @@
         <v>layout12 = ''</v>
       </c>
     </row>
-    <row r="118" spans="5:23" x14ac:dyDescent="0.3">
+    <row r="118" spans="2:23" x14ac:dyDescent="0.3">
+      <c r="B118" t="s">
+        <v>1898</v>
+      </c>
+      <c r="E118" t="s">
+        <v>2155</v>
+      </c>
+      <c r="F118" t="s">
+        <v>2149</v>
+      </c>
+      <c r="G118" t="str">
+        <f t="shared" si="57"/>
+        <v>{{ ev_sim3 }}</v>
+      </c>
+      <c r="H118">
+        <v>155</v>
+      </c>
+      <c r="I118" t="s">
+        <v>1755</v>
+      </c>
       <c r="J118" t="s">
         <v>649</v>
       </c>
@@ -49404,11 +49647,71 @@
         <v>689</v>
       </c>
       <c r="L118" t="str">
-        <f t="shared" si="59"/>
+        <f t="shared" si="58"/>
         <v>'m_supl_evac' : r_val['m_supl_evac'],</v>
       </c>
+      <c r="M118" t="str">
+        <f t="shared" ref="M118:M123" si="59">+_xlfn.CONCAT("'",E118,"': ",E118,",")</f>
+        <v>'ev_sim3': ev_sim3,</v>
+      </c>
+      <c r="N118" t="s">
+        <v>557</v>
+      </c>
+      <c r="O118" t="str">
+        <f t="shared" ref="O118:O123" si="60">+_xlfn.CONCAT("img_path_",E118," = os.path.join(IMAGES_PATH, r_val[""",E118,"""])")</f>
+        <v>img_path_ev_sim3 = os.path.join(IMAGES_PATH, r_val["ev_sim3"])</v>
+      </c>
+      <c r="P118" t="str">
+        <f t="shared" ref="P118:P123" si="61">+_xlfn.CONCAT("if os.path.exists(img_path_",E118,"):")</f>
+        <v>if os.path.exists(img_path_ev_sim3):</v>
+      </c>
+      <c r="Q118" t="str">
+        <f t="shared" ref="Q118:Q123" si="62">+_xlfn.CONCAT(E118," = InlineImage(docx_tpl, img_path_",E118,", ",I118,"=Mm(",H118,"))")</f>
+        <v>ev_sim3 = InlineImage(docx_tpl, img_path_ev_sim3, width=Mm(155))</v>
+      </c>
+      <c r="R118" t="s">
+        <v>559</v>
+      </c>
+      <c r="S118" t="str">
+        <f t="shared" ref="S118:S123" si="63">+_xlfn.CONCAT("print(f'Advertencia: No se encontró la imagen {r_val[""",E118,"""]}')")</f>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["ev_sim3"]}')</v>
+      </c>
+      <c r="T118" t="str">
+        <f t="shared" ref="T118:T123" si="64">+_xlfn.CONCAT(E118," = ''")</f>
+        <v>ev_sim3 = ''</v>
+      </c>
+      <c r="U118" t="s">
+        <v>558</v>
+      </c>
+      <c r="V118" t="str">
+        <f t="shared" ref="V118:V123" si="65">+_xlfn.CONCAT("print(f'Advertencia: No se pudo cargar la imagen {r_val[""",E118,"""]}: {e}')")</f>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["ev_sim3"]}: {e}')</v>
+      </c>
+      <c r="W118" t="str">
+        <f t="shared" ref="W118:W123" si="66">+_xlfn.CONCAT(E118," = ''")</f>
+        <v>ev_sim3 = ''</v>
+      </c>
     </row>
-    <row r="119" spans="5:23" x14ac:dyDescent="0.3">
+    <row r="119" spans="2:23" x14ac:dyDescent="0.3">
+      <c r="B119" t="s">
+        <v>1898</v>
+      </c>
+      <c r="E119" t="s">
+        <v>2156</v>
+      </c>
+      <c r="F119" t="s">
+        <v>2150</v>
+      </c>
+      <c r="G119" t="str">
+        <f t="shared" ref="G119:G123" si="67">+_xlfn.CONCAT("{{ ",E119," }}")</f>
+        <v>{{ ev_sim4 }}</v>
+      </c>
+      <c r="H119">
+        <v>155</v>
+      </c>
+      <c r="I119" t="s">
+        <v>1755</v>
+      </c>
       <c r="J119" t="s">
         <v>205</v>
       </c>
@@ -49416,11 +49719,71 @@
         <v>320</v>
       </c>
       <c r="L119" t="str">
+        <f t="shared" si="58"/>
+        <v>'incendios' : r_val['incendios'],</v>
+      </c>
+      <c r="M119" t="str">
         <f t="shared" si="59"/>
-        <v>'incendios' : r_val['incendios'],</v>
+        <v>'ev_sim4': ev_sim4,</v>
+      </c>
+      <c r="N119" t="s">
+        <v>557</v>
+      </c>
+      <c r="O119" t="str">
+        <f t="shared" si="60"/>
+        <v>img_path_ev_sim4 = os.path.join(IMAGES_PATH, r_val["ev_sim4"])</v>
+      </c>
+      <c r="P119" t="str">
+        <f t="shared" si="61"/>
+        <v>if os.path.exists(img_path_ev_sim4):</v>
+      </c>
+      <c r="Q119" t="str">
+        <f t="shared" si="62"/>
+        <v>ev_sim4 = InlineImage(docx_tpl, img_path_ev_sim4, width=Mm(155))</v>
+      </c>
+      <c r="R119" t="s">
+        <v>559</v>
+      </c>
+      <c r="S119" t="str">
+        <f t="shared" si="63"/>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["ev_sim4"]}')</v>
+      </c>
+      <c r="T119" t="str">
+        <f t="shared" si="64"/>
+        <v>ev_sim4 = ''</v>
+      </c>
+      <c r="U119" t="s">
+        <v>558</v>
+      </c>
+      <c r="V119" t="str">
+        <f t="shared" si="65"/>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["ev_sim4"]}: {e}')</v>
+      </c>
+      <c r="W119" t="str">
+        <f t="shared" si="66"/>
+        <v>ev_sim4 = ''</v>
       </c>
     </row>
-    <row r="120" spans="5:23" x14ac:dyDescent="0.3">
+    <row r="120" spans="2:23" x14ac:dyDescent="0.3">
+      <c r="B120" t="s">
+        <v>1898</v>
+      </c>
+      <c r="E120" t="s">
+        <v>2157</v>
+      </c>
+      <c r="F120" t="s">
+        <v>2151</v>
+      </c>
+      <c r="G120" t="str">
+        <f t="shared" si="67"/>
+        <v>{{ ev_sim5 }}</v>
+      </c>
+      <c r="H120">
+        <v>155</v>
+      </c>
+      <c r="I120" t="s">
+        <v>1755</v>
+      </c>
       <c r="J120" t="s">
         <v>582</v>
       </c>
@@ -49428,11 +49791,71 @@
         <v>590</v>
       </c>
       <c r="L120" t="str">
+        <f t="shared" si="58"/>
+        <v>'incen_puesto' : r_val['incen_puesto'],</v>
+      </c>
+      <c r="M120" t="str">
         <f t="shared" si="59"/>
-        <v>'incen_puesto' : r_val['incen_puesto'],</v>
+        <v>'ev_sim5': ev_sim5,</v>
+      </c>
+      <c r="N120" t="s">
+        <v>557</v>
+      </c>
+      <c r="O120" t="str">
+        <f t="shared" si="60"/>
+        <v>img_path_ev_sim5 = os.path.join(IMAGES_PATH, r_val["ev_sim5"])</v>
+      </c>
+      <c r="P120" t="str">
+        <f t="shared" si="61"/>
+        <v>if os.path.exists(img_path_ev_sim5):</v>
+      </c>
+      <c r="Q120" t="str">
+        <f t="shared" si="62"/>
+        <v>ev_sim5 = InlineImage(docx_tpl, img_path_ev_sim5, width=Mm(155))</v>
+      </c>
+      <c r="R120" t="s">
+        <v>559</v>
+      </c>
+      <c r="S120" t="str">
+        <f t="shared" si="63"/>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["ev_sim5"]}')</v>
+      </c>
+      <c r="T120" t="str">
+        <f t="shared" si="64"/>
+        <v>ev_sim5 = ''</v>
+      </c>
+      <c r="U120" t="s">
+        <v>558</v>
+      </c>
+      <c r="V120" t="str">
+        <f t="shared" si="65"/>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["ev_sim5"]}: {e}')</v>
+      </c>
+      <c r="W120" t="str">
+        <f t="shared" si="66"/>
+        <v>ev_sim5 = ''</v>
       </c>
     </row>
-    <row r="121" spans="5:23" x14ac:dyDescent="0.3">
+    <row r="121" spans="2:23" x14ac:dyDescent="0.3">
+      <c r="B121" t="s">
+        <v>1898</v>
+      </c>
+      <c r="E121" t="s">
+        <v>2158</v>
+      </c>
+      <c r="F121" t="s">
+        <v>2152</v>
+      </c>
+      <c r="G121" t="str">
+        <f t="shared" si="67"/>
+        <v>{{ ev_sim6 }}</v>
+      </c>
+      <c r="H121">
+        <v>155</v>
+      </c>
+      <c r="I121" t="s">
+        <v>1755</v>
+      </c>
       <c r="J121" t="s">
         <v>650</v>
       </c>
@@ -49440,11 +49863,71 @@
         <v>690</v>
       </c>
       <c r="L121" t="str">
+        <f t="shared" si="58"/>
+        <v>'m_inc' : r_val['m_inc'],</v>
+      </c>
+      <c r="M121" t="str">
         <f t="shared" si="59"/>
-        <v>'m_inc' : r_val['m_inc'],</v>
+        <v>'ev_sim6': ev_sim6,</v>
+      </c>
+      <c r="N121" t="s">
+        <v>557</v>
+      </c>
+      <c r="O121" t="str">
+        <f t="shared" si="60"/>
+        <v>img_path_ev_sim6 = os.path.join(IMAGES_PATH, r_val["ev_sim6"])</v>
+      </c>
+      <c r="P121" t="str">
+        <f t="shared" si="61"/>
+        <v>if os.path.exists(img_path_ev_sim6):</v>
+      </c>
+      <c r="Q121" t="str">
+        <f t="shared" si="62"/>
+        <v>ev_sim6 = InlineImage(docx_tpl, img_path_ev_sim6, width=Mm(155))</v>
+      </c>
+      <c r="R121" t="s">
+        <v>559</v>
+      </c>
+      <c r="S121" t="str">
+        <f t="shared" si="63"/>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["ev_sim6"]}')</v>
+      </c>
+      <c r="T121" t="str">
+        <f t="shared" si="64"/>
+        <v>ev_sim6 = ''</v>
+      </c>
+      <c r="U121" t="s">
+        <v>558</v>
+      </c>
+      <c r="V121" t="str">
+        <f t="shared" si="65"/>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["ev_sim6"]}: {e}')</v>
+      </c>
+      <c r="W121" t="str">
+        <f t="shared" si="66"/>
+        <v>ev_sim6 = ''</v>
       </c>
     </row>
-    <row r="122" spans="5:23" x14ac:dyDescent="0.3">
+    <row r="122" spans="2:23" x14ac:dyDescent="0.3">
+      <c r="B122" t="s">
+        <v>1898</v>
+      </c>
+      <c r="E122" t="s">
+        <v>2159</v>
+      </c>
+      <c r="F122" t="s">
+        <v>2173</v>
+      </c>
+      <c r="G122" t="str">
+        <f t="shared" si="67"/>
+        <v>{{ ev_sim7 }}</v>
+      </c>
+      <c r="H122">
+        <v>155</v>
+      </c>
+      <c r="I122" t="s">
+        <v>1755</v>
+      </c>
       <c r="J122" t="s">
         <v>206</v>
       </c>
@@ -49452,11 +49935,71 @@
         <v>321</v>
       </c>
       <c r="L122" t="str">
+        <f t="shared" si="58"/>
+        <v>'inc_suplente' : r_val['inc_suplente'],</v>
+      </c>
+      <c r="M122" t="str">
         <f t="shared" si="59"/>
-        <v>'inc_suplente' : r_val['inc_suplente'],</v>
+        <v>'ev_sim7': ev_sim7,</v>
+      </c>
+      <c r="N122" t="s">
+        <v>557</v>
+      </c>
+      <c r="O122" t="str">
+        <f t="shared" si="60"/>
+        <v>img_path_ev_sim7 = os.path.join(IMAGES_PATH, r_val["ev_sim7"])</v>
+      </c>
+      <c r="P122" t="str">
+        <f t="shared" si="61"/>
+        <v>if os.path.exists(img_path_ev_sim7):</v>
+      </c>
+      <c r="Q122" t="str">
+        <f t="shared" si="62"/>
+        <v>ev_sim7 = InlineImage(docx_tpl, img_path_ev_sim7, width=Mm(155))</v>
+      </c>
+      <c r="R122" t="s">
+        <v>559</v>
+      </c>
+      <c r="S122" t="str">
+        <f t="shared" si="63"/>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["ev_sim7"]}')</v>
+      </c>
+      <c r="T122" t="str">
+        <f t="shared" si="64"/>
+        <v>ev_sim7 = ''</v>
+      </c>
+      <c r="U122" t="s">
+        <v>558</v>
+      </c>
+      <c r="V122" t="str">
+        <f t="shared" si="65"/>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["ev_sim7"]}: {e}')</v>
+      </c>
+      <c r="W122" t="str">
+        <f t="shared" si="66"/>
+        <v>ev_sim7 = ''</v>
       </c>
     </row>
-    <row r="123" spans="5:23" x14ac:dyDescent="0.3">
+    <row r="123" spans="2:23" x14ac:dyDescent="0.3">
+      <c r="B123" t="s">
+        <v>1898</v>
+      </c>
+      <c r="E123" t="s">
+        <v>2160</v>
+      </c>
+      <c r="F123" t="s">
+        <v>2174</v>
+      </c>
+      <c r="G123" t="str">
+        <f t="shared" si="67"/>
+        <v>{{ ev_sim8 }}</v>
+      </c>
+      <c r="H123">
+        <v>155</v>
+      </c>
+      <c r="I123" t="s">
+        <v>1755</v>
+      </c>
       <c r="J123" t="s">
         <v>583</v>
       </c>
@@ -49464,11 +50007,72 @@
         <v>591</v>
       </c>
       <c r="L123" t="str">
+        <f t="shared" si="58"/>
+        <v>'supl_inc_puesto' : r_val['supl_inc_puesto'],</v>
+      </c>
+      <c r="M123" t="str">
         <f t="shared" si="59"/>
-        <v>'supl_inc_puesto' : r_val['supl_inc_puesto'],</v>
+        <v>'ev_sim8': ev_sim8,</v>
+      </c>
+      <c r="N123" t="s">
+        <v>557</v>
+      </c>
+      <c r="O123" t="str">
+        <f t="shared" si="60"/>
+        <v>img_path_ev_sim8 = os.path.join(IMAGES_PATH, r_val["ev_sim8"])</v>
+      </c>
+      <c r="P123" t="str">
+        <f t="shared" si="61"/>
+        <v>if os.path.exists(img_path_ev_sim8):</v>
+      </c>
+      <c r="Q123" t="str">
+        <f t="shared" si="62"/>
+        <v>ev_sim8 = InlineImage(docx_tpl, img_path_ev_sim8, width=Mm(155))</v>
+      </c>
+      <c r="R123" t="s">
+        <v>559</v>
+      </c>
+      <c r="S123" t="str">
+        <f t="shared" si="63"/>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["ev_sim8"]}')</v>
+      </c>
+      <c r="T123" t="str">
+        <f t="shared" si="64"/>
+        <v>ev_sim8 = ''</v>
+      </c>
+      <c r="U123" t="s">
+        <v>558</v>
+      </c>
+      <c r="V123" t="str">
+        <f t="shared" si="65"/>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["ev_sim8"]}: {e}')</v>
+      </c>
+      <c r="W123" t="str">
+        <f t="shared" si="66"/>
+        <v>ev_sim8 = ''</v>
       </c>
     </row>
-    <row r="124" spans="5:23" x14ac:dyDescent="0.3">
+    <row r="124" spans="2:23" x14ac:dyDescent="0.3">
+      <c r="B124" t="s">
+        <v>1898</v>
+      </c>
+      <c r="E124" t="s">
+        <v>2153</v>
+      </c>
+      <c r="F124" t="str">
+        <f t="shared" ref="F124:F125" si="68">+_xlfn.CONCAT(E124,".png")</f>
+        <v>acta3.png</v>
+      </c>
+      <c r="G124" t="str">
+        <f t="shared" ref="G124:G125" si="69">+_xlfn.CONCAT("{{ ",E124," }}")</f>
+        <v>{{ acta3 }}</v>
+      </c>
+      <c r="H124">
+        <v>155</v>
+      </c>
+      <c r="I124" t="s">
+        <v>1755</v>
+      </c>
       <c r="J124" t="s">
         <v>651</v>
       </c>
@@ -49476,11 +50080,72 @@
         <v>691</v>
       </c>
       <c r="L124" t="str">
-        <f t="shared" si="59"/>
+        <f t="shared" si="58"/>
         <v>'m_supl_inc' : r_val['m_supl_inc'],</v>
       </c>
+      <c r="M124" t="str">
+        <f t="shared" ref="M124:M125" si="70">+_xlfn.CONCAT("'",E124,"': ",E124,",")</f>
+        <v>'acta3': acta3,</v>
+      </c>
+      <c r="N124" t="s">
+        <v>557</v>
+      </c>
+      <c r="O124" t="str">
+        <f t="shared" ref="O124:O125" si="71">+_xlfn.CONCAT("img_path_",E124," = os.path.join(IMAGES_PATH, r_val[""",E124,"""])")</f>
+        <v>img_path_acta3 = os.path.join(IMAGES_PATH, r_val["acta3"])</v>
+      </c>
+      <c r="P124" t="str">
+        <f t="shared" ref="P124:P125" si="72">+_xlfn.CONCAT("if os.path.exists(img_path_",E124,"):")</f>
+        <v>if os.path.exists(img_path_acta3):</v>
+      </c>
+      <c r="Q124" t="str">
+        <f t="shared" ref="Q124:Q125" si="73">+_xlfn.CONCAT(E124," = InlineImage(docx_tpl, img_path_",E124,", ",I124,"=Mm(",H124,"))")</f>
+        <v>acta3 = InlineImage(docx_tpl, img_path_acta3, width=Mm(155))</v>
+      </c>
+      <c r="R124" t="s">
+        <v>559</v>
+      </c>
+      <c r="S124" t="str">
+        <f t="shared" ref="S124:S125" si="74">+_xlfn.CONCAT("print(f'Advertencia: No se encontró la imagen {r_val[""",E124,"""]}')")</f>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["acta3"]}')</v>
+      </c>
+      <c r="T124" t="str">
+        <f t="shared" ref="T124:T125" si="75">+_xlfn.CONCAT(E124," = ''")</f>
+        <v>acta3 = ''</v>
+      </c>
+      <c r="U124" t="s">
+        <v>558</v>
+      </c>
+      <c r="V124" t="str">
+        <f t="shared" ref="V124:V125" si="76">+_xlfn.CONCAT("print(f'Advertencia: No se pudo cargar la imagen {r_val[""",E124,"""]}: {e}')")</f>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["acta3"]}: {e}')</v>
+      </c>
+      <c r="W124" t="str">
+        <f t="shared" ref="W124:W125" si="77">+_xlfn.CONCAT(E124," = ''")</f>
+        <v>acta3 = ''</v>
+      </c>
     </row>
-    <row r="125" spans="5:23" x14ac:dyDescent="0.3">
+    <row r="125" spans="2:23" x14ac:dyDescent="0.3">
+      <c r="B125" t="s">
+        <v>1898</v>
+      </c>
+      <c r="E125" t="s">
+        <v>2154</v>
+      </c>
+      <c r="F125" t="str">
+        <f t="shared" si="68"/>
+        <v>acta4.png</v>
+      </c>
+      <c r="G125" t="str">
+        <f t="shared" si="69"/>
+        <v>{{ acta4 }}</v>
+      </c>
+      <c r="H125">
+        <v>155</v>
+      </c>
+      <c r="I125" t="s">
+        <v>1755</v>
+      </c>
       <c r="J125" t="s">
         <v>207</v>
       </c>
@@ -49488,11 +50153,52 @@
         <v>322</v>
       </c>
       <c r="L125" t="str">
-        <f t="shared" si="59"/>
+        <f t="shared" si="58"/>
         <v>'primeros_auxilios' : r_val['primeros_auxilios'],</v>
       </c>
+      <c r="M125" t="str">
+        <f t="shared" si="70"/>
+        <v>'acta4': acta4,</v>
+      </c>
+      <c r="N125" t="s">
+        <v>557</v>
+      </c>
+      <c r="O125" t="str">
+        <f t="shared" si="71"/>
+        <v>img_path_acta4 = os.path.join(IMAGES_PATH, r_val["acta4"])</v>
+      </c>
+      <c r="P125" t="str">
+        <f t="shared" si="72"/>
+        <v>if os.path.exists(img_path_acta4):</v>
+      </c>
+      <c r="Q125" t="str">
+        <f t="shared" si="73"/>
+        <v>acta4 = InlineImage(docx_tpl, img_path_acta4, width=Mm(155))</v>
+      </c>
+      <c r="R125" t="s">
+        <v>559</v>
+      </c>
+      <c r="S125" t="str">
+        <f t="shared" si="74"/>
+        <v>print(f'Advertencia: No se encontró la imagen {r_val["acta4"]}')</v>
+      </c>
+      <c r="T125" t="str">
+        <f t="shared" si="75"/>
+        <v>acta4 = ''</v>
+      </c>
+      <c r="U125" t="s">
+        <v>558</v>
+      </c>
+      <c r="V125" t="str">
+        <f t="shared" si="76"/>
+        <v>print(f'Advertencia: No se pudo cargar la imagen {r_val["acta4"]}: {e}')</v>
+      </c>
+      <c r="W125" t="str">
+        <f t="shared" si="77"/>
+        <v>acta4 = ''</v>
+      </c>
     </row>
-    <row r="126" spans="5:23" x14ac:dyDescent="0.3">
+    <row r="126" spans="2:23" x14ac:dyDescent="0.3">
       <c r="J126" t="s">
         <v>584</v>
       </c>
@@ -49500,11 +50206,11 @@
         <v>592</v>
       </c>
       <c r="L126" t="str">
-        <f t="shared" si="59"/>
+        <f t="shared" si="58"/>
         <v>'prim_aux_puesto' : r_val['prim_aux_puesto'],</v>
       </c>
     </row>
-    <row r="127" spans="5:23" x14ac:dyDescent="0.3">
+    <row r="127" spans="2:23" x14ac:dyDescent="0.3">
       <c r="J127" t="s">
         <v>652</v>
       </c>
@@ -49512,11 +50218,11 @@
         <v>692</v>
       </c>
       <c r="L127" t="str">
-        <f t="shared" si="59"/>
+        <f t="shared" si="58"/>
         <v>'m_prim_aux' : r_val['m_prim_aux'],</v>
       </c>
     </row>
-    <row r="128" spans="5:23" x14ac:dyDescent="0.3">
+    <row r="128" spans="2:23" x14ac:dyDescent="0.3">
       <c r="J128" t="s">
         <v>208</v>
       </c>
@@ -49524,7 +50230,7 @@
         <v>323</v>
       </c>
       <c r="L128" t="str">
-        <f t="shared" si="59"/>
+        <f t="shared" si="58"/>
         <v>'aux_suplente' : r_val['aux_suplente'],</v>
       </c>
     </row>
@@ -49536,7 +50242,7 @@
         <v>593</v>
       </c>
       <c r="L129" t="str">
-        <f t="shared" si="59"/>
+        <f t="shared" si="58"/>
         <v>'supl_prim_aux_puesto' : r_val['supl_prim_aux_puesto'],</v>
       </c>
     </row>
@@ -49548,7 +50254,7 @@
         <v>693</v>
       </c>
       <c r="L130" t="str">
-        <f t="shared" si="59"/>
+        <f t="shared" si="58"/>
         <v>'m_supl_paux' : r_val['m_supl_paux'],</v>
       </c>
     </row>
@@ -49560,7 +50266,7 @@
         <v>324</v>
       </c>
       <c r="L131" t="str">
-        <f t="shared" si="59"/>
+        <f t="shared" si="58"/>
         <v>'busqueda' : r_val['busqueda'],</v>
       </c>
     </row>
@@ -49572,7 +50278,7 @@
         <v>594</v>
       </c>
       <c r="L132" t="str">
-        <f t="shared" si="59"/>
+        <f t="shared" si="58"/>
         <v>'busq_puesto' : r_val['busq_puesto'],</v>
       </c>
     </row>
@@ -49584,7 +50290,7 @@
         <v>694</v>
       </c>
       <c r="L133" t="str">
-        <f t="shared" si="59"/>
+        <f t="shared" si="58"/>
         <v>'m_busq' : r_val['m_busq'],</v>
       </c>
     </row>
@@ -49596,7 +50302,7 @@
         <v>325</v>
       </c>
       <c r="L134" t="str">
-        <f t="shared" si="59"/>
+        <f t="shared" si="58"/>
         <v>'busq_suplente' : r_val['busq_suplente'],</v>
       </c>
     </row>
@@ -49608,7 +50314,7 @@
         <v>595</v>
       </c>
       <c r="L135" t="str">
-        <f t="shared" si="59"/>
+        <f t="shared" si="58"/>
         <v>'supl_busq_puesto' : r_val['supl_busq_puesto'],</v>
       </c>
     </row>
@@ -49620,7 +50326,7 @@
         <v>695</v>
       </c>
       <c r="L136" t="str">
-        <f t="shared" si="59"/>
+        <f t="shared" si="58"/>
         <v>'m_supl_busq' : r_val['m_supl_busq'],</v>
       </c>
     </row>
@@ -49632,7 +50338,7 @@
         <v>326</v>
       </c>
       <c r="L137" t="str">
-        <f t="shared" si="59"/>
+        <f t="shared" si="58"/>
         <v>'descrip_gi' : r_val['descrip_gi'],</v>
       </c>
     </row>
@@ -49644,7 +50350,7 @@
         <v>327</v>
       </c>
       <c r="L138" t="str">
-        <f t="shared" si="59"/>
+        <f t="shared" si="58"/>
         <v>'gas_inflamable' : r_val['gas_inflamable'],</v>
       </c>
     </row>
@@ -49656,7 +50362,7 @@
         <v>328</v>
       </c>
       <c r="L139" t="str">
-        <f t="shared" si="59"/>
+        <f t="shared" si="58"/>
         <v>'valor_gi' : r_val['valor_gi'],</v>
       </c>
     </row>
@@ -49668,7 +50374,7 @@
         <v>329</v>
       </c>
       <c r="L140" t="str">
-        <f t="shared" si="59"/>
+        <f t="shared" si="58"/>
         <v>'descrp_li' : r_val['descrp_li'],</v>
       </c>
     </row>
@@ -49680,7 +50386,7 @@
         <v>330</v>
       </c>
       <c r="L141" t="str">
-        <f t="shared" si="59"/>
+        <f t="shared" si="58"/>
         <v>'liquido_inflamable' : r_val['liquido_inflamable'],</v>
       </c>
     </row>
@@ -49692,7 +50398,7 @@
         <v>331</v>
       </c>
       <c r="L142" t="str">
-        <f t="shared" si="59"/>
+        <f t="shared" si="58"/>
         <v>'valor_li' : r_val['valor_li'],</v>
       </c>
     </row>
@@ -49704,7 +50410,7 @@
         <v>332</v>
       </c>
       <c r="L143" t="str">
-        <f t="shared" ref="L143:L181" si="60">+_xlfn.CONCAT("'",J143,"' : r_val['",J143,"'],")</f>
+        <f t="shared" ref="L143:L181" si="78">+_xlfn.CONCAT("'",J143,"' : r_val['",J143,"'],")</f>
         <v>'descrip_lc' : r_val['descrip_lc'],</v>
       </c>
     </row>
@@ -49716,7 +50422,7 @@
         <v>333</v>
       </c>
       <c r="L144" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'liquido_combustible' : r_val['liquido_combustible'],</v>
       </c>
     </row>
@@ -49728,7 +50434,7 @@
         <v>334</v>
       </c>
       <c r="L145" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'valor_lc' : r_val['valor_lc'],</v>
       </c>
     </row>
@@ -49740,7 +50446,7 @@
         <v>335</v>
       </c>
       <c r="L146" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'descrip_sc' : r_val['descrip_sc'],</v>
       </c>
     </row>
@@ -49752,7 +50458,7 @@
         <v>336</v>
       </c>
       <c r="L147" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'solido_combusible' : r_val['solido_combusible'],</v>
       </c>
     </row>
@@ -49764,7 +50470,7 @@
         <v>337</v>
       </c>
       <c r="L148" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'valor_sc' : r_val['valor_sc'],</v>
       </c>
     </row>
@@ -49776,7 +50482,7 @@
         <v>338</v>
       </c>
       <c r="L149" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'tipo_riesgo' : r_val['tipo_riesgo'],</v>
       </c>
     </row>
@@ -49788,7 +50494,7 @@
         <v>656</v>
       </c>
       <c r="L150" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'nombre1' : r_val['nombre1'],</v>
       </c>
     </row>
@@ -49800,7 +50506,7 @@
         <v>657</v>
       </c>
       <c r="L151" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'puesto1' : r_val['puesto1'],</v>
       </c>
     </row>
@@ -49812,7 +50518,7 @@
         <v>658</v>
       </c>
       <c r="L152" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'m1' : r_val['m1'],</v>
       </c>
     </row>
@@ -49824,7 +50530,7 @@
         <v>659</v>
       </c>
       <c r="L153" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'nombre2' : r_val['nombre2'],</v>
       </c>
     </row>
@@ -49836,7 +50542,7 @@
         <v>660</v>
       </c>
       <c r="L154" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'puesto2' : r_val['puesto2'],</v>
       </c>
     </row>
@@ -49848,7 +50554,7 @@
         <v>661</v>
       </c>
       <c r="L155" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'m2' : r_val['m2'],</v>
       </c>
     </row>
@@ -49860,7 +50566,7 @@
         <v>662</v>
       </c>
       <c r="L156" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'nombre3' : r_val['nombre3'],</v>
       </c>
     </row>
@@ -49872,7 +50578,7 @@
         <v>663</v>
       </c>
       <c r="L157" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'puesto3' : r_val['puesto3'],</v>
       </c>
     </row>
@@ -49884,7 +50590,7 @@
         <v>664</v>
       </c>
       <c r="L158" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'m3' : r_val['m3'],</v>
       </c>
     </row>
@@ -49896,7 +50602,7 @@
         <v>665</v>
       </c>
       <c r="L159" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'nombre4' : r_val['nombre4'],</v>
       </c>
     </row>
@@ -49908,7 +50614,7 @@
         <v>666</v>
       </c>
       <c r="L160" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'puesto4' : r_val['puesto4'],</v>
       </c>
     </row>
@@ -49920,7 +50626,7 @@
         <v>667</v>
       </c>
       <c r="L161" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'m4' : r_val['m4'],</v>
       </c>
     </row>
@@ -49932,7 +50638,7 @@
         <v>668</v>
       </c>
       <c r="L162" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'nombre5' : r_val['nombre5'],</v>
       </c>
     </row>
@@ -49944,7 +50650,7 @@
         <v>669</v>
       </c>
       <c r="L163" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'puesto5' : r_val['puesto5'],</v>
       </c>
     </row>
@@ -49956,7 +50662,7 @@
         <v>670</v>
       </c>
       <c r="L164" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'m5' : r_val['m5'],</v>
       </c>
     </row>
@@ -49968,7 +50674,7 @@
         <v>671</v>
       </c>
       <c r="L165" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'nombre6' : r_val['nombre6'],</v>
       </c>
     </row>
@@ -49980,7 +50686,7 @@
         <v>672</v>
       </c>
       <c r="L166" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'puesto6' : r_val['puesto6'],</v>
       </c>
     </row>
@@ -49992,7 +50698,7 @@
         <v>673</v>
       </c>
       <c r="L167" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'m6' : r_val['m6'],</v>
       </c>
     </row>
@@ -50004,7 +50710,7 @@
         <v>674</v>
       </c>
       <c r="L168" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'nombre7' : r_val['nombre7'],</v>
       </c>
     </row>
@@ -50016,7 +50722,7 @@
         <v>675</v>
       </c>
       <c r="L169" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'puesto7' : r_val['puesto7'],</v>
       </c>
     </row>
@@ -50028,7 +50734,7 @@
         <v>676</v>
       </c>
       <c r="L170" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'m7' : r_val['m7'],</v>
       </c>
     </row>
@@ -50040,7 +50746,7 @@
         <v>677</v>
       </c>
       <c r="L171" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'nombre8' : r_val['nombre8'],</v>
       </c>
     </row>
@@ -50052,7 +50758,7 @@
         <v>678</v>
       </c>
       <c r="L172" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'puesto8' : r_val['puesto8'],</v>
       </c>
     </row>
@@ -50064,7 +50770,7 @@
         <v>679</v>
       </c>
       <c r="L173" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'m8' : r_val['m8'],</v>
       </c>
     </row>
@@ -50076,7 +50782,7 @@
         <v>680</v>
       </c>
       <c r="L174" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'nombre9' : r_val['nombre9'],</v>
       </c>
     </row>
@@ -50088,7 +50794,7 @@
         <v>681</v>
       </c>
       <c r="L175" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'puesto9' : r_val['puesto9'],</v>
       </c>
     </row>
@@ -50100,7 +50806,7 @@
         <v>682</v>
       </c>
       <c r="L176" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'m9' : r_val['m9'],</v>
       </c>
     </row>
@@ -50112,7 +50818,7 @@
         <v>683</v>
       </c>
       <c r="L177" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'nombre10' : r_val['nombre10'],</v>
       </c>
     </row>
@@ -50124,7 +50830,7 @@
         <v>684</v>
       </c>
       <c r="L178" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'puesto10' : r_val['puesto10'],</v>
       </c>
     </row>
@@ -50136,7 +50842,7 @@
         <v>685</v>
       </c>
       <c r="L179" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'m10' : r_val['m10'],</v>
       </c>
     </row>
@@ -50149,7 +50855,7 @@
         <v>{{ registro_perito }}</v>
       </c>
       <c r="L180" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'registro_perito' : r_val['registro_perito'],</v>
       </c>
     </row>
@@ -50162,7 +50868,7 @@
         <v>{{ no_registro }}</v>
       </c>
       <c r="L181" t="str">
-        <f t="shared" si="60"/>
+        <f t="shared" si="78"/>
         <v>'no_registro' : r_val['no_registro'],</v>
       </c>
     </row>
@@ -50171,11 +50877,11 @@
         <v>1732</v>
       </c>
       <c r="K182" t="str">
-        <f t="shared" ref="K182:K183" si="61">+_xlfn.CONCAT("{{ ",J182," }}")</f>
+        <f t="shared" ref="K182:K183" si="79">+_xlfn.CONCAT("{{ ",J182," }}")</f>
         <v>{{ dh_int }}</v>
       </c>
       <c r="L182" t="str">
-        <f t="shared" ref="L182:L183" si="62">+_xlfn.CONCAT("'",J182,"' : r_val['",J182,"'],")</f>
+        <f t="shared" ref="L182:L183" si="80">+_xlfn.CONCAT("'",J182,"' : r_val['",J182,"'],")</f>
         <v>'dh_int' : r_val['dh_int'],</v>
       </c>
     </row>
@@ -50184,11 +50890,11 @@
         <v>1733</v>
       </c>
       <c r="K183" t="str">
-        <f t="shared" si="61"/>
+        <f t="shared" si="79"/>
         <v>{{ dh_ext }}</v>
       </c>
       <c r="L183" t="str">
-        <f t="shared" si="62"/>
+        <f t="shared" si="80"/>
         <v>'dh_ext' : r_val['dh_ext'],</v>
       </c>
     </row>
@@ -50197,11 +50903,11 @@
         <v>1734</v>
       </c>
       <c r="K184" t="str">
-        <f t="shared" ref="K184" si="63">+_xlfn.CONCAT("{{ ",J184," }}")</f>
+        <f t="shared" ref="K184" si="81">+_xlfn.CONCAT("{{ ",J184," }}")</f>
         <v>{{ detectores_ext }}</v>
       </c>
       <c r="L184" t="str">
-        <f t="shared" ref="L184" si="64">+_xlfn.CONCAT("'",J184,"' : r_val['",J184,"'],")</f>
+        <f t="shared" ref="L184" si="82">+_xlfn.CONCAT("'",J184,"' : r_val['",J184,"'],")</f>
         <v>'detectores_ext' : r_val['detectores_ext'],</v>
       </c>
     </row>
@@ -50210,11 +50916,11 @@
         <v>1735</v>
       </c>
       <c r="K185" t="str">
-        <f t="shared" ref="K185" si="65">+_xlfn.CONCAT("{{ ",J185," }}")</f>
+        <f t="shared" ref="K185" si="83">+_xlfn.CONCAT("{{ ",J185," }}")</f>
         <v>{{ coord_sup_puesto }}</v>
       </c>
       <c r="L185" t="str">
-        <f t="shared" ref="L185" si="66">+_xlfn.CONCAT("'",J185,"' : r_val['",J185,"'],")</f>
+        <f t="shared" ref="L185" si="84">+_xlfn.CONCAT("'",J185,"' : r_val['",J185,"'],")</f>
         <v>'coord_sup_puesto' : r_val['coord_sup_puesto'],</v>
       </c>
     </row>
@@ -50223,11 +50929,11 @@
         <v>1741</v>
       </c>
       <c r="K186" t="str">
-        <f t="shared" ref="K186:K189" si="67">+_xlfn.CONCAT("{{ ",J186," }}")</f>
+        <f t="shared" ref="K186:K189" si="85">+_xlfn.CONCAT("{{ ",J186," }}")</f>
         <v>{{ riesgo1 }}</v>
       </c>
       <c r="L186" t="str">
-        <f t="shared" ref="L186:L189" si="68">+_xlfn.CONCAT("'",J186,"' : r_val['",J186,"'],")</f>
+        <f t="shared" ref="L186:L189" si="86">+_xlfn.CONCAT("'",J186,"' : r_val['",J186,"'],")</f>
         <v>'riesgo1' : r_val['riesgo1'],</v>
       </c>
     </row>
@@ -50236,11 +50942,11 @@
         <v>1742</v>
       </c>
       <c r="K187" t="str">
-        <f t="shared" si="67"/>
+        <f t="shared" si="85"/>
         <v>{{ riesgo2 }}</v>
       </c>
       <c r="L187" t="str">
-        <f t="shared" si="68"/>
+        <f t="shared" si="86"/>
         <v>'riesgo2' : r_val['riesgo2'],</v>
       </c>
     </row>
@@ -50249,11 +50955,11 @@
         <v>1743</v>
       </c>
       <c r="K188" t="str">
-        <f t="shared" si="67"/>
+        <f t="shared" si="85"/>
         <v>{{ riesgo3 }}</v>
       </c>
       <c r="L188" t="str">
-        <f t="shared" si="68"/>
+        <f t="shared" si="86"/>
         <v>'riesgo3' : r_val['riesgo3'],</v>
       </c>
     </row>
@@ -50262,11 +50968,11 @@
         <v>1744</v>
       </c>
       <c r="K189" t="str">
-        <f t="shared" si="67"/>
+        <f t="shared" si="85"/>
         <v>{{ riesgo4 }}</v>
       </c>
       <c r="L189" t="str">
-        <f t="shared" si="68"/>
+        <f t="shared" si="86"/>
         <v>'riesgo4' : r_val['riesgo4'],</v>
       </c>
     </row>
@@ -50275,11 +50981,11 @@
         <v>1748</v>
       </c>
       <c r="K190" t="str">
-        <f t="shared" ref="K190" si="69">+_xlfn.CONCAT("{{ ",J190," }}")</f>
+        <f t="shared" ref="K190" si="87">+_xlfn.CONCAT("{{ ",J190," }}")</f>
         <v>{{ valor_gri }}</v>
       </c>
       <c r="L190" t="str">
-        <f t="shared" ref="L190" si="70">+_xlfn.CONCAT("'",J190,"' : r_val['",J190,"'],")</f>
+        <f t="shared" ref="L190" si="88">+_xlfn.CONCAT("'",J190,"' : r_val['",J190,"'],")</f>
         <v>'valor_gri' : r_val['valor_gri'],</v>
       </c>
     </row>
@@ -50288,11 +50994,11 @@
         <v>1749</v>
       </c>
       <c r="K191" t="str">
-        <f t="shared" ref="K191:K194" si="71">+_xlfn.CONCAT("{{ ",J191," }}")</f>
+        <f t="shared" ref="K191:K194" si="89">+_xlfn.CONCAT("{{ ",J191," }}")</f>
         <v>{{ medidas_ries1 }}</v>
       </c>
       <c r="L191" t="str">
-        <f t="shared" ref="L191:L194" si="72">+_xlfn.CONCAT("'",J191,"' : r_val['",J191,"'],")</f>
+        <f t="shared" ref="L191:L194" si="90">+_xlfn.CONCAT("'",J191,"' : r_val['",J191,"'],")</f>
         <v>'medidas_ries1' : r_val['medidas_ries1'],</v>
       </c>
     </row>
@@ -50301,11 +51007,11 @@
         <v>1750</v>
       </c>
       <c r="K192" t="str">
-        <f t="shared" si="71"/>
+        <f t="shared" si="89"/>
         <v>{{ medidas_ries2 }}</v>
       </c>
       <c r="L192" t="str">
-        <f t="shared" si="72"/>
+        <f t="shared" si="90"/>
         <v>'medidas_ries2' : r_val['medidas_ries2'],</v>
       </c>
     </row>
@@ -50314,11 +51020,11 @@
         <v>1751</v>
       </c>
       <c r="K193" t="str">
-        <f t="shared" si="71"/>
+        <f t="shared" si="89"/>
         <v>{{ medidas_ries3 }}</v>
       </c>
       <c r="L193" t="str">
-        <f t="shared" si="72"/>
+        <f t="shared" si="90"/>
         <v>'medidas_ries3' : r_val['medidas_ries3'],</v>
       </c>
     </row>
@@ -50327,11 +51033,11 @@
         <v>1752</v>
       </c>
       <c r="K194" t="str">
-        <f t="shared" si="71"/>
+        <f t="shared" si="89"/>
         <v>{{ medidas_ries4 }}</v>
       </c>
       <c r="L194" t="str">
-        <f t="shared" si="72"/>
+        <f t="shared" si="90"/>
         <v>'medidas_ries4' : r_val['medidas_ries4'],</v>
       </c>
     </row>
@@ -50340,11 +51046,11 @@
         <v>2075</v>
       </c>
       <c r="K195" t="str">
-        <f t="shared" ref="K195:K210" si="73">+_xlfn.CONCAT("{{ ",J195," }}")</f>
+        <f t="shared" ref="K195:K210" si="91">+_xlfn.CONCAT("{{ ",J195," }}")</f>
         <v>{{ barretas }}</v>
       </c>
       <c r="L195" t="str">
-        <f t="shared" ref="L195:L210" si="74">+_xlfn.CONCAT("'",J195,"' : r_val['",J195,"'],")</f>
+        <f t="shared" ref="L195:L210" si="92">+_xlfn.CONCAT("'",J195,"' : r_val['",J195,"'],")</f>
         <v>'barretas' : r_val['barretas'],</v>
       </c>
     </row>
@@ -50353,11 +51059,11 @@
         <v>2076</v>
       </c>
       <c r="K196" t="str">
-        <f t="shared" si="73"/>
+        <f t="shared" si="91"/>
         <v>{{ barretas_ubicacion }}</v>
       </c>
       <c r="L196" t="str">
-        <f t="shared" si="74"/>
+        <f t="shared" si="92"/>
         <v>'barretas_ubicacion' : r_val['barretas_ubicacion'],</v>
       </c>
     </row>
@@ -50366,11 +51072,11 @@
         <v>2077</v>
       </c>
       <c r="K197" t="str">
-        <f t="shared" si="73"/>
+        <f t="shared" si="91"/>
         <v>{{ banderines }}</v>
       </c>
       <c r="L197" t="str">
-        <f t="shared" si="74"/>
+        <f t="shared" si="92"/>
         <v>'banderines' : r_val['banderines'],</v>
       </c>
     </row>
@@ -50379,11 +51085,11 @@
         <v>2078</v>
       </c>
       <c r="K198" t="str">
-        <f t="shared" si="73"/>
+        <f t="shared" si="91"/>
         <v>{{ banderines_ubicacion }}</v>
       </c>
       <c r="L198" t="str">
-        <f t="shared" si="74"/>
+        <f t="shared" si="92"/>
         <v>'banderines_ubicacion' : r_val['banderines_ubicacion'],</v>
       </c>
     </row>
@@ -50392,11 +51098,11 @@
         <v>2079</v>
       </c>
       <c r="K199" t="str">
-        <f t="shared" si="73"/>
+        <f t="shared" si="91"/>
         <v>{{ casco }}</v>
       </c>
       <c r="L199" t="str">
-        <f t="shared" si="74"/>
+        <f t="shared" si="92"/>
         <v>'casco' : r_val['casco'],</v>
       </c>
     </row>
@@ -50405,11 +51111,11 @@
         <v>2080</v>
       </c>
       <c r="K200" t="str">
-        <f t="shared" si="73"/>
+        <f t="shared" si="91"/>
         <v>{{ casco_ubicacion }}</v>
       </c>
       <c r="L200" t="str">
-        <f t="shared" si="74"/>
+        <f t="shared" si="92"/>
         <v>'casco_ubicacion' : r_val['casco_ubicacion'],</v>
       </c>
     </row>
@@ -50418,11 +51124,11 @@
         <v>2081</v>
       </c>
       <c r="K201" t="str">
-        <f t="shared" si="73"/>
+        <f t="shared" si="91"/>
         <v>{{ guantes }}</v>
       </c>
       <c r="L201" t="str">
-        <f t="shared" si="74"/>
+        <f t="shared" si="92"/>
         <v>'guantes' : r_val['guantes'],</v>
       </c>
     </row>
@@ -50431,11 +51137,11 @@
         <v>2082</v>
       </c>
       <c r="K202" t="str">
-        <f t="shared" si="73"/>
+        <f t="shared" si="91"/>
         <v>{{ guantes_ubicacion }}</v>
       </c>
       <c r="L202" t="str">
-        <f t="shared" si="74"/>
+        <f t="shared" si="92"/>
         <v>'guantes_ubicacion' : r_val['guantes_ubicacion'],</v>
       </c>
     </row>
@@ -50444,11 +51150,11 @@
         <v>2083</v>
       </c>
       <c r="K203" t="str">
-        <f t="shared" si="73"/>
+        <f t="shared" si="91"/>
         <v>{{ linterna }}</v>
       </c>
       <c r="L203" t="str">
-        <f t="shared" si="74"/>
+        <f t="shared" si="92"/>
         <v>'linterna' : r_val['linterna'],</v>
       </c>
     </row>
@@ -50457,11 +51163,11 @@
         <v>2084</v>
       </c>
       <c r="K204" t="str">
-        <f t="shared" si="73"/>
+        <f t="shared" si="91"/>
         <v>{{ linterna_ubicacion }}</v>
       </c>
       <c r="L204" t="str">
-        <f t="shared" si="74"/>
+        <f t="shared" si="92"/>
         <v>'linterna_ubicacion' : r_val['linterna_ubicacion'],</v>
       </c>
     </row>
@@ -50470,11 +51176,11 @@
         <v>2085</v>
       </c>
       <c r="K205" t="str">
-        <f t="shared" si="73"/>
+        <f t="shared" si="91"/>
         <v>{{ pala }}</v>
       </c>
       <c r="L205" t="str">
-        <f t="shared" si="74"/>
+        <f t="shared" si="92"/>
         <v>'pala' : r_val['pala'],</v>
       </c>
     </row>
@@ -50483,11 +51189,11 @@
         <v>2086</v>
       </c>
       <c r="K206" t="str">
-        <f t="shared" si="73"/>
+        <f t="shared" si="91"/>
         <v>{{ pala_ubicacion }}</v>
       </c>
       <c r="L206" t="str">
-        <f t="shared" si="74"/>
+        <f t="shared" si="92"/>
         <v>'pala_ubicacion' : r_val['pala_ubicacion'],</v>
       </c>
     </row>
@@ -50496,11 +51202,11 @@
         <v>2087</v>
       </c>
       <c r="K207" t="str">
-        <f t="shared" si="73"/>
+        <f t="shared" si="91"/>
         <v>{{ pico }}</v>
       </c>
       <c r="L207" t="str">
-        <f t="shared" si="74"/>
+        <f t="shared" si="92"/>
         <v>'pico' : r_val['pico'],</v>
       </c>
     </row>
@@ -50509,11 +51215,11 @@
         <v>2088</v>
       </c>
       <c r="K208" t="str">
-        <f t="shared" si="73"/>
+        <f t="shared" si="91"/>
         <v>{{ pico_ubicacion }}</v>
       </c>
       <c r="L208" t="str">
-        <f t="shared" si="74"/>
+        <f t="shared" si="92"/>
         <v>'pico_ubicacion' : r_val['pico_ubicacion'],</v>
       </c>
     </row>
@@ -50522,11 +51228,11 @@
         <v>2089</v>
       </c>
       <c r="K209" t="str">
-        <f t="shared" si="73"/>
+        <f t="shared" si="91"/>
         <v>{{ camilla }}</v>
       </c>
       <c r="L209" t="str">
-        <f t="shared" si="74"/>
+        <f t="shared" si="92"/>
         <v>'camilla' : r_val['camilla'],</v>
       </c>
     </row>
@@ -50535,11 +51241,11 @@
         <v>2090</v>
       </c>
       <c r="K210" t="str">
-        <f t="shared" si="73"/>
+        <f t="shared" si="91"/>
         <v>{{ camilla_ubicacion }}</v>
       </c>
       <c r="L210" t="str">
-        <f t="shared" si="74"/>
+        <f t="shared" si="92"/>
         <v>'camilla_ubicacion' : r_val['camilla_ubicacion'],</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Plantilla para UVP y plantilla General
</commit_message>
<xml_diff>
--- a/Inputs/BD.xlsx
+++ b/Inputs/BD.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/078e1a455e5c02ce/Documentos/GitHub/Proyecto_PIPC/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6340" documentId="13_ncr:1_{7D3A426E-EC5E-453A-8CC7-F83B71F24F18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D9538B94-DA9D-401D-B864-ED3FC7B63852}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{898522BF-B0F8-4888-9748-DC730D5D6CBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4A66393B-FE24-4A2A-8A20-28854F4232E6}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3F095A75-F066-4695-8672-8D4315F1EF23}"/>
   </bookViews>
@@ -563,7 +563,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7178" uniqueCount="2175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7254" uniqueCount="2203">
   <si>
     <t>dia</t>
   </si>
@@ -7088,6 +7088,90 @@
   </si>
   <si>
     <t>ev_sim (8).png</t>
+  </si>
+  <si>
+    <t>comunicación</t>
+  </si>
+  <si>
+    <t>CASTELLANOS PAREDES ESMERALDA JAMÍN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VELÁZQUEZ RÍOS ARMANDO DE JESÚS </t>
+  </si>
+  <si>
+    <t>JORGE ISRAEL URRUTIA VEGA</t>
+  </si>
+  <si>
+    <t>ANA BERTHA MEZA MORALES</t>
+  </si>
+  <si>
+    <t>MAURICIO PIÑÓN VARGAS</t>
+  </si>
+  <si>
+    <t>THE HOME ASIAN</t>
+  </si>
+  <si>
+    <t>THE HOME MARKET</t>
+  </si>
+  <si>
+    <t>HAS210217PH8</t>
+  </si>
+  <si>
+    <t>TIENDA DEPARTAMENTAL</t>
+  </si>
+  <si>
+    <t>BLVD INTERAMERICANO</t>
+  </si>
+  <si>
+    <t>LOMAS DE ANGELOPOLIS, SAN BERNANDINO TLAXCALANCINGO</t>
+  </si>
+  <si>
+    <t>fechamone22@gmail.com</t>
+  </si>
+  <si>
+    <t>NUEVO</t>
+  </si>
+  <si>
+    <t>JIAHAO BAO</t>
+  </si>
+  <si>
+    <t>MARIA FERNANDA NAVA SEGURA</t>
+  </si>
+  <si>
+    <t>10:00 A 21:00 HORAS</t>
+  </si>
+  <si>
+    <t>18.997954848887275, -98.27588030433564</t>
+  </si>
+  <si>
+    <t>ARBYS</t>
+  </si>
+  <si>
+    <t>ANGELES SANCHEZ</t>
+  </si>
+  <si>
+    <t>MARIA LOURDES FLORES PEREZ</t>
+  </si>
+  <si>
+    <t>JAHZEEL ROJAS TORRES</t>
+  </si>
+  <si>
+    <t>ISAI FLORES MARTINEZ</t>
+  </si>
+  <si>
+    <t>PAMELA MONTSERRAT VALDE VEGA</t>
+  </si>
+  <si>
+    <t>LIZBETH FLORES ORTIZ</t>
+  </si>
+  <si>
+    <t>MARISOL GARCIA MORALES</t>
+  </si>
+  <si>
+    <t>VALERIA PAREDES GONZALEZ</t>
+  </si>
+  <si>
+    <t>UVP</t>
   </si>
 </sst>
 </file>
@@ -7710,7 +7794,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp1.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Spin" dx="26" fmlaLink="$A$1" max="30000" min="1" page="10" val="53"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Spin" dx="26" fmlaLink="$A$1" max="30000" min="1" page="10" val="61"/>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7766,10 +7850,6 @@
     <mc:Fallback/>
   </mc:AlternateContent>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8105,10 +8185,13 @@
   <sheetData>
     <row r="1" spans="1:322" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="DS1" t="s">
         <v>1969</v>
+      </c>
+      <c r="EO1" s="11" t="s">
+        <v>2175</v>
       </c>
     </row>
     <row r="2" spans="1:322" x14ac:dyDescent="0.3">
@@ -31015,7 +31098,7 @@
         <v>53</v>
       </c>
       <c r="B55" t="s">
-        <v>551</v>
+        <v>2202</v>
       </c>
       <c r="C55" t="s">
         <v>2037</v>
@@ -31293,6 +31376,21 @@
       <c r="EG55" t="s">
         <v>443</v>
       </c>
+      <c r="EL55" s="11" t="s">
+        <v>2176</v>
+      </c>
+      <c r="EO55" s="11" t="s">
+        <v>2177</v>
+      </c>
+      <c r="ER55" s="11" t="s">
+        <v>2178</v>
+      </c>
+      <c r="EX55" s="11" t="s">
+        <v>2179</v>
+      </c>
+      <c r="FD55" s="11" t="s">
+        <v>2180</v>
+      </c>
       <c r="FJ55" t="s">
         <v>2095</v>
       </c>
@@ -31322,7 +31420,7 @@
         <v>455</v>
       </c>
       <c r="FT55">
-        <f t="shared" ref="FT55:FT62" si="25">60*AG55</f>
+        <f t="shared" ref="FT55:FT63" si="25">60*AG55</f>
         <v>4200</v>
       </c>
       <c r="FU55" s="4">
@@ -31343,7 +31441,7 @@
         <v>54</v>
       </c>
       <c r="B56" t="s">
-        <v>551</v>
+        <v>2202</v>
       </c>
       <c r="C56" t="s">
         <v>2037</v>
@@ -31397,7 +31495,7 @@
         <v>2096</v>
       </c>
       <c r="T56" t="str">
-        <f t="shared" ref="T56:T62" si="26">+IF(V56&gt;1000,"JORGE MANUEL ISLAS GOWER", "NOE MORA RAMIREZ")</f>
+        <f t="shared" ref="T56:T63" si="26">+IF(V56&gt;1000,"JORGE MANUEL ISLAS GOWER", "NOE MORA RAMIREZ")</f>
         <v>NOE MORA RAMIREZ</v>
       </c>
       <c r="V56">
@@ -31468,7 +31566,7 @@
       </c>
       <c r="AR56" s="4">
         <f t="shared" si="18"/>
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="AS56">
         <v>3</v>
@@ -31548,6 +31646,9 @@
       <c r="CF56">
         <v>4</v>
       </c>
+      <c r="CH56">
+        <v>1</v>
+      </c>
       <c r="CI56">
         <v>9</v>
       </c>
@@ -31558,6 +31659,9 @@
         <f t="shared" si="19"/>
         <v>0</v>
       </c>
+      <c r="CM56">
+        <v>2</v>
+      </c>
       <c r="CS56">
         <v>10</v>
       </c>
@@ -31605,6 +31709,21 @@
       </c>
       <c r="EG56" t="s">
         <v>443</v>
+      </c>
+      <c r="EL56" s="11" t="s">
+        <v>2176</v>
+      </c>
+      <c r="EO56" s="11" t="s">
+        <v>2177</v>
+      </c>
+      <c r="ER56" s="11" t="s">
+        <v>2178</v>
+      </c>
+      <c r="EX56" s="11" t="s">
+        <v>2179</v>
+      </c>
+      <c r="FD56" s="11" t="s">
+        <v>2180</v>
       </c>
       <c r="FJ56" t="s">
         <v>820</v>
@@ -31655,7 +31774,7 @@
         <v>55</v>
       </c>
       <c r="B57" t="s">
-        <v>551</v>
+        <v>2202</v>
       </c>
       <c r="C57" t="s">
         <v>2037</v>
@@ -31780,7 +31899,7 @@
       </c>
       <c r="AR57" s="4">
         <f t="shared" si="18"/>
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="AS57">
         <v>2</v>
@@ -31857,6 +31976,9 @@
       <c r="CG57">
         <v>1</v>
       </c>
+      <c r="CH57">
+        <v>1</v>
+      </c>
       <c r="CI57">
         <v>2</v>
       </c>
@@ -31911,6 +32033,21 @@
       </c>
       <c r="EG57" t="s">
         <v>443</v>
+      </c>
+      <c r="EL57" s="11" t="s">
+        <v>2176</v>
+      </c>
+      <c r="EO57" s="11" t="s">
+        <v>2177</v>
+      </c>
+      <c r="ER57" s="11" t="s">
+        <v>2178</v>
+      </c>
+      <c r="EX57" s="11" t="s">
+        <v>2179</v>
+      </c>
+      <c r="FD57" s="11" t="s">
+        <v>2180</v>
       </c>
       <c r="FJ57" t="s">
         <v>2110</v>
@@ -31961,7 +32098,7 @@
         <v>56</v>
       </c>
       <c r="B58" t="s">
-        <v>551</v>
+        <v>2202</v>
       </c>
       <c r="C58" t="s">
         <v>2037</v>
@@ -32226,6 +32363,21 @@
       </c>
       <c r="EG58" t="s">
         <v>443</v>
+      </c>
+      <c r="EL58" s="11" t="s">
+        <v>2176</v>
+      </c>
+      <c r="EO58" s="11" t="s">
+        <v>2177</v>
+      </c>
+      <c r="ER58" s="11" t="s">
+        <v>2178</v>
+      </c>
+      <c r="EX58" s="11" t="s">
+        <v>2179</v>
+      </c>
+      <c r="FD58" s="11" t="s">
+        <v>2180</v>
       </c>
       <c r="FK58">
         <v>0</v>
@@ -32273,7 +32425,7 @@
         <v>57</v>
       </c>
       <c r="B59" t="s">
-        <v>551</v>
+        <v>2202</v>
       </c>
       <c r="C59" t="s">
         <v>2037</v>
@@ -32398,7 +32550,7 @@
       </c>
       <c r="AR59" s="4">
         <f t="shared" si="18"/>
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="AS59">
         <v>2</v>
@@ -32466,6 +32618,12 @@
       <c r="CF59">
         <v>4</v>
       </c>
+      <c r="CH59">
+        <v>1</v>
+      </c>
+      <c r="CI59">
+        <v>1</v>
+      </c>
       <c r="CJ59">
         <v>1</v>
       </c>
@@ -32508,6 +32666,21 @@
       </c>
       <c r="EG59" t="s">
         <v>443</v>
+      </c>
+      <c r="EL59" s="11" t="s">
+        <v>2176</v>
+      </c>
+      <c r="EO59" s="11" t="s">
+        <v>2177</v>
+      </c>
+      <c r="ER59" s="11" t="s">
+        <v>2178</v>
+      </c>
+      <c r="EX59" s="11" t="s">
+        <v>2179</v>
+      </c>
+      <c r="FD59" s="11" t="s">
+        <v>2180</v>
       </c>
       <c r="FJ59" t="s">
         <v>2110</v>
@@ -32558,7 +32731,7 @@
         <v>58</v>
       </c>
       <c r="B60" t="s">
-        <v>551</v>
+        <v>2202</v>
       </c>
       <c r="C60" t="s">
         <v>2037</v>
@@ -32683,7 +32856,7 @@
       </c>
       <c r="AR60" s="4">
         <f t="shared" si="18"/>
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="AS60">
         <v>2</v>
@@ -32751,6 +32924,9 @@
       <c r="CF60">
         <v>7</v>
       </c>
+      <c r="CH60">
+        <v>1</v>
+      </c>
       <c r="CI60">
         <v>5</v>
       </c>
@@ -32811,6 +32987,21 @@
       </c>
       <c r="EG60" t="s">
         <v>443</v>
+      </c>
+      <c r="EL60" s="11" t="s">
+        <v>2176</v>
+      </c>
+      <c r="EO60" s="11" t="s">
+        <v>2177</v>
+      </c>
+      <c r="ER60" s="11" t="s">
+        <v>2178</v>
+      </c>
+      <c r="EX60" s="11" t="s">
+        <v>2179</v>
+      </c>
+      <c r="FD60" s="11" t="s">
+        <v>2180</v>
       </c>
       <c r="FJ60" t="s">
         <v>820</v>
@@ -32861,7 +33052,7 @@
         <v>59</v>
       </c>
       <c r="B61" t="s">
-        <v>551</v>
+        <v>2202</v>
       </c>
       <c r="C61" t="s">
         <v>2037</v>
@@ -32986,7 +33177,7 @@
       </c>
       <c r="AR61" s="4">
         <f t="shared" si="18"/>
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="AS61">
         <v>1</v>
@@ -33053,6 +33244,9 @@
       </c>
       <c r="CF61">
         <v>25</v>
+      </c>
+      <c r="CH61">
+        <v>1</v>
       </c>
       <c r="CI61">
         <v>7</v>
@@ -33114,6 +33308,21 @@
       </c>
       <c r="EG61" t="s">
         <v>443</v>
+      </c>
+      <c r="EL61" s="11" t="s">
+        <v>2176</v>
+      </c>
+      <c r="EO61" s="11" t="s">
+        <v>2177</v>
+      </c>
+      <c r="ER61" s="11" t="s">
+        <v>2178</v>
+      </c>
+      <c r="EX61" s="11" t="s">
+        <v>2179</v>
+      </c>
+      <c r="FD61" s="11" t="s">
+        <v>2180</v>
       </c>
       <c r="FK61">
         <v>0</v>
@@ -33161,7 +33370,7 @@
         <v>60</v>
       </c>
       <c r="B62" t="s">
-        <v>551</v>
+        <v>2202</v>
       </c>
       <c r="C62" t="s">
         <v>2037</v>
@@ -33417,6 +33626,21 @@
       </c>
       <c r="EG62" t="s">
         <v>443</v>
+      </c>
+      <c r="EL62" s="11" t="s">
+        <v>2176</v>
+      </c>
+      <c r="EO62" s="11" t="s">
+        <v>2177</v>
+      </c>
+      <c r="ER62" s="11" t="s">
+        <v>2178</v>
+      </c>
+      <c r="EX62" s="11" t="s">
+        <v>2179</v>
+      </c>
+      <c r="FD62" s="11" t="s">
+        <v>2180</v>
       </c>
       <c r="FJ62" t="s">
         <v>820</v>
@@ -33466,6 +33690,121 @@
       <c r="A63">
         <v>61</v>
       </c>
+      <c r="B63" t="s">
+        <v>2202</v>
+      </c>
+      <c r="C63" t="s">
+        <v>2181</v>
+      </c>
+      <c r="D63" t="s">
+        <v>2182</v>
+      </c>
+      <c r="E63" t="s">
+        <v>2183</v>
+      </c>
+      <c r="G63" t="s">
+        <v>2184</v>
+      </c>
+      <c r="I63" t="s">
+        <v>2185</v>
+      </c>
+      <c r="J63">
+        <v>129</v>
+      </c>
+      <c r="K63" s="10" t="s">
+        <v>2132</v>
+      </c>
+      <c r="L63" t="s">
+        <v>2186</v>
+      </c>
+      <c r="M63" t="s">
+        <v>1492</v>
+      </c>
+      <c r="N63" t="s">
+        <v>424</v>
+      </c>
+      <c r="O63">
+        <v>72830</v>
+      </c>
+      <c r="P63">
+        <v>2213924942</v>
+      </c>
+      <c r="Q63" s="3" t="s">
+        <v>2187</v>
+      </c>
+      <c r="R63" t="s">
+        <v>2188</v>
+      </c>
+      <c r="T63" t="str">
+        <f t="shared" si="26"/>
+        <v>JORGE MANUEL ISLAS GOWER</v>
+      </c>
+      <c r="V63">
+        <v>3000</v>
+      </c>
+      <c r="W63">
+        <v>3000</v>
+      </c>
+      <c r="X63">
+        <v>1</v>
+      </c>
+      <c r="Y63">
+        <v>1</v>
+      </c>
+      <c r="Z63">
+        <v>2</v>
+      </c>
+      <c r="AA63">
+        <v>2</v>
+      </c>
+      <c r="AB63">
+        <v>0</v>
+      </c>
+      <c r="AC63">
+        <v>0</v>
+      </c>
+      <c r="AD63" t="s">
+        <v>912</v>
+      </c>
+      <c r="AE63" t="s">
+        <v>2189</v>
+      </c>
+      <c r="AF63" t="s">
+        <v>2190</v>
+      </c>
+      <c r="AG63">
+        <v>30</v>
+      </c>
+      <c r="AH63">
+        <v>0</v>
+      </c>
+      <c r="AI63">
+        <v>16</v>
+      </c>
+      <c r="AJ63">
+        <v>14</v>
+      </c>
+      <c r="AK63">
+        <v>0</v>
+      </c>
+      <c r="AL63">
+        <v>0</v>
+      </c>
+      <c r="AM63">
+        <v>1</v>
+      </c>
+      <c r="AN63">
+        <v>200</v>
+      </c>
+      <c r="AO63">
+        <v>10</v>
+      </c>
+      <c r="AP63" t="s">
+        <v>430</v>
+      </c>
+      <c r="AQ63" t="s">
+        <v>2191</v>
+      </c>
       <c r="AR63" s="4">
         <f t="shared" si="18"/>
         <v>0</v>
@@ -33474,25 +33813,98 @@
         <f t="shared" si="19"/>
         <v>0</v>
       </c>
+      <c r="DW63">
+        <v>16</v>
+      </c>
+      <c r="DX63" t="s">
+        <v>2054</v>
+      </c>
+      <c r="DY63">
+        <v>2014</v>
+      </c>
+      <c r="DZ63" t="s">
+        <v>2192</v>
+      </c>
+      <c r="EA63" t="s">
+        <v>2193</v>
+      </c>
+      <c r="EB63" t="s">
+        <v>554</v>
+      </c>
+      <c r="EC63" t="s">
+        <v>554</v>
+      </c>
+      <c r="ED63" t="s">
+        <v>554</v>
+      </c>
+      <c r="EF63" t="s">
+        <v>442</v>
+      </c>
+      <c r="EG63" t="s">
+        <v>443</v>
+      </c>
+      <c r="EI63" s="11" t="s">
+        <v>2189</v>
+      </c>
+      <c r="EL63" s="11" t="s">
+        <v>2194</v>
+      </c>
+      <c r="EO63" s="11" t="s">
+        <v>2195</v>
+      </c>
+      <c r="ER63" s="11" t="s">
+        <v>2196</v>
+      </c>
+      <c r="EU63" s="11" t="s">
+        <v>2197</v>
+      </c>
+      <c r="EX63" s="11" t="s">
+        <v>2198</v>
+      </c>
+      <c r="FA63" s="11" t="s">
+        <v>2199</v>
+      </c>
+      <c r="FD63" s="11" t="s">
+        <v>2200</v>
+      </c>
+      <c r="FG63" s="11" t="s">
+        <v>2201</v>
+      </c>
+      <c r="FK63">
+        <v>0</v>
+      </c>
       <c r="FL63" s="4">
         <f t="shared" si="20"/>
         <v>0</v>
       </c>
+      <c r="FN63">
+        <v>0</v>
+      </c>
       <c r="FO63" s="4">
         <f t="shared" si="21"/>
         <v>0</v>
       </c>
+      <c r="FQ63">
+        <v>0</v>
+      </c>
       <c r="FR63" s="4">
         <f t="shared" si="22"/>
         <v>0</v>
       </c>
+      <c r="FS63" t="s">
+        <v>455</v>
+      </c>
+      <c r="FT63">
+        <f t="shared" si="25"/>
+        <v>1800</v>
+      </c>
       <c r="FU63" s="4">
         <f t="shared" si="23"/>
-        <v>0</v>
+        <v>0.12</v>
       </c>
       <c r="FV63" s="4">
         <f t="shared" si="24"/>
-        <v>0</v>
+        <v>0.12</v>
       </c>
       <c r="FW63" s="4" t="str">
         <f t="shared" si="27"/>
@@ -38511,7 +38923,7 @@
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="A3:FV13 FX3:GC43 B14:G14 I14:FV14 KD14:LJ42 A14:A201 D15:FV60 B15:C68 GL43:GW43 GY43:HA43 HC43:HD43 HF43 HK43 HP43:HR43 IC43 IE43 IH43:IJ43 IL43 FX44:IM60 D61:IM201 B69 B70:C201 A202:IM208">
+  <conditionalFormatting sqref="A3:FV13 FX3:GC43 B14:G14 I14:FV14 KD14:LJ42 A14:A201 D15:FV58 GL43:GW43 GY43:HA43 HC43:HD43 HF43 HK43 HP43:HR43 IC43 IE43 IH43:IJ43 IL43 FX44:IM60 EM59:FV60 D59:EL62 EM61:IM62 D63:IM201 B69 B70:C201 A202:IM208 B15:C68">
     <cfRule type="expression" dxfId="40" priority="581">
       <formula>$A3=$A$1</formula>
     </cfRule>
@@ -38718,7 +39130,7 @@
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3:B201" xr:uid="{41C0D522-5D90-43F5-9DB3-E0F81FDE0774}">
-      <formula1>"BANCO, BBVA, COMPARTAMOS, GASOLINERA, GENERAL, GDL"</formula1>
+      <formula1>"BANCO, BBVA, COMPARTAMOS, GASOLINERA, GENERAL, GDL, UVP"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
@@ -38758,16 +39170,17 @@
     <hyperlink ref="Q51" r:id="rId34" xr:uid="{DDE804A1-A1F2-4C98-8E4E-FF4954DAAB88}"/>
     <hyperlink ref="Q55" r:id="rId35" xr:uid="{B9F1BA52-AC5D-4251-9008-A4D12466756B}"/>
     <hyperlink ref="Q56:Q62" r:id="rId36" display="serv.medico@uvp.mx" xr:uid="{35C2D78B-CC24-428B-B9D9-6B044FB382AB}"/>
+    <hyperlink ref="Q63" r:id="rId37" xr:uid="{BAC1ACDE-29E9-44FE-B95B-93A859FE6E4F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId37"/>
-  <legacyDrawing r:id="rId38"/>
+  <drawing r:id="rId38"/>
+  <legacyDrawing r:id="rId39"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x14">
       <controls>
         <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
           <mc:Choice Requires="x14">
-            <control shapeId="1025" r:id="rId39" name="Spinner 1">
+            <control shapeId="1025" r:id="rId40" name="Spinner 1">
               <controlPr defaultSize="0" autoPict="0">
                 <anchor moveWithCells="1" sizeWithCells="1">
                   <from>
@@ -38801,7 +39214,7 @@
     <row r="1" spans="1:310" x14ac:dyDescent="0.3">
       <c r="A1">
         <f>+BD!A1</f>
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="B1" t="s">
         <v>134</v>
@@ -39734,39 +40147,39 @@
     <row r="2" spans="1:310" x14ac:dyDescent="0.3">
       <c r="B2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,2, FALSE)</f>
-        <v>GENERAL</v>
+        <v>UVP</v>
       </c>
       <c r="C2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,3, FALSE)</f>
-        <v>UNIVERSIDAD DEL VALLE DE PUEBLA SC</v>
+        <v>THE HOME ASIAN</v>
       </c>
       <c r="D2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,4, FALSE)</f>
-        <v>COMPLEJO AZTLAN</v>
+        <v>THE HOME MARKET</v>
       </c>
       <c r="E2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,5, FALSE)</f>
-        <v>UVP810305C25</v>
-      </c>
-      <c r="F2" t="str">
+        <v>HAS210217PH8</v>
+      </c>
+      <c r="F2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,6, FALSE)</f>
-        <v>COMPLEJO AZTLAN</v>
+        <v>0</v>
       </c>
       <c r="G2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,7, FALSE)</f>
-        <v>ESCUELA DE EDUCACION MEDIA Y SUPERIOR</v>
-      </c>
-      <c r="H2" t="str">
+        <v>TIENDA DEPARTAMENTAL</v>
+      </c>
+      <c r="H2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,8, FALSE)</f>
-        <v>IMPARTICIÓN DE PROGRAMAS ACADÉMICOS, DESDE LICENCIATURAS HASTA POSGRADOS. ADEMÁS, PROMUEVE LA FORMACIÓN CONTINUA Y RECURSOS DE APRENDIZAJE.</v>
+        <v>0</v>
       </c>
       <c r="I2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,9, FALSE)</f>
-        <v>5 SUR</v>
+        <v>BLVD INTERAMERICANO</v>
       </c>
       <c r="J2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,10, FALSE)</f>
-        <v>5906</v>
+        <v>129</v>
       </c>
       <c r="K2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,11, FALSE)</f>
@@ -39774,11 +40187,11 @@
       </c>
       <c r="L2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,12, FALSE)</f>
-        <v>EL CERRITO</v>
+        <v>LOMAS DE ANGELOPOLIS, SAN BERNANDINO TLAXCALANCINGO</v>
       </c>
       <c r="M2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,13, FALSE)</f>
-        <v>PUEBLA</v>
+        <v>SAN ANDRES CHOLULA</v>
       </c>
       <c r="N2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,14, FALSE)</f>
@@ -39786,23 +40199,23 @@
       </c>
       <c r="O2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,15, FALSE)</f>
-        <v>72440</v>
-      </c>
-      <c r="P2" t="str">
+        <v>72830</v>
+      </c>
+      <c r="P2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,16, FALSE)</f>
-        <v>222 2669488 Ext: 353 y 355</v>
+        <v>2213924942</v>
       </c>
       <c r="Q2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,17, FALSE)</f>
-        <v>serv.medico@uvp.mx</v>
-      </c>
-      <c r="R2">
+        <v>fechamone22@gmail.com</v>
+      </c>
+      <c r="R2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,18, FALSE)</f>
-        <v>13</v>
-      </c>
-      <c r="S2" t="str">
+        <v>NUEVO</v>
+      </c>
+      <c r="S2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,19, FALSE)</f>
-        <v>6 DE DICIEMBRE DE 2010</v>
+        <v>0</v>
       </c>
       <c r="T2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,20, FALSE)</f>
@@ -39814,19 +40227,19 @@
       </c>
       <c r="V2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,22, FALSE)</f>
-        <v>2485</v>
+        <v>3000</v>
       </c>
       <c r="W2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,23, FALSE)</f>
-        <v>4639.5200000000004</v>
+        <v>3000</v>
       </c>
       <c r="X2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,24, FALSE)</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Y2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,25, FALSE)</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Z2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,26, FALSE)</f>
@@ -39838,7 +40251,7 @@
       </c>
       <c r="AB2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,28, FALSE)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,29, FALSE)</f>
@@ -39846,19 +40259,19 @@
       </c>
       <c r="AD2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,30, FALSE)</f>
-        <v>6 CAJONES</v>
+        <v>10 CAJONES</v>
       </c>
       <c r="AE2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,31, FALSE)</f>
-        <v>PRISCILIANO GERARDO ILLESCAS LOZANO</v>
+        <v>JIAHAO BAO</v>
       </c>
       <c r="AF2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,32, FALSE)</f>
-        <v>MODESTO ALFONSO HERNÁNDEZ ORTIZ</v>
+        <v>MARIA FERNANDA NAVA SEGURA</v>
       </c>
       <c r="AG2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,33, FALSE)</f>
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="AH2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,34, FALSE)</f>
@@ -39866,11 +40279,11 @@
       </c>
       <c r="AI2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,35, FALSE)</f>
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="AJ2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,36, FALSE)</f>
-        <v>40</v>
+        <v>14</v>
       </c>
       <c r="AK2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,37, FALSE)</f>
@@ -39886,47 +40299,47 @@
       </c>
       <c r="AN2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,40, FALSE)</f>
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="AO2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,41, FALSE)</f>
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="AP2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,42, FALSE)</f>
-        <v>LUNES - SABADO</v>
+        <v>LUNES - DOMINGO</v>
       </c>
       <c r="AQ2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,43, FALSE)</f>
-        <v>07:00 A 21:00 HORAS</v>
+        <v>10:00 A 21:00 HORAS</v>
       </c>
       <c r="AR2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,44, FALSE)</f>
-        <v>92</v>
+        <v>0</v>
       </c>
       <c r="AS2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,45, FALSE)</f>
-        <v>4</v>
-      </c>
-      <c r="AT2" t="str">
+        <v>0</v>
+      </c>
+      <c r="AT2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,46, FALSE)</f>
-        <v>RECEPCION, BIBLIOTECA, CAI, CAPS</v>
+        <v>0</v>
       </c>
       <c r="AU2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,47, FALSE)</f>
-        <v>39</v>
-      </c>
-      <c r="AV2" t="str">
+        <v>0</v>
+      </c>
+      <c r="AV2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,48, FALSE)</f>
-        <v>EN TODO EL INMUEBLE</v>
+        <v>0</v>
       </c>
       <c r="AW2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,49, FALSE)</f>
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="AX2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,50, FALSE)</f>
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="AY2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,51, FALSE)</f>
@@ -39954,11 +40367,11 @@
       </c>
       <c r="BE2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,57, FALSE)</f>
-        <v>2</v>
-      </c>
-      <c r="BF2" t="str">
+        <v>0</v>
+      </c>
+      <c r="BF2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,58, FALSE)</f>
-        <v>MEGAFONO</v>
+        <v>0</v>
       </c>
       <c r="BG2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,59, FALSE)</f>
@@ -39968,9 +40381,9 @@
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,60, FALSE)</f>
         <v>0</v>
       </c>
-      <c r="BI2" t="str">
+      <c r="BI2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,61, FALSE)</f>
-        <v>COORDINACION, VIGILANCIA, CONTROL EXTERNO</v>
+        <v>0</v>
       </c>
       <c r="BJ2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,62, FALSE)</f>
@@ -39982,51 +40395,51 @@
       </c>
       <c r="BL2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,64, FALSE)</f>
-        <v>5</v>
-      </c>
-      <c r="BM2" t="str">
+        <v>0</v>
+      </c>
+      <c r="BM2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,65, FALSE)</f>
-        <v>OFICINAS</v>
+        <v>0</v>
       </c>
       <c r="BN2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,66, FALSE)</f>
-        <v>1</v>
-      </c>
-      <c r="BO2" t="str">
+        <v>0</v>
+      </c>
+      <c r="BO2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,67, FALSE)</f>
-        <v>GABINETE</v>
+        <v>0</v>
       </c>
       <c r="BP2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,68, FALSE)</f>
-        <v>5</v>
-      </c>
-      <c r="BQ2" t="str">
+        <v>0</v>
+      </c>
+      <c r="BQ2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,69, FALSE)</f>
-        <v>GABINETE</v>
+        <v>0</v>
       </c>
       <c r="BR2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,70, FALSE)</f>
-        <v>4</v>
-      </c>
-      <c r="BS2" t="str">
+        <v>0</v>
+      </c>
+      <c r="BS2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,71, FALSE)</f>
-        <v>GABINETE</v>
+        <v>0</v>
       </c>
       <c r="BT2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,72, FALSE)</f>
-        <v>2</v>
-      </c>
-      <c r="BU2" t="str">
+        <v>0</v>
+      </c>
+      <c r="BU2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,73, FALSE)</f>
-        <v>GABINETE</v>
+        <v>0</v>
       </c>
       <c r="BV2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,74, FALSE)</f>
-        <v>1</v>
-      </c>
-      <c r="BW2" t="str">
+        <v>0</v>
+      </c>
+      <c r="BW2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,75, FALSE)</f>
-        <v>COORDINACION</v>
+        <v>0</v>
       </c>
       <c r="BX2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,76, FALSE)</f>
@@ -40038,31 +40451,31 @@
       </c>
       <c r="BZ2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,78, FALSE)</f>
-        <v>1</v>
-      </c>
-      <c r="CA2" t="str">
+        <v>0</v>
+      </c>
+      <c r="CA2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,79, FALSE)</f>
-        <v>GABINETE</v>
+        <v>0</v>
       </c>
       <c r="CB2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,80, FALSE)</f>
-        <v>2</v>
-      </c>
-      <c r="CC2" t="str">
+        <v>0</v>
+      </c>
+      <c r="CC2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,81, FALSE)</f>
-        <v>GABINETE</v>
+        <v>0</v>
       </c>
       <c r="CD2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,82, FALSE)</f>
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="CE2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,83, FALSE)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CF2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,84, FALSE)</f>
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="CG2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,85, FALSE)</f>
@@ -40070,27 +40483,27 @@
       </c>
       <c r="CH2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,86, FALSE)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CI2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,87, FALSE)</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="CJ2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,88, FALSE)</f>
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="CK2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,89, FALSE)</f>
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="CL2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,90, FALSE)</f>
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="CM2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,91, FALSE)</f>
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="CN2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,92, FALSE)</f>
@@ -40114,11 +40527,11 @@
       </c>
       <c r="CS2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,97, FALSE)</f>
-        <v>9</v>
-      </c>
-      <c r="CT2" t="str">
+        <v>0</v>
+      </c>
+      <c r="CT2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,98, FALSE)</f>
-        <v>AREA COMÚN</v>
+        <v>0</v>
       </c>
       <c r="CU2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,99, FALSE)</f>
@@ -40154,19 +40567,19 @@
       </c>
       <c r="DC2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,107, FALSE)</f>
-        <v>20</v>
-      </c>
-      <c r="DD2" t="str">
+        <v>0</v>
+      </c>
+      <c r="DD2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,108, FALSE)</f>
-        <v>BRIGADISTAS</v>
+        <v>0</v>
       </c>
       <c r="DE2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,109, FALSE)</f>
-        <v>11</v>
-      </c>
-      <c r="DF2" t="str">
+        <v>0</v>
+      </c>
+      <c r="DF2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,110, FALSE)</f>
-        <v>AREA COMÚN</v>
+        <v>0</v>
       </c>
       <c r="DG2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,111, FALSE)</f>
@@ -40234,7 +40647,7 @@
       </c>
       <c r="DW2" s="5">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,127, FALSE)</f>
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="DX2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,128, FALSE)</f>
@@ -40242,27 +40655,27 @@
       </c>
       <c r="DY2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,129, FALSE)</f>
-        <v>2024</v>
+        <v>2014</v>
       </c>
       <c r="DZ2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,130, FALSE)</f>
-        <v>19.017749517200585, -98.2183180754988</v>
+        <v>18.997954848887275, -98.27588030433564</v>
       </c>
       <c r="EA2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,131, FALSE)</f>
-        <v>TAQUERIA</v>
+        <v>ARBYS</v>
       </c>
       <c r="EB2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,132, FALSE)</f>
-        <v>UVP TEOCALLI</v>
+        <v>TERRENO</v>
       </c>
       <c r="EC2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,133, FALSE)</f>
-        <v>CASA HABITACION</v>
+        <v>TERRENO</v>
       </c>
       <c r="ED2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,134, FALSE)</f>
-        <v>PARQUE EL ELEFANTE</v>
+        <v>TERRENO</v>
       </c>
       <c r="EE2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,135, FALSE)</f>
@@ -40280,9 +40693,9 @@
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,138, FALSE)</f>
         <v>0</v>
       </c>
-      <c r="EI2">
+      <c r="EI2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,139, FALSE)</f>
-        <v>0</v>
+        <v>JIAHAO BAO</v>
       </c>
       <c r="EJ2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,140, FALSE)</f>
@@ -40292,9 +40705,9 @@
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,141, FALSE)</f>
         <v>0</v>
       </c>
-      <c r="EL2">
+      <c r="EL2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,142, FALSE)</f>
-        <v>0</v>
+        <v>ANGELES SANCHEZ</v>
       </c>
       <c r="EM2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,143, FALSE)</f>
@@ -40304,9 +40717,9 @@
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,144, FALSE)</f>
         <v>0</v>
       </c>
-      <c r="EO2">
+      <c r="EO2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,145, FALSE)</f>
-        <v>0</v>
+        <v>MARIA LOURDES FLORES PEREZ</v>
       </c>
       <c r="EP2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,146, FALSE)</f>
@@ -40316,9 +40729,9 @@
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,147, FALSE)</f>
         <v>0</v>
       </c>
-      <c r="ER2">
+      <c r="ER2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,148, FALSE)</f>
-        <v>0</v>
+        <v>JAHZEEL ROJAS TORRES</v>
       </c>
       <c r="ES2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,149, FALSE)</f>
@@ -40328,9 +40741,9 @@
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,150, FALSE)</f>
         <v>0</v>
       </c>
-      <c r="EU2">
+      <c r="EU2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,151, FALSE)</f>
-        <v>0</v>
+        <v>ISAI FLORES MARTINEZ</v>
       </c>
       <c r="EV2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,152, FALSE)</f>
@@ -40340,9 +40753,9 @@
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,153, FALSE)</f>
         <v>0</v>
       </c>
-      <c r="EX2">
+      <c r="EX2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,154, FALSE)</f>
-        <v>0</v>
+        <v>PAMELA MONTSERRAT VALDE VEGA</v>
       </c>
       <c r="EY2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,155, FALSE)</f>
@@ -40352,9 +40765,9 @@
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,156, FALSE)</f>
         <v>0</v>
       </c>
-      <c r="FA2">
+      <c r="FA2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,157, FALSE)</f>
-        <v>0</v>
+        <v>LIZBETH FLORES ORTIZ</v>
       </c>
       <c r="FB2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,158, FALSE)</f>
@@ -40364,9 +40777,9 @@
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,159, FALSE)</f>
         <v>0</v>
       </c>
-      <c r="FD2">
+      <c r="FD2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,160, FALSE)</f>
-        <v>0</v>
+        <v>MARISOL GARCIA MORALES</v>
       </c>
       <c r="FE2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,161, FALSE)</f>
@@ -40376,9 +40789,9 @@
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,162, FALSE)</f>
         <v>0</v>
       </c>
-      <c r="FG2">
+      <c r="FG2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,163, FALSE)</f>
-        <v>0</v>
+        <v>VALERIA PAREDES GONZALEZ</v>
       </c>
       <c r="FH2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,164, FALSE)</f>
@@ -40388,17 +40801,17 @@
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,165, FALSE)</f>
         <v>0</v>
       </c>
-      <c r="FJ2" t="str">
+      <c r="FJ2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,166, FALSE)</f>
-        <v>GAS LP Y GAS NATURAL</v>
+        <v>0</v>
       </c>
       <c r="FK2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,167, FALSE)</f>
-        <v>20480</v>
+        <v>0</v>
       </c>
       <c r="FL2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,168, FALSE)</f>
-        <v>6.8266666666666671</v>
+        <v>0</v>
       </c>
       <c r="FM2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,169, FALSE)</f>
@@ -40430,19 +40843,19 @@
       </c>
       <c r="FT2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,176, FALSE)</f>
-        <v>4200</v>
+        <v>1800</v>
       </c>
       <c r="FU2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,177, FALSE)</f>
-        <v>0.28000000000000003</v>
+        <v>0.12</v>
       </c>
       <c r="FV2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,178, FALSE)</f>
-        <v>7.1066666666666674</v>
+        <v>0.12</v>
       </c>
       <c r="FW2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,179, FALSE)</f>
-        <v>ALTO</v>
+        <v>ORDINARIO</v>
       </c>
       <c r="FX2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,180, FALSE)</f>

</xml_diff>

<commit_message>
Actualizacion base de datos
</commit_message>
<xml_diff>
--- a/Inputs/BD.xlsx
+++ b/Inputs/BD.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/078e1a455e5c02ce/Documentos/GitHub/Proyecto_PIPC/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="384" documentId="13_ncr:1_{898522BF-B0F8-4888-9748-DC730D5D6CBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{661B8319-A996-4DB9-AF99-FAEA8E9222EC}"/>
+  <xr:revisionPtr revIDLastSave="544" documentId="13_ncr:1_{898522BF-B0F8-4888-9748-DC730D5D6CBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FBD41185-BEC0-48F2-BCE0-29EF60BE5DF0}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3F095A75-F066-4695-8672-8D4315F1EF23}"/>
   </bookViews>
@@ -563,7 +563,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7441" uniqueCount="2268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7507" uniqueCount="2302">
   <si>
     <t>dia</t>
   </si>
@@ -7367,6 +7367,108 @@
   </si>
   <si>
     <t>9:00 AM A 19:00 HRS Y 9:00 AM A 2:00 PM.</t>
+  </si>
+  <si>
+    <t>FIBRA A LA CASA SA DE CV</t>
+  </si>
+  <si>
+    <t>ZOOY</t>
+  </si>
+  <si>
+    <t>FCA2005056RA</t>
+  </si>
+  <si>
+    <t>SERVICIOS DE TELECOMUNICACIONES</t>
+  </si>
+  <si>
+    <t>CALLE JUAREZ</t>
+  </si>
+  <si>
+    <t>LOCALES 7 Y 8</t>
+  </si>
+  <si>
+    <t>AMOZOC DE MOTA</t>
+  </si>
+  <si>
+    <t>ate3@zooy.com.mx</t>
+  </si>
+  <si>
+    <t>13 DE MAYO DE 2024</t>
+  </si>
+  <si>
+    <t>2 CAJONES</t>
+  </si>
+  <si>
+    <t>HECTOR ERICK CELIS VAZQUEZ</t>
+  </si>
+  <si>
+    <t>ALAN FABRICIO DOMINGUEZ PEÑA</t>
+  </si>
+  <si>
+    <t>LUNES A DOMINGO</t>
+  </si>
+  <si>
+    <t>9:00 A 19:00 Y 9:00 A 17:30</t>
+  </si>
+  <si>
+    <t>ALARMA</t>
+  </si>
+  <si>
+    <t>JUNIO</t>
+  </si>
+  <si>
+    <t>19.04339117024435, -98.04489831452031</t>
+  </si>
+  <si>
+    <t>PROPIEDAD PRIVADA</t>
+  </si>
+  <si>
+    <t>ESTACIONAMIENTO LOCALES COMERCIALES</t>
+  </si>
+  <si>
+    <t>JANET RAMIREZ SOMBRERERO</t>
+  </si>
+  <si>
+    <t>GESTIÓN DE REDES Y SISTEMAS DE COMUNICACIÓN, ASÍ COMO LA ATENCIÓN Y SOPORTE TÉCNICO A LOS CLIENTES.</t>
+  </si>
+  <si>
+    <t>CARRETERA FEDERAL PUEBLA-TEHUACAN</t>
+  </si>
+  <si>
+    <t>KM 9, 310</t>
+  </si>
+  <si>
+    <t>LOCAL 4</t>
+  </si>
+  <si>
+    <t>CASA BLANCA</t>
+  </si>
+  <si>
+    <t>diana.sanchez@zooy.com.mx</t>
+  </si>
+  <si>
+    <t>FEBRERO DE 2023</t>
+  </si>
+  <si>
+    <t>DIANA ABIGAIL SANCHEZ CARRASCO</t>
+  </si>
+  <si>
+    <t>COMEDOR Y ENTRADA</t>
+  </si>
+  <si>
+    <t>19.04536865683799, -98.1211494223927</t>
+  </si>
+  <si>
+    <t>LOCAL</t>
+  </si>
+  <si>
+    <t>CAMPO REAL</t>
+  </si>
+  <si>
+    <t>KARLA MORALES MEZA</t>
+  </si>
+  <si>
+    <t>ADRIANA LIMON GARCIA</t>
   </si>
 </sst>
 </file>
@@ -7989,7 +8091,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp1.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Spin" dx="26" fmlaLink="$A$1" max="30000" min="1" page="10" val="65"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Spin" dx="26" fmlaLink="$A$1" max="30000" min="1" page="10" val="66"/>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -8385,7 +8487,7 @@
   <sheetData>
     <row r="1" spans="1:322" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="DS1" t="s">
         <v>1968</v>
@@ -31620,7 +31722,7 @@
         <v>454</v>
       </c>
       <c r="FT55">
-        <f t="shared" ref="FT55:FT68" si="25">60*AG55</f>
+        <f t="shared" ref="FT55:FT74" si="25">60*AG55</f>
         <v>4200</v>
       </c>
       <c r="FU55" s="4">
@@ -35415,6 +35517,10 @@
         <f t="shared" si="22"/>
         <v>0</v>
       </c>
+      <c r="FT69">
+        <f t="shared" si="25"/>
+        <v>0</v>
+      </c>
       <c r="FU69" s="4">
         <f t="shared" si="23"/>
         <v>0</v>
@@ -35464,6 +35570,10 @@
         <f t="shared" si="22"/>
         <v>0</v>
       </c>
+      <c r="FT70">
+        <f t="shared" si="25"/>
+        <v>0</v>
+      </c>
       <c r="FU70" s="4">
         <f t="shared" si="23"/>
         <v>0</v>
@@ -35513,6 +35623,10 @@
         <f t="shared" si="22"/>
         <v>0</v>
       </c>
+      <c r="FT71">
+        <f t="shared" si="25"/>
+        <v>0</v>
+      </c>
       <c r="FU71" s="4">
         <f t="shared" si="23"/>
         <v>0</v>
@@ -35562,6 +35676,10 @@
         <f t="shared" si="22"/>
         <v>0</v>
       </c>
+      <c r="FT72">
+        <f t="shared" si="25"/>
+        <v>0</v>
+      </c>
       <c r="FU72" s="4">
         <f t="shared" si="23"/>
         <v>0</v>
@@ -35582,33 +35700,232 @@
       <c r="B73" t="s">
         <v>550</v>
       </c>
+      <c r="C73" t="s">
+        <v>2268</v>
+      </c>
+      <c r="D73" t="s">
+        <v>2269</v>
+      </c>
+      <c r="E73" t="s">
+        <v>2270</v>
+      </c>
+      <c r="G73" t="s">
+        <v>2271</v>
+      </c>
+      <c r="H73" t="s">
+        <v>2288</v>
+      </c>
+      <c r="I73" t="s">
+        <v>2272</v>
+      </c>
+      <c r="J73">
+        <v>107</v>
+      </c>
+      <c r="K73" t="s">
+        <v>2273</v>
+      </c>
+      <c r="L73" t="s">
+        <v>421</v>
+      </c>
+      <c r="M73" t="s">
+        <v>2274</v>
+      </c>
+      <c r="N73" t="s">
+        <v>423</v>
+      </c>
+      <c r="O73">
+        <v>72980</v>
+      </c>
+      <c r="P73">
+        <v>2241240669</v>
+      </c>
+      <c r="Q73" s="3" t="s">
+        <v>2275</v>
+      </c>
+      <c r="S73" t="s">
+        <v>2276</v>
+      </c>
+      <c r="T73" t="s">
+        <v>2229</v>
+      </c>
+      <c r="V73">
+        <v>50</v>
+      </c>
+      <c r="W73">
+        <v>50</v>
+      </c>
+      <c r="X73">
+        <v>1</v>
+      </c>
+      <c r="Y73">
+        <v>1</v>
+      </c>
+      <c r="Z73">
+        <v>1</v>
+      </c>
+      <c r="AA73">
+        <v>1</v>
+      </c>
+      <c r="AB73">
+        <v>0</v>
+      </c>
+      <c r="AC73">
+        <v>0</v>
+      </c>
+      <c r="AD73" t="s">
+        <v>2277</v>
+      </c>
+      <c r="AE73" t="s">
+        <v>2278</v>
+      </c>
+      <c r="AF73" t="s">
+        <v>2279</v>
+      </c>
+      <c r="AG73">
+        <v>2</v>
+      </c>
+      <c r="AH73">
+        <v>0</v>
+      </c>
+      <c r="AI73">
+        <v>1</v>
+      </c>
+      <c r="AJ73">
+        <v>1</v>
+      </c>
+      <c r="AK73">
+        <v>0</v>
+      </c>
+      <c r="AL73">
+        <v>0</v>
+      </c>
+      <c r="AM73">
+        <v>1</v>
+      </c>
+      <c r="AN73">
+        <v>20</v>
+      </c>
+      <c r="AO73">
+        <v>1</v>
+      </c>
+      <c r="AP73" t="s">
+        <v>2280</v>
+      </c>
+      <c r="AQ73" t="s">
+        <v>2281</v>
+      </c>
       <c r="AR73" s="4">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="AS73">
+        <v>1</v>
+      </c>
+      <c r="AT73" t="s">
+        <v>2113</v>
+      </c>
+      <c r="AU73">
+        <v>2</v>
+      </c>
+      <c r="AV73" t="s">
+        <v>2113</v>
+      </c>
+      <c r="AW73">
+        <v>2</v>
+      </c>
+      <c r="BE73">
+        <v>1</v>
+      </c>
+      <c r="BF73" t="s">
+        <v>2282</v>
+      </c>
+      <c r="BI73" t="s">
+        <v>2227</v>
+      </c>
+      <c r="CD73">
+        <v>2</v>
+      </c>
+      <c r="CJ73">
+        <v>1</v>
       </c>
       <c r="CK73" s="4">
         <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="CL73">
+        <v>1</v>
+      </c>
+      <c r="CM73">
+        <v>1</v>
+      </c>
+      <c r="DW73">
+        <v>3</v>
+      </c>
+      <c r="DX73" t="s">
+        <v>2283</v>
+      </c>
+      <c r="DY73">
+        <v>2024</v>
+      </c>
+      <c r="DZ73" t="s">
+        <v>2284</v>
+      </c>
+      <c r="EA73" t="s">
+        <v>2285</v>
+      </c>
+      <c r="EB73" t="s">
+        <v>2286</v>
+      </c>
+      <c r="EC73" t="s">
+        <v>2285</v>
+      </c>
+      <c r="ED73" t="s">
+        <v>439</v>
+      </c>
+      <c r="EF73" t="s">
+        <v>441</v>
+      </c>
+      <c r="EG73" t="s">
+        <v>442</v>
+      </c>
+      <c r="EI73" s="11" t="s">
+        <v>2287</v>
+      </c>
+      <c r="FK73">
         <v>0</v>
       </c>
       <c r="FL73" s="4">
         <f t="shared" si="20"/>
         <v>0</v>
       </c>
+      <c r="FN73">
+        <v>0</v>
+      </c>
       <c r="FO73" s="4">
         <f t="shared" si="21"/>
         <v>0</v>
       </c>
+      <c r="FQ73">
+        <v>0</v>
+      </c>
       <c r="FR73" s="4">
         <f t="shared" si="22"/>
         <v>0</v>
       </c>
+      <c r="FS73" t="s">
+        <v>454</v>
+      </c>
+      <c r="FT73">
+        <f t="shared" si="25"/>
+        <v>120</v>
+      </c>
       <c r="FU73" s="4">
         <f t="shared" si="23"/>
-        <v>0</v>
+        <v>8.0000000000000002E-3</v>
       </c>
       <c r="FV73" s="4">
         <f t="shared" si="24"/>
-        <v>0</v>
+        <v>8.0000000000000002E-3</v>
       </c>
       <c r="FW73" s="4" t="str">
         <f t="shared" si="27"/>
@@ -35622,33 +35939,241 @@
       <c r="B74" t="s">
         <v>550</v>
       </c>
+      <c r="C74" t="s">
+        <v>2268</v>
+      </c>
+      <c r="D74" t="s">
+        <v>2269</v>
+      </c>
+      <c r="E74" t="s">
+        <v>2270</v>
+      </c>
+      <c r="G74" t="s">
+        <v>2271</v>
+      </c>
+      <c r="H74" t="s">
+        <v>2288</v>
+      </c>
+      <c r="I74" t="s">
+        <v>2289</v>
+      </c>
+      <c r="J74" t="s">
+        <v>2290</v>
+      </c>
+      <c r="K74" t="s">
+        <v>2291</v>
+      </c>
+      <c r="L74" t="s">
+        <v>2292</v>
+      </c>
+      <c r="M74" t="s">
+        <v>2274</v>
+      </c>
+      <c r="N74" t="s">
+        <v>423</v>
+      </c>
+      <c r="O74">
+        <v>72995</v>
+      </c>
+      <c r="P74">
+        <v>2241240669</v>
+      </c>
+      <c r="Q74" s="3" t="s">
+        <v>2293</v>
+      </c>
+      <c r="S74" t="s">
+        <v>2294</v>
+      </c>
+      <c r="T74" t="s">
+        <v>2229</v>
+      </c>
+      <c r="V74">
+        <v>82</v>
+      </c>
+      <c r="W74">
+        <v>82</v>
+      </c>
+      <c r="X74">
+        <v>1</v>
+      </c>
+      <c r="Y74">
+        <v>1</v>
+      </c>
+      <c r="Z74">
+        <v>1</v>
+      </c>
+      <c r="AA74">
+        <v>1</v>
+      </c>
+      <c r="AB74">
+        <v>0</v>
+      </c>
+      <c r="AC74">
+        <v>0</v>
+      </c>
+      <c r="AD74" t="s">
+        <v>462</v>
+      </c>
+      <c r="AE74" t="s">
+        <v>2278</v>
+      </c>
+      <c r="AF74" t="s">
+        <v>2295</v>
+      </c>
+      <c r="AG74">
+        <v>3</v>
+      </c>
+      <c r="AH74">
+        <v>0</v>
+      </c>
+      <c r="AI74">
+        <v>0</v>
+      </c>
+      <c r="AJ74">
+        <v>3</v>
+      </c>
+      <c r="AK74">
+        <v>0</v>
+      </c>
+      <c r="AL74">
+        <v>0</v>
+      </c>
+      <c r="AM74">
+        <v>1</v>
+      </c>
+      <c r="AN74">
+        <v>100</v>
+      </c>
+      <c r="AO74">
+        <v>1</v>
+      </c>
+      <c r="AP74" t="s">
+        <v>2280</v>
+      </c>
+      <c r="AQ74" t="s">
+        <v>2281</v>
+      </c>
       <c r="AR74" s="4">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>9</v>
+      </c>
+      <c r="AS74">
+        <v>1</v>
+      </c>
+      <c r="AT74" t="s">
+        <v>431</v>
+      </c>
+      <c r="AU74">
+        <v>2</v>
+      </c>
+      <c r="AV74" t="s">
+        <v>2296</v>
+      </c>
+      <c r="AW74">
+        <v>2</v>
+      </c>
+      <c r="BE74">
+        <v>1</v>
+      </c>
+      <c r="BF74" t="s">
+        <v>2282</v>
+      </c>
+      <c r="BI74" t="s">
+        <v>2227</v>
+      </c>
+      <c r="CD74">
+        <v>3</v>
+      </c>
+      <c r="CF74">
+        <v>1</v>
+      </c>
+      <c r="CI74">
+        <v>1</v>
+      </c>
+      <c r="CJ74">
+        <v>2</v>
       </c>
       <c r="CK74" s="4">
         <f t="shared" si="19"/>
+        <v>1</v>
+      </c>
+      <c r="CL74">
+        <v>1</v>
+      </c>
+      <c r="CM74">
+        <v>2</v>
+      </c>
+      <c r="DW74">
+        <v>3</v>
+      </c>
+      <c r="DX74" t="s">
+        <v>2283</v>
+      </c>
+      <c r="DY74">
+        <v>2024</v>
+      </c>
+      <c r="DZ74" t="s">
+        <v>2297</v>
+      </c>
+      <c r="EA74" t="s">
+        <v>2298</v>
+      </c>
+      <c r="EB74" t="s">
+        <v>2298</v>
+      </c>
+      <c r="EC74" t="s">
+        <v>1793</v>
+      </c>
+      <c r="ED74" t="s">
+        <v>2299</v>
+      </c>
+      <c r="EF74" t="s">
+        <v>441</v>
+      </c>
+      <c r="EG74" t="s">
+        <v>442</v>
+      </c>
+      <c r="EI74" s="11" t="s">
+        <v>2300</v>
+      </c>
+      <c r="EL74" s="11" t="s">
+        <v>2301</v>
+      </c>
+      <c r="FK74">
         <v>0</v>
       </c>
       <c r="FL74" s="4">
         <f t="shared" si="20"/>
         <v>0</v>
       </c>
+      <c r="FN74">
+        <v>0</v>
+      </c>
       <c r="FO74" s="4">
         <f t="shared" si="21"/>
         <v>0</v>
       </c>
+      <c r="FQ74">
+        <v>0</v>
+      </c>
       <c r="FR74" s="4">
         <f t="shared" si="22"/>
         <v>0</v>
       </c>
+      <c r="FS74" t="s">
+        <v>454</v>
+      </c>
+      <c r="FT74">
+        <f t="shared" si="25"/>
+        <v>180</v>
+      </c>
       <c r="FU74" s="4">
         <f t="shared" si="23"/>
-        <v>0</v>
+        <v>1.2E-2</v>
       </c>
       <c r="FV74" s="4">
         <f t="shared" si="24"/>
-        <v>0</v>
+        <v>1.2E-2</v>
       </c>
       <c r="FW74" s="4" t="str">
         <f t="shared" si="27"/>
@@ -40260,7 +40785,7 @@
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="A3:FV13 FX3:GC43 B14:G14 I14:FV14 KD14:LJ42 A14:A201 D15:FV58 B15:C68 GL43:GW43 GY43:HA43 HC43:HD43 HF43 HK43 HP43:HR43 IC43 IE43 IH43:IJ43 IL43 FX44:IM60 EM59:FV60 D59:EL62 EM61:IM62 D63:IM201 B69 B70:C201 A202:IM208">
+  <conditionalFormatting sqref="A3:FV13 FX3:GC43 B14:G14 I14:FV14 KD14:LJ42 A14:A201 D15:FV58 B15:C68 GL43:GW43 GY43:HA43 HC43:HD43 HF43 HK43 HP43:HR43 IC43 IE43 IH43:IJ43 IL43 FX44:IM60 EM59:FV60 D59:EL62 EM61:IM62 D63:IM73 B69 B70:C73 B74:IM201 A202:IM208">
     <cfRule type="expression" dxfId="40" priority="581">
       <formula>$A3=$A$1</formula>
     </cfRule>
@@ -40513,16 +41038,18 @@
     <hyperlink ref="Q66" r:id="rId40" xr:uid="{19D5C0DF-B072-400B-A9E9-5EBBA974FB88}"/>
     <hyperlink ref="Q67" r:id="rId41" xr:uid="{A7FC72C6-B0DB-4FC9-B190-B58CFCCCC457}"/>
     <hyperlink ref="Q68" r:id="rId42" xr:uid="{07B79AC2-D0BB-4053-B52A-2218F9C8D957}"/>
+    <hyperlink ref="Q73" r:id="rId43" xr:uid="{AC530E9D-142F-47C1-9FA2-9326C9E7E289}"/>
+    <hyperlink ref="Q74" r:id="rId44" xr:uid="{3666EBA2-130E-4794-96A0-D6F6C3ACD1EE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId43"/>
-  <legacyDrawing r:id="rId44"/>
+  <drawing r:id="rId45"/>
+  <legacyDrawing r:id="rId46"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x14">
       <controls>
         <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
           <mc:Choice Requires="x14">
-            <control shapeId="1025" r:id="rId45" name="Spinner 1">
+            <control shapeId="1025" r:id="rId47" name="Spinner 1">
               <controlPr defaultSize="0" autoPict="0">
                 <anchor moveWithCells="1" sizeWithCells="1">
                   <from>
@@ -40556,7 +41083,7 @@
     <row r="1" spans="1:310" x14ac:dyDescent="0.3">
       <c r="A1">
         <f>+BD!A1</f>
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B1" t="s">
         <v>133</v>
@@ -41497,7 +42024,7 @@
       </c>
       <c r="D2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,4, FALSE)</f>
-        <v>DHL PBC BUGAMBILIAS</v>
+        <v>DHL PBC GUADALUPE HIDALGO</v>
       </c>
       <c r="E2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,5, FALSE)</f>
@@ -41517,19 +42044,19 @@
       </c>
       <c r="I2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,9, FALSE)</f>
-        <v>PROLONGACION 16 DE SEPTIEMBRE</v>
+        <v>11 SUR</v>
       </c>
       <c r="J2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,10, FALSE)</f>
-        <v>6348</v>
+        <v>12923</v>
       </c>
       <c r="K2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,11, FALSE)</f>
-        <v>LOCAL C</v>
+        <v>LOCAL 1</v>
       </c>
       <c r="L2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,12, FALSE)</f>
-        <v>VISTA HERMOSA</v>
+        <v>SAN ISIDRO CASTILLOTLA</v>
       </c>
       <c r="M2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,13, FALSE)</f>
@@ -41541,23 +42068,23 @@
       </c>
       <c r="O2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,15, FALSE)</f>
-        <v>72470</v>
+        <v>72498</v>
       </c>
       <c r="P2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,16, FALSE)</f>
-        <v>2221938507</v>
+        <v>2223234754</v>
       </c>
       <c r="Q2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,17, FALSE)</f>
-        <v>servicepoint.bam@dhl.com</v>
+        <v>servicepoint.ghi@dhl.com</v>
       </c>
       <c r="R2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,18, FALSE)</f>
-        <v>6</v>
-      </c>
-      <c r="S2">
+        <v>10</v>
+      </c>
+      <c r="S2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,19, FALSE)</f>
-        <v>2018</v>
+        <v>1 DE NOVIEMBRE DE 2014</v>
       </c>
       <c r="T2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,20, FALSE)</f>
@@ -41569,11 +42096,11 @@
       </c>
       <c r="V2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,22, FALSE)</f>
-        <v>80</v>
+        <v>55</v>
       </c>
       <c r="W2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,23, FALSE)</f>
-        <v>80</v>
+        <v>55</v>
       </c>
       <c r="X2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,24, FALSE)</f>
@@ -41601,7 +42128,7 @@
       </c>
       <c r="AD2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,30, FALSE)</f>
-        <v>3 CAJONES</v>
+        <v>4 CAJONES</v>
       </c>
       <c r="AE2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,31, FALSE)</f>
@@ -41609,7 +42136,7 @@
       </c>
       <c r="AF2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,32, FALSE)</f>
-        <v>JULIO OMAR SERRANO GUERRERO</v>
+        <v>MARIA DE LA PAZ CORDERO R</v>
       </c>
       <c r="AG2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,33, FALSE)</f>
@@ -41621,11 +42148,11 @@
       </c>
       <c r="AI2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,35, FALSE)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,36, FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AK2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,37, FALSE)</f>
@@ -41641,7 +42168,7 @@
       </c>
       <c r="AN2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,40, FALSE)</f>
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="AO2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,41, FALSE)</f>
@@ -41657,7 +42184,7 @@
       </c>
       <c r="AR2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,44, FALSE)</f>
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="AS2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,45, FALSE)</f>
@@ -41809,7 +42336,7 @@
       </c>
       <c r="CD2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,82, FALSE)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="CE2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,83, FALSE)</f>
@@ -41829,7 +42356,7 @@
       </c>
       <c r="CI2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,87, FALSE)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="CJ2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,88, FALSE)</f>
@@ -41921,7 +42448,7 @@
       </c>
       <c r="DF2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,110, FALSE)</f>
-        <v>AREA INTERNA Y AREA EXTERNA</v>
+        <v>AREA INTERNA</v>
       </c>
       <c r="DG2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,111, FALSE)</f>
@@ -42001,23 +42528,23 @@
       </c>
       <c r="DZ2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,130, FALSE)</f>
-        <v>19.005951538063638, -98.21983914958865</v>
+        <v>18.980469690072912, -98.25416721650755</v>
       </c>
       <c r="EA2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,131, FALSE)</f>
-        <v>EBANO</v>
+        <v>PRIVADA DE LOS NARANJOS</v>
       </c>
       <c r="EB2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,132, FALSE)</f>
-        <v>CIPRES</v>
+        <v>DE LA ROSA</v>
       </c>
       <c r="EC2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,133, FALSE)</f>
-        <v>VISTA HERMOSA</v>
+        <v>ACC. PRINCIPAL 11 SUR</v>
       </c>
       <c r="ED2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,134, FALSE)</f>
-        <v>LIRIOS</v>
+        <v>CALLE FAROLES</v>
       </c>
       <c r="EE2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,135, FALSE)</f>

</xml_diff>

<commit_message>
Forzar el borrado de Output ignorando errores de permisos
</commit_message>
<xml_diff>
--- a/Inputs/BD.xlsx
+++ b/Inputs/BD.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/078e1a455e5c02ce/Documentos/GitHub/Proyecto_PIPC/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3552" documentId="13_ncr:1_{898522BF-B0F8-4888-9748-DC730D5D6CBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2BB84500-45D8-4789-985F-114D4BBF4110}"/>
+  <xr:revisionPtr revIDLastSave="3555" documentId="13_ncr:1_{898522BF-B0F8-4888-9748-DC730D5D6CBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E7FEF42E-8519-436C-ACEB-7C41B76787B2}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{3F095A75-F066-4695-8672-8D4315F1EF23}"/>
   </bookViews>
@@ -563,7 +563,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8820" uniqueCount="2876">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8820" uniqueCount="2877">
   <si>
     <t>dia</t>
   </si>
@@ -9191,6 +9191,9 @@
   </si>
   <si>
     <t>ARMANDO REFA CEROLIA</t>
+  </si>
+  <si>
+    <t>19.09299651391994, -98.2190241178244</t>
   </si>
 </sst>
 </file>
@@ -9877,7 +9880,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp1.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Spin" dx="26" fmlaLink="$A$1" max="30000" min="1" page="10" val="103"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="Spin" dx="26" fmlaLink="$A$1" max="30000" min="1" page="10" val="105"/>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -10273,7 +10276,7 @@
   <sheetData>
     <row r="1" spans="1:322" ht="28.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="DS1" t="s">
         <v>1968</v>
@@ -47147,7 +47150,7 @@
         <v>2024</v>
       </c>
       <c r="DZ107" t="s">
-        <v>2856</v>
+        <v>2876</v>
       </c>
       <c r="EA107" t="s">
         <v>1952</v>
@@ -50945,7 +50948,7 @@
     <row r="1" spans="1:310" x14ac:dyDescent="0.3">
       <c r="A1">
         <f>+BD!A1</f>
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B1" t="s">
         <v>133</v>
@@ -51882,15 +51885,15 @@
       </c>
       <c r="C2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,3, FALSE)</f>
-        <v>EFREN CONTRERAS ZAFRA</v>
+        <v>ESTAFETA MEXICANA SA DE CV</v>
       </c>
       <c r="D2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,4, FALSE)</f>
-        <v>DOMINICA 19</v>
+        <v>COP PUEBLA</v>
       </c>
       <c r="E2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,5, FALSE)</f>
-        <v>COZE850822S40</v>
+        <v>EME880309SK5</v>
       </c>
       <c r="F2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,6, FALSE)</f>
@@ -51898,31 +51901,31 @@
       </c>
       <c r="G2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,7, FALSE)</f>
-        <v>CAFETERIA, RESTAURANTE</v>
+        <v>BODEGA DE DISTRIBUCION</v>
       </c>
       <c r="H2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,8, FALSE)</f>
-        <v>PREPARAR Y SERVIR ALIMENTOS Y BEBIDAS, OFRECIENDO DESAYUNOS, COMIDAS, POSTRES Y CAFÉ</v>
+        <v>RECEPCIÓN, ALMACENAMIENTO, CONTROL DE INVENTARIOS, PREPARACIÓN DE PEDIDOS, EMBALAJE Y DESPACHO DE PRODUCTOS PARA GARANTIZAR UNA ENTREGA EFICIENTE Y PRECISA</v>
       </c>
       <c r="I2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,9, FALSE)</f>
-        <v>BOULEVARD DE LAS CASCADAS</v>
+        <v>PROLONGACION 5 DE MAYO</v>
       </c>
       <c r="J2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,10, FALSE)</f>
-        <v>1301</v>
-      </c>
-      <c r="K2" t="str">
+        <v>44</v>
+      </c>
+      <c r="K2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,11, FALSE)</f>
-        <v>Q01</v>
+        <v>0</v>
       </c>
       <c r="L2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,12, FALSE)</f>
-        <v>LOMAS DE ANGELOPOLIS III</v>
+        <v>SAN JERONIMO CALERAS</v>
       </c>
       <c r="M2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,13, FALSE)</f>
-        <v>SANTA CLARA OCOYUCAN</v>
+        <v>PUEBLA</v>
       </c>
       <c r="N2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,14, FALSE)</f>
@@ -51930,23 +51933,23 @@
       </c>
       <c r="O2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,15, FALSE)</f>
-        <v>72830</v>
+        <v>72100</v>
       </c>
       <c r="P2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,16, FALSE)</f>
-        <v>0</v>
+        <v>2211898677</v>
       </c>
       <c r="Q2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,17, FALSE)</f>
-        <v>administracion@dominica19.com</v>
+        <v>moises.mendez@estafeta.com</v>
       </c>
       <c r="R2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,18, FALSE)</f>
-        <v>0.5</v>
+        <v>30</v>
       </c>
       <c r="S2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,19, FALSE)</f>
-        <v>DICIEMBRE DE 2024</v>
+        <v>01 DE ENERO DE 1994</v>
       </c>
       <c r="T2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,20, FALSE)</f>
@@ -51958,11 +51961,11 @@
       </c>
       <c r="V2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,22, FALSE)</f>
-        <v>220</v>
+        <v>10700</v>
       </c>
       <c r="W2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,23, FALSE)</f>
-        <v>70</v>
+        <v>10700</v>
       </c>
       <c r="X2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,24, FALSE)</f>
@@ -51970,19 +51973,19 @@
       </c>
       <c r="Y2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,25, FALSE)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Z2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,26, FALSE)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AA2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,27, FALSE)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AB2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,28, FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,29, FALSE)</f>
@@ -51990,35 +51993,35 @@
       </c>
       <c r="AD2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,30, FALSE)</f>
-        <v>20 CAJONES</v>
+        <v>10 CAJONES</v>
       </c>
       <c r="AE2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,31, FALSE)</f>
-        <v>EFREN CONTRERAS ZAFRA</v>
+        <v>JOSE GILBERTO SANCHEZ ARROYO</v>
       </c>
       <c r="AF2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,32, FALSE)</f>
-        <v>JOSE LUIS RODOLFO RODRIGUEZ</v>
+        <v>JOSE GILBERTO SANCHEZ ARROYO</v>
       </c>
       <c r="AG2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,33, FALSE)</f>
-        <v>5</v>
+        <v>60</v>
       </c>
       <c r="AH2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,34, FALSE)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AI2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,35, FALSE)</f>
-        <v>3</v>
+        <v>40</v>
       </c>
       <c r="AJ2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,36, FALSE)</f>
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="AK2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,37, FALSE)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AL2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,38, FALSE)</f>
@@ -52026,51 +52029,51 @@
       </c>
       <c r="AM2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,39, FALSE)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AN2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,40, FALSE)</f>
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="AO2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,41, FALSE)</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AP2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,42, FALSE)</f>
-        <v>LUNES A DOMINGO</v>
+        <v>LUNES A VIERNES Y SABADO</v>
       </c>
       <c r="AQ2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,43, FALSE)</f>
-        <v>8:00 A 23:00 HORAS</v>
+        <v>9:00 A 18:00 Y 9:00 A 13:00 HORAS</v>
       </c>
       <c r="AR2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,44, FALSE)</f>
-        <v>3</v>
+        <v>45</v>
       </c>
       <c r="AS2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,45, FALSE)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AT2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,46, FALSE)</f>
-        <v>COCINA</v>
+        <v>OFICINA Y ALMACEN</v>
       </c>
       <c r="AU2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,47, FALSE)</f>
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="AV2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,48, FALSE)</f>
-        <v>MOSTRADOR, ALMACEN</v>
+        <v>EN TODA LA BODEGA</v>
       </c>
       <c r="AW2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,49, FALSE)</f>
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="AX2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,50, FALSE)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AY2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,51, FALSE)</f>
@@ -52098,11 +52101,11 @@
       </c>
       <c r="BE2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,57, FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="BF2">
+        <v>1</v>
+      </c>
+      <c r="BF2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,58, FALSE)</f>
-        <v>0</v>
+        <v>ALARMA</v>
       </c>
       <c r="BG2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,59, FALSE)</f>
@@ -52112,9 +52115,9 @@
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,60, FALSE)</f>
         <v>0</v>
       </c>
-      <c r="BI2">
+      <c r="BI2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,61, FALSE)</f>
-        <v>0</v>
+        <v>BODEGA</v>
       </c>
       <c r="BJ2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,62, FALSE)</f>
@@ -52198,7 +52201,7 @@
       </c>
       <c r="CD2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,82, FALSE)</f>
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="CE2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,83, FALSE)</f>
@@ -52206,7 +52209,7 @@
       </c>
       <c r="CF2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,84, FALSE)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="CG2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,85, FALSE)</f>
@@ -52214,11 +52217,11 @@
       </c>
       <c r="CH2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,86, FALSE)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="CI2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,87, FALSE)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="CJ2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,88, FALSE)</f>
@@ -52390,23 +52393,23 @@
       </c>
       <c r="DZ2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,130, FALSE)</f>
-        <v>18.970035879601955, -98.2852424490102</v>
+        <v>19.09299651391994, -98.2190241178244</v>
       </c>
       <c r="EA2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,131, FALSE)</f>
-        <v>LOCAL COMERCIAL</v>
+        <v>BODEGA</v>
       </c>
       <c r="EB2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,132, FALSE)</f>
-        <v>ESTACIONAMIENTO</v>
+        <v>CALLE</v>
       </c>
       <c r="EC2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,133, FALSE)</f>
-        <v>ESTACIONAMIENTO</v>
+        <v>BODEGA</v>
       </c>
       <c r="ED2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,134, FALSE)</f>
-        <v>CHEDRAUI</v>
+        <v>CASA HABITACION</v>
       </c>
       <c r="EE2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,135, FALSE)</f>
@@ -52426,7 +52429,7 @@
       </c>
       <c r="EI2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,139, FALSE)</f>
-        <v>AXEL SUAREZ PEREZ</v>
+        <v>MOISES MENDEZ L</v>
       </c>
       <c r="EJ2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,140, FALSE)</f>
@@ -52438,7 +52441,7 @@
       </c>
       <c r="EL2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,142, FALSE)</f>
-        <v>ANA KAREN SANCHEZ ROJAS</v>
+        <v>DANIEL GARCIA FLORES</v>
       </c>
       <c r="EM2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,143, FALSE)</f>
@@ -52450,7 +52453,7 @@
       </c>
       <c r="EO2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,145, FALSE)</f>
-        <v>CASSANDRA SANCHEZ PEREZ</v>
+        <v>BRENDIRE RUTH MUÑOZ PEÑA</v>
       </c>
       <c r="EP2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,146, FALSE)</f>
@@ -52460,9 +52463,9 @@
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,147, FALSE)</f>
         <v>0</v>
       </c>
-      <c r="ER2">
+      <c r="ER2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,148, FALSE)</f>
-        <v>0</v>
+        <v>GUSTAVO CESAR C MENDEZ</v>
       </c>
       <c r="ES2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,149, FALSE)</f>
@@ -52472,9 +52475,9 @@
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,150, FALSE)</f>
         <v>0</v>
       </c>
-      <c r="EU2">
+      <c r="EU2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,151, FALSE)</f>
-        <v>0</v>
+        <v>ANGEL ROGELIO FLORES LOPEZ</v>
       </c>
       <c r="EV2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,152, FALSE)</f>
@@ -52484,9 +52487,9 @@
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,153, FALSE)</f>
         <v>0</v>
       </c>
-      <c r="EX2">
+      <c r="EX2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,154, FALSE)</f>
-        <v>0</v>
+        <v>JORGE LUIS CALDERON GARCIA</v>
       </c>
       <c r="EY2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,155, FALSE)</f>
@@ -52496,9 +52499,9 @@
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,156, FALSE)</f>
         <v>0</v>
       </c>
-      <c r="FA2">
+      <c r="FA2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,157, FALSE)</f>
-        <v>0</v>
+        <v>CARLOS ALBERTO POBLANO CHALTELL</v>
       </c>
       <c r="FB2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,158, FALSE)</f>
@@ -52508,9 +52511,9 @@
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,159, FALSE)</f>
         <v>0</v>
       </c>
-      <c r="FD2">
+      <c r="FD2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,160, FALSE)</f>
-        <v>0</v>
+        <v>LETICIA LANDERO ROSALIANO</v>
       </c>
       <c r="FE2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,161, FALSE)</f>
@@ -52520,9 +52523,9 @@
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,162, FALSE)</f>
         <v>0</v>
       </c>
-      <c r="FG2">
+      <c r="FG2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,163, FALSE)</f>
-        <v>0</v>
+        <v>ARMANDO REFA CEROLIA</v>
       </c>
       <c r="FH2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,164, FALSE)</f>
@@ -52532,29 +52535,29 @@
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,165, FALSE)</f>
         <v>0</v>
       </c>
-      <c r="FJ2" t="str">
+      <c r="FJ2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,166, FALSE)</f>
-        <v>GAS NATURAL</v>
+        <v>0</v>
       </c>
       <c r="FK2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,167, FALSE)</f>
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="FL2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,168, FALSE)</f>
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="FM2">
+        <v>0</v>
+      </c>
+      <c r="FM2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,169, FALSE)</f>
-        <v>0</v>
+        <v>GASOLINA</v>
       </c>
       <c r="FN2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,170, FALSE)</f>
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="FO2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,171, FALSE)</f>
-        <v>0</v>
+        <v>5.7142857142857144</v>
       </c>
       <c r="FP2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,172, FALSE)</f>
@@ -52574,19 +52577,19 @@
       </c>
       <c r="FT2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,176, FALSE)</f>
-        <v>300</v>
+        <v>14000</v>
       </c>
       <c r="FU2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,177, FALSE)</f>
-        <v>0.02</v>
+        <v>0.93333333333333335</v>
       </c>
       <c r="FV2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,178, FALSE)</f>
-        <v>0.35333333333333333</v>
+        <v>6.647619047619048</v>
       </c>
       <c r="FW2" t="str">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,179, FALSE)</f>
-        <v>ORDINARIO</v>
+        <v>ALTO</v>
       </c>
       <c r="FX2">
         <f>VLOOKUP($A$1,BD!$A$3:$IF$210,180, FALSE)</f>

</xml_diff>

<commit_message>
lee y agrega a word tablas relacionadas
</commit_message>
<xml_diff>
--- a/Inputs/BD.xlsx
+++ b/Inputs/BD.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/078e1a455e5c02ce/Documentos/GitHub/Proyecto_PIPC/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="629" documentId="13_ncr:1_{898522BF-B0F8-4888-9748-DC730D5D6CBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A0EC7853-F432-4F17-9836-8E6DA938593D}"/>
+  <xr:revisionPtr revIDLastSave="7293" documentId="13_ncr:1_{898522BF-B0F8-4888-9748-DC730D5D6CBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A0B91A92-70DB-4C92-9220-CD54A55EFFE4}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3F095A75-F066-4695-8672-8D4315F1EF23}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="2" xr2:uid="{3F095A75-F066-4695-8672-8D4315F1EF23}"/>
   </bookViews>
   <sheets>
     <sheet name="BD" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
cidur y BD modificaciones
</commit_message>
<xml_diff>
--- a/Inputs/BD.xlsx
+++ b/Inputs/BD.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/078e1a455e5c02ce/Documentos/GitHub/Proyecto_PIPC/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7292" documentId="13_ncr:1_{898522BF-B0F8-4888-9748-DC730D5D6CBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C3024D4A-E2CD-4791-BBF1-A7AF139B53E0}"/>
+  <xr:revisionPtr revIDLastSave="7543" documentId="13_ncr:1_{898522BF-B0F8-4888-9748-DC730D5D6CBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E53BA482-5013-4DFA-B919-3BE1BF1C1266}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{3F095A75-F066-4695-8672-8D4315F1EF23}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3F095A75-F066-4695-8672-8D4315F1EF23}"/>
   </bookViews>
   <sheets>
     <sheet name="BD" sheetId="1" r:id="rId1"/>
@@ -563,7 +563,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10814" uniqueCount="3576">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10821" uniqueCount="3576">
   <si>
     <t>dia</t>
   </si>
@@ -60831,6 +60831,9 @@
       <c r="A173">
         <v>171</v>
       </c>
+      <c r="B173" t="s">
+        <v>809</v>
+      </c>
       <c r="C173" t="s">
         <v>3469</v>
       </c>
@@ -61051,6 +61054,9 @@
       <c r="A174">
         <v>172</v>
       </c>
+      <c r="B174" t="s">
+        <v>809</v>
+      </c>
       <c r="C174" t="s">
         <v>3469</v>
       </c>
@@ -61268,6 +61274,9 @@
       <c r="A175">
         <v>173</v>
       </c>
+      <c r="B175" t="s">
+        <v>809</v>
+      </c>
       <c r="C175" t="s">
         <v>3469</v>
       </c>
@@ -61488,6 +61497,9 @@
       <c r="A176">
         <v>174</v>
       </c>
+      <c r="B176" t="s">
+        <v>809</v>
+      </c>
       <c r="C176" t="s">
         <v>3469</v>
       </c>
@@ -61705,6 +61717,9 @@
       <c r="A177">
         <v>175</v>
       </c>
+      <c r="B177" t="s">
+        <v>809</v>
+      </c>
       <c r="C177" t="s">
         <v>3469</v>
       </c>
@@ -61925,6 +61940,9 @@
       <c r="A178">
         <v>176</v>
       </c>
+      <c r="B178" t="s">
+        <v>809</v>
+      </c>
       <c r="C178" t="s">
         <v>3469</v>
       </c>
@@ -62144,6 +62162,9 @@
     <row r="179" spans="1:179" x14ac:dyDescent="0.3">
       <c r="A179">
         <v>177</v>
+      </c>
+      <c r="B179" t="s">
+        <v>809</v>
       </c>
       <c r="C179" t="s">
         <v>3469</v>
@@ -64052,7 +64073,7 @@
       <formula>#REF!=$A$1</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations disablePrompts="1" count="1">
+  <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3:B201" xr:uid="{D5CD9EE6-9E02-4584-93C4-B4A613E84A37}">
       <formula1>"BANCO, BBVA, COMPARTAMOS, DHL, GASERA, GASOLINERA, GENERAL, GDL, UVP"</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
eliminacion tablas, ajuste imagenes
</commit_message>
<xml_diff>
--- a/Inputs/BD.xlsx
+++ b/Inputs/BD.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/078e1a455e5c02ce/Documentos/GitHub/Proyecto_PIPC/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7535" documentId="13_ncr:1_{898522BF-B0F8-4888-9748-DC730D5D6CBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A4BDAC0D-D39F-43A9-B1E9-FE93C46A5A74}"/>
+  <xr:revisionPtr revIDLastSave="7544" documentId="13_ncr:1_{898522BF-B0F8-4888-9748-DC730D5D6CBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EB5780CA-5E3B-4D82-9D95-FFE31B5866AA}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3F095A75-F066-4695-8672-8D4315F1EF23}"/>
   </bookViews>
@@ -53643,7 +53643,7 @@
       <formula>$A172=#REF!</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AQ1 AT1:BF1 CI1:CJ1 EN1 FR1:FS207 A2:A12 FV2:GA42 B2:I171 Q2:AE171 AL2:AN171 CA2:CC171 CG2:CH171 J2:P207 AF2:AH207 AO2:BZ207 CI2:CL207 CO2:EV207 FT2:FU207 KB13:LH41 A13:B200 GJ42:GU42 GW42:GY42 HA42:HB42 HD42 HI42 HN42:HP42 IA42 IC42 IF42:IH42 IJ42 FV43:IK207 C172:C178 B179:E200 F179:I207 Q179:AE207 AL179:AN207 CA179:CC207 CG179:CH207 A201:E207 Q1048575:Q1048576 EX2:FQ207">
+  <conditionalFormatting sqref="AQ1 AT1:BF1 CI1:CJ1 EN1 FR1:FS207 A2:A12 FV2:GA42 B2:I171 Q2:AE171 AL2:AN171 CA2:CC171 CG2:CH171 J2:P207 AF2:AH207 AO2:BZ207 CI2:CL207 CO2:EV207 EX2:FQ207 FT2:FU207 KB13:LH41 A13:B200 GJ42:GU42 GW42:GY42 HA42:HB42 HD42 HI42 HN42:HP42 IA42 IC42 IF42:IH42 IJ42 FV43:IK207 C172:C178 B179:E200 F179:I207 Q179:AE207 AL179:AN207 CA179:CC207 CG179:CH207 A201:E207 Q1048575:Q1048576">
     <cfRule type="expression" dxfId="35" priority="612">
       <formula>$A1=#REF!</formula>
     </cfRule>

</xml_diff>